<commit_message>
add time slices to Scen_test.xlsx
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{561E85D3-19C1-49A8-A495-81667B131C60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2009323-3CC6-4177-A29D-90B08F64A144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demand" sheetId="1" r:id="rId1"/>
-    <sheet name="trade" sheetId="2" r:id="rId2"/>
-    <sheet name="fuel_costs" sheetId="3" r:id="rId3"/>
+    <sheet name="timeslices" sheetId="4" r:id="rId2"/>
+    <sheet name="trade" sheetId="2" r:id="rId3"/>
+    <sheet name="fuel_costs" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="79">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -119,6 +120,162 @@
   </si>
   <si>
     <t>cap_bnd</t>
+  </si>
+  <si>
+    <t>season</t>
+  </si>
+  <si>
+    <t>weekly</t>
+  </si>
+  <si>
+    <t>daynite</t>
+  </si>
+  <si>
+    <t>wparent</t>
+  </si>
+  <si>
+    <t>dparent</t>
+  </si>
+  <si>
+    <t>timeslice</t>
+  </si>
+  <si>
+    <t>com_fr</t>
+  </si>
+  <si>
+    <t>g_yrfr</t>
+  </si>
+  <si>
+    <t>com_pkflx</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>ncap_afs</t>
+  </si>
+  <si>
+    <t>pset_ci</t>
+  </si>
+  <si>
+    <t>AllS</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>AllH</t>
+  </si>
+  <si>
+    <t>elc_spv_001</t>
+  </si>
+  <si>
+    <t>AllSaAllH</t>
+  </si>
+  <si>
+    <t>IMPNRGZ</t>
+  </si>
+  <si>
+    <t>elc_won_001</t>
+  </si>
+  <si>
+    <t>elc_wof_001</t>
+  </si>
+  <si>
+    <t>ELC</t>
+  </si>
+  <si>
+    <t>hydro</t>
+  </si>
+  <si>
+    <t>elc_spv_002</t>
+  </si>
+  <si>
+    <t>elc_won_002</t>
+  </si>
+  <si>
+    <t>elc_wof_002</t>
+  </si>
+  <si>
+    <t>elc_spv_003</t>
+  </si>
+  <si>
+    <t>elc_won_003</t>
+  </si>
+  <si>
+    <t>elc_wof_003</t>
+  </si>
+  <si>
+    <t>elc_spv_004</t>
+  </si>
+  <si>
+    <t>elc_won_004</t>
+  </si>
+  <si>
+    <t>elc_wof_004</t>
+  </si>
+  <si>
+    <t>elc_spv_005</t>
+  </si>
+  <si>
+    <t>elc_won_005</t>
+  </si>
+  <si>
+    <t>elc_wof_005</t>
+  </si>
+  <si>
+    <t>elc_spv_006</t>
+  </si>
+  <si>
+    <t>elc_won_006</t>
+  </si>
+  <si>
+    <t>elc_wof_006</t>
+  </si>
+  <si>
+    <t>elc_spv_007</t>
+  </si>
+  <si>
+    <t>elc_won_007</t>
+  </si>
+  <si>
+    <t>elc_wof_007</t>
+  </si>
+  <si>
+    <t>elc_spv_008</t>
+  </si>
+  <si>
+    <t>elc_won_008</t>
+  </si>
+  <si>
+    <t>elc_wof_008</t>
+  </si>
+  <si>
+    <t>elc_spv_009</t>
+  </si>
+  <si>
+    <t>elc_won_009</t>
+  </si>
+  <si>
+    <t>elc_wof_009</t>
+  </si>
+  <si>
+    <t>elc_spv_010</t>
+  </si>
+  <si>
+    <t>elc_won_010</t>
+  </si>
+  <si>
+    <t>elc_wof_010</t>
+  </si>
+  <si>
+    <t>~TimeSlices</t>
+  </si>
+  <si>
+    <t>~TFM_DINS-AT</t>
+  </si>
+  <si>
+    <t>~TFM_INS-AT</t>
   </si>
 </sst>
 </file>
@@ -436,14 +593,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B4:J12"/>
+  <dimension ref="B5:J17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>0</v>
-      </c>
-    </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>1</v>
@@ -484,19 +639,19 @@
         <v>0</v>
       </c>
       <c r="E6">
-        <v>0.11641499999999998</v>
+        <v>0</v>
       </c>
       <c r="F6">
         <v>0.13133999999999996</v>
       </c>
       <c r="G6">
-        <v>0.14924999999999997</v>
+        <v>0.30645999999999995</v>
       </c>
       <c r="H6">
-        <v>0.3343199999999999</v>
+        <v>0.32635999999999987</v>
       </c>
       <c r="I6">
-        <v>0.5402849999999999</v>
+        <v>0.76415999999999984</v>
       </c>
       <c r="J6" t="s">
         <v>4</v>
@@ -510,22 +665,22 @@
         <v>3.581999999999999</v>
       </c>
       <c r="D7">
-        <v>3.3431999999999995</v>
+        <v>3.5521499999999997</v>
       </c>
       <c r="E7">
-        <v>3.6088649999999989</v>
+        <v>3.6397099999999987</v>
       </c>
       <c r="F7">
-        <v>3.8088599999999988</v>
+        <v>3.940199999999999</v>
       </c>
       <c r="G7">
-        <v>4.3282499999999988</v>
+        <v>4.4436699999999991</v>
       </c>
       <c r="H7">
-        <v>4.8476399999999975</v>
+        <v>5.0585799999999983</v>
       </c>
       <c r="I7">
-        <v>5.4028499999999982</v>
+        <v>5.9222399999999986</v>
       </c>
       <c r="J7" t="s">
         <v>4</v>
@@ -539,22 +694,22 @@
         <v>5.969999999999998</v>
       </c>
       <c r="D8">
-        <v>6.2684999999999986</v>
+        <v>6.1640249999999988</v>
       </c>
       <c r="E8">
-        <v>6.9848999999999979</v>
+        <v>6.9271899999999977</v>
       </c>
       <c r="F8">
-        <v>7.4863799999999978</v>
+        <v>7.3550399999999989</v>
       </c>
       <c r="G8">
-        <v>8.0594999999999981</v>
+        <v>8.2744199999999992</v>
       </c>
       <c r="H8">
-        <v>8.6923199999999969</v>
+        <v>8.648539999999997</v>
       </c>
       <c r="I8">
-        <v>9.5450349999999986</v>
+        <v>10.316159999999998</v>
       </c>
       <c r="J8" t="s">
         <v>4</v>
@@ -597,22 +752,22 @@
         <v>9.950000000000081E-2</v>
       </c>
       <c r="D10">
-        <v>0.53729999999999833</v>
+        <v>0.43282499999999935</v>
       </c>
       <c r="E10">
-        <v>0.74923499999999876</v>
+        <v>0.8755999999999986</v>
       </c>
       <c r="F10">
-        <v>1.54026</v>
+        <v>1.5402599999999982</v>
       </c>
       <c r="G10">
-        <v>2.2387499999999996</v>
+        <v>2.3064099999999979</v>
       </c>
       <c r="H10">
-        <v>2.8775399999999998</v>
+        <v>2.3123799999999974</v>
       </c>
       <c r="I10">
-        <v>2.7631149999999991</v>
+        <v>2.5670999999999964</v>
       </c>
       <c r="J10" t="s">
         <v>4</v>
@@ -623,29 +778,34 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
         <v>10</v>
       </c>
-      <c r="D12">
+      <c r="D17">
         <v>0</v>
       </c>
-      <c r="E12">
-        <v>7.1480000000000002E-2</v>
-      </c>
-      <c r="F12">
-        <v>0.10442</v>
-      </c>
-      <c r="G12">
-        <v>0.13485</v>
-      </c>
-      <c r="H12">
-        <v>0.17809999999999998</v>
-      </c>
-      <c r="I12">
-        <v>0.20945</v>
-      </c>
-      <c r="J12" t="s">
+      <c r="E17">
+        <v>6.336E-2</v>
+      </c>
+      <c r="F17">
+        <v>0.15481999999999999</v>
+      </c>
+      <c r="G17">
+        <v>0.17208999999999999</v>
+      </c>
+      <c r="H17">
+        <v>0.25386999999999998</v>
+      </c>
+      <c r="I17">
+        <v>0.28502999999999995</v>
+      </c>
+      <c r="J17" t="s">
         <v>11</v>
       </c>
     </row>
@@ -655,6 +815,607 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05B64E1E-DC66-450D-AA2A-D1B01A72BCA4}">
+  <dimension ref="A2:AL13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>76</v>
+      </c>
+      <c r="G2" t="s">
+        <v>77</v>
+      </c>
+      <c r="L2" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>77</v>
+      </c>
+      <c r="V2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>77</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I3" t="s">
+        <v>33</v>
+      </c>
+      <c r="J3" t="s">
+        <v>12</v>
+      </c>
+      <c r="L3" t="s">
+        <v>1</v>
+      </c>
+      <c r="M3" t="s">
+        <v>32</v>
+      </c>
+      <c r="N3" t="s">
+        <v>33</v>
+      </c>
+      <c r="O3" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>1</v>
+      </c>
+      <c r="R3" t="s">
+        <v>32</v>
+      </c>
+      <c r="S3" t="s">
+        <v>33</v>
+      </c>
+      <c r="T3" t="s">
+        <v>12</v>
+      </c>
+      <c r="V3" t="s">
+        <v>34</v>
+      </c>
+      <c r="W3" t="s">
+        <v>33</v>
+      </c>
+      <c r="X3" t="s">
+        <v>32</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>1</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>32</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>1</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>32</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>35</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>36</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>32</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>37</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G4" t="s">
+        <v>42</v>
+      </c>
+      <c r="H4" t="s">
+        <v>43</v>
+      </c>
+      <c r="I4">
+        <v>1.0000000000000016</v>
+      </c>
+      <c r="J4" t="s">
+        <v>44</v>
+      </c>
+      <c r="L4" t="s">
+        <v>45</v>
+      </c>
+      <c r="M4" t="s">
+        <v>43</v>
+      </c>
+      <c r="N4">
+        <v>1.0000000000000044</v>
+      </c>
+      <c r="O4" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>46</v>
+      </c>
+      <c r="R4" t="s">
+        <v>43</v>
+      </c>
+      <c r="S4">
+        <v>1.0000000000000016</v>
+      </c>
+      <c r="T4" t="s">
+        <v>44</v>
+      </c>
+      <c r="V4">
+        <v>1</v>
+      </c>
+      <c r="W4">
+        <v>1.0000000000000002</v>
+      </c>
+      <c r="X4" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>8</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>6</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>43</v>
+      </c>
+      <c r="AC4">
+        <v>1</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>47</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG4">
+        <v>0.30209170858371315</v>
+      </c>
+      <c r="AI4">
+        <v>2020</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>39</v>
+      </c>
+      <c r="AK4">
+        <v>0</v>
+      </c>
+      <c r="AL4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="5" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="G5" t="s">
+        <v>49</v>
+      </c>
+      <c r="H5" t="s">
+        <v>43</v>
+      </c>
+      <c r="I5">
+        <v>1.0000000000000013</v>
+      </c>
+      <c r="J5" t="s">
+        <v>44</v>
+      </c>
+      <c r="L5" t="s">
+        <v>50</v>
+      </c>
+      <c r="M5" t="s">
+        <v>43</v>
+      </c>
+      <c r="N5">
+        <v>0.99999999999999956</v>
+      </c>
+      <c r="O5" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>51</v>
+      </c>
+      <c r="R5" t="s">
+        <v>43</v>
+      </c>
+      <c r="S5">
+        <v>0.99999999999999722</v>
+      </c>
+      <c r="T5" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>5</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>43</v>
+      </c>
+      <c r="AC5">
+        <v>1</v>
+      </c>
+      <c r="AI5">
+        <v>2021</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>39</v>
+      </c>
+      <c r="AK5">
+        <v>0</v>
+      </c>
+      <c r="AL5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="G6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H6" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6">
+        <v>0.99999999999999933</v>
+      </c>
+      <c r="J6" t="s">
+        <v>44</v>
+      </c>
+      <c r="L6" t="s">
+        <v>53</v>
+      </c>
+      <c r="M6" t="s">
+        <v>43</v>
+      </c>
+      <c r="N6">
+        <v>1.0000000000000013</v>
+      </c>
+      <c r="O6" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>54</v>
+      </c>
+      <c r="R6" t="s">
+        <v>43</v>
+      </c>
+      <c r="S6">
+        <v>0.99999999999999867</v>
+      </c>
+      <c r="T6" t="s">
+        <v>44</v>
+      </c>
+      <c r="AI6">
+        <v>2022</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>39</v>
+      </c>
+      <c r="AK6">
+        <v>0</v>
+      </c>
+      <c r="AL6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="G7" t="s">
+        <v>55</v>
+      </c>
+      <c r="H7" t="s">
+        <v>43</v>
+      </c>
+      <c r="I7">
+        <v>0.99999999999999745</v>
+      </c>
+      <c r="J7" t="s">
+        <v>44</v>
+      </c>
+      <c r="L7" t="s">
+        <v>56</v>
+      </c>
+      <c r="M7" t="s">
+        <v>43</v>
+      </c>
+      <c r="N7">
+        <v>0.99999999999999956</v>
+      </c>
+      <c r="O7" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>57</v>
+      </c>
+      <c r="R7" t="s">
+        <v>43</v>
+      </c>
+      <c r="S7">
+        <v>0.99999999999999445</v>
+      </c>
+      <c r="T7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="G8" t="s">
+        <v>58</v>
+      </c>
+      <c r="H8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I8">
+        <v>0.99999999999999922</v>
+      </c>
+      <c r="J8" t="s">
+        <v>44</v>
+      </c>
+      <c r="L8" t="s">
+        <v>59</v>
+      </c>
+      <c r="M8" t="s">
+        <v>43</v>
+      </c>
+      <c r="N8">
+        <v>1.0000000000000027</v>
+      </c>
+      <c r="O8" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>60</v>
+      </c>
+      <c r="R8" t="s">
+        <v>43</v>
+      </c>
+      <c r="S8">
+        <v>0.99999999999999867</v>
+      </c>
+      <c r="T8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="G9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H9" t="s">
+        <v>43</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9" t="s">
+        <v>44</v>
+      </c>
+      <c r="L9" t="s">
+        <v>62</v>
+      </c>
+      <c r="M9" t="s">
+        <v>43</v>
+      </c>
+      <c r="N9">
+        <v>1.0000000000000018</v>
+      </c>
+      <c r="O9" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>63</v>
+      </c>
+      <c r="R9" t="s">
+        <v>43</v>
+      </c>
+      <c r="S9">
+        <v>1.0000000000000016</v>
+      </c>
+      <c r="T9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="G10" t="s">
+        <v>64</v>
+      </c>
+      <c r="H10" t="s">
+        <v>43</v>
+      </c>
+      <c r="I10">
+        <v>0.99999999999999856</v>
+      </c>
+      <c r="J10" t="s">
+        <v>44</v>
+      </c>
+      <c r="L10" t="s">
+        <v>65</v>
+      </c>
+      <c r="M10" t="s">
+        <v>43</v>
+      </c>
+      <c r="N10">
+        <v>0.99999999999999911</v>
+      </c>
+      <c r="O10" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>66</v>
+      </c>
+      <c r="R10" t="s">
+        <v>43</v>
+      </c>
+      <c r="S10">
+        <v>1.0000000000000013</v>
+      </c>
+      <c r="T10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="G11" t="s">
+        <v>67</v>
+      </c>
+      <c r="H11" t="s">
+        <v>43</v>
+      </c>
+      <c r="I11">
+        <v>1.0000000000000016</v>
+      </c>
+      <c r="J11" t="s">
+        <v>44</v>
+      </c>
+      <c r="L11" t="s">
+        <v>68</v>
+      </c>
+      <c r="M11" t="s">
+        <v>43</v>
+      </c>
+      <c r="N11">
+        <v>1.0000000000000018</v>
+      </c>
+      <c r="O11" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>69</v>
+      </c>
+      <c r="R11" t="s">
+        <v>43</v>
+      </c>
+      <c r="S11">
+        <v>0.99999999999999856</v>
+      </c>
+      <c r="T11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="G12" t="s">
+        <v>70</v>
+      </c>
+      <c r="H12" t="s">
+        <v>43</v>
+      </c>
+      <c r="I12">
+        <v>0.99999999999999789</v>
+      </c>
+      <c r="J12" t="s">
+        <v>44</v>
+      </c>
+      <c r="L12" t="s">
+        <v>71</v>
+      </c>
+      <c r="M12" t="s">
+        <v>43</v>
+      </c>
+      <c r="N12">
+        <v>0.99999999999999789</v>
+      </c>
+      <c r="O12" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>72</v>
+      </c>
+      <c r="R12" t="s">
+        <v>43</v>
+      </c>
+      <c r="S12">
+        <v>0.99999999999999967</v>
+      </c>
+      <c r="T12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="G13" t="s">
+        <v>73</v>
+      </c>
+      <c r="H13" t="s">
+        <v>43</v>
+      </c>
+      <c r="I13">
+        <v>0.99999999999999745</v>
+      </c>
+      <c r="J13" t="s">
+        <v>44</v>
+      </c>
+      <c r="L13" t="s">
+        <v>74</v>
+      </c>
+      <c r="M13" t="s">
+        <v>43</v>
+      </c>
+      <c r="N13">
+        <v>1.0000000000000004</v>
+      </c>
+      <c r="O13" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>75</v>
+      </c>
+      <c r="R13" t="s">
+        <v>43</v>
+      </c>
+      <c r="S13">
+        <v>1.0000000000000004</v>
+      </c>
+      <c r="T13" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F0573AE-84FA-4F18-8D18-B7F3EC5B3273}">
   <dimension ref="B4:K14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -794,7 +1555,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48BDE16D-C995-4313-9FD3-ABCD01C0EB3D}">
   <dimension ref="B6:J11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
correcting demand in Scen_test.xlsx
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2009323-3CC6-4177-A29D-90B08F64A144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7892C85A-146B-4848-8981-F9669F2EC3DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demand" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="79">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -593,12 +593,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B5:J17"/>
+  <dimension ref="B4:J17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>0</v>
+      </c>
+    </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
Adding flow emissions part 2
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93507772-13B0-4CA5-99F7-4217AEBD1C35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25E805B9-83AC-48B1-9D3B-5096F8A26DBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1034,6 +1034,9 @@
         <v>87</v>
       </c>
       <c r="E25">
+        <v>400</v>
+      </c>
+      <c r="J25">
         <v>338.40000000000003</v>
       </c>
     </row>
@@ -1048,6 +1051,9 @@
         <v>87</v>
       </c>
       <c r="E26">
+        <v>200</v>
+      </c>
+      <c r="J26">
         <v>198</v>
       </c>
     </row>
@@ -1062,6 +1068,9 @@
         <v>87</v>
       </c>
       <c r="E27">
+        <v>300</v>
+      </c>
+      <c r="J27">
         <v>252</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adding flow emissions part 3
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25E805B9-83AC-48B1-9D3B-5096F8A26DBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A9E78A-80C3-4172-9E54-1150D236ED21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demand" sheetId="1" r:id="rId1"/>
@@ -1830,7 +1830,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48BDE16D-C995-4313-9FD3-ABCD01C0EB3D}">
-  <dimension ref="B6:T11"/>
+  <dimension ref="B6:T15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
@@ -1911,25 +1911,25 @@
         <v>21</v>
       </c>
       <c r="D9">
-        <v>13.7</v>
+        <v>14</v>
       </c>
       <c r="E9">
-        <v>13.974</v>
+        <v>14</v>
       </c>
       <c r="F9">
-        <v>14.522</v>
+        <v>14</v>
       </c>
       <c r="G9">
-        <v>14.659000000000001</v>
+        <v>14</v>
       </c>
       <c r="H9">
-        <v>14.795999999999999</v>
+        <v>14</v>
       </c>
       <c r="I9">
-        <v>15.07</v>
+        <v>14</v>
       </c>
       <c r="J9">
-        <v>15.344000000000001</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="2:20" x14ac:dyDescent="0.25">
@@ -1988,6 +1988,29 @@
       </c>
       <c r="J11">
         <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="D15">
+        <v>13.7</v>
+      </c>
+      <c r="E15">
+        <v>13.974</v>
+      </c>
+      <c r="F15">
+        <v>14.522</v>
+      </c>
+      <c r="G15">
+        <v>14.659000000000001</v>
+      </c>
+      <c r="H15">
+        <v>14.795999999999999</v>
+      </c>
+      <c r="I15">
+        <v>15.07</v>
+      </c>
+      <c r="J15">
+        <v>15.344000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding flow emissions part 4
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A9E78A-80C3-4172-9E54-1150D236ED21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B150B749-CB3D-49D9-A5F6-CE301B690957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demand" sheetId="1" r:id="rId1"/>
@@ -327,6 +327,9 @@
     <t>value</t>
   </si>
   <si>
+    <t>VDA_EMCB</t>
+  </si>
+  <si>
     <t>coal</t>
   </si>
   <si>
@@ -337,9 +340,6 @@
   </si>
   <si>
     <t>oil</t>
-  </si>
-  <si>
-    <t>FLO_EMIS</t>
   </si>
 </sst>
 </file>
@@ -1025,13 +1025,13 @@
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D25" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E25">
         <v>400</v>
@@ -1042,13 +1042,13 @@
     </row>
     <row r="26" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C26" t="s">
+        <v>89</v>
+      </c>
+      <c r="D26" t="s">
         <v>88</v>
-      </c>
-      <c r="D26" t="s">
-        <v>87</v>
       </c>
       <c r="E26">
         <v>200</v>
@@ -1059,13 +1059,13 @@
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
+        <v>86</v>
+      </c>
+      <c r="C27" t="s">
         <v>90</v>
       </c>
-      <c r="C27" t="s">
-        <v>89</v>
-      </c>
       <c r="D27" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E27">
         <v>300</v>
@@ -1830,7 +1830,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48BDE16D-C995-4313-9FD3-ABCD01C0EB3D}">
-  <dimension ref="B6:T15"/>
+  <dimension ref="B6:T11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
@@ -1911,25 +1911,25 @@
         <v>21</v>
       </c>
       <c r="D9">
-        <v>14</v>
+        <v>13.7</v>
       </c>
       <c r="E9">
-        <v>14</v>
+        <v>13.974</v>
       </c>
       <c r="F9">
-        <v>14</v>
+        <v>14.522</v>
       </c>
       <c r="G9">
-        <v>14</v>
+        <v>14.659000000000001</v>
       </c>
       <c r="H9">
-        <v>14</v>
+        <v>14.795999999999999</v>
       </c>
       <c r="I9">
-        <v>14</v>
+        <v>15.07</v>
       </c>
       <c r="J9">
-        <v>14</v>
+        <v>15.344000000000001</v>
       </c>
     </row>
     <row r="10" spans="2:20" x14ac:dyDescent="0.25">
@@ -1988,29 +1988,6 @@
       </c>
       <c r="J11">
         <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="D15">
-        <v>13.7</v>
-      </c>
-      <c r="E15">
-        <v>13.974</v>
-      </c>
-      <c r="F15">
-        <v>14.522</v>
-      </c>
-      <c r="G15">
-        <v>14.659000000000001</v>
-      </c>
-      <c r="H15">
-        <v>14.795999999999999</v>
-      </c>
-      <c r="I15">
-        <v>15.07</v>
-      </c>
-      <c r="J15">
-        <v>15.344000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adding flow emissions part 5
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B150B749-CB3D-49D9-A5F6-CE301B690957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0524A07-4D21-4D1A-81FF-9D3AC0A43F8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="93">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -340,6 +340,12 @@
   </si>
   <si>
     <t>oil</t>
+  </si>
+  <si>
+    <t>COM_AGG</t>
+  </si>
+  <si>
+    <t>co2</t>
   </si>
 </sst>
 </file>
@@ -681,7 +687,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B3:T27"/>
+  <dimension ref="B3:T28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
@@ -1034,9 +1040,6 @@
         <v>88</v>
       </c>
       <c r="E25">
-        <v>400</v>
-      </c>
-      <c r="J25">
         <v>338.40000000000003</v>
       </c>
     </row>
@@ -1051,9 +1054,6 @@
         <v>88</v>
       </c>
       <c r="E26">
-        <v>200</v>
-      </c>
-      <c r="J26">
         <v>198</v>
       </c>
     </row>
@@ -1068,10 +1068,21 @@
         <v>88</v>
       </c>
       <c r="E27">
-        <v>300</v>
-      </c>
-      <c r="J27">
         <v>252</v>
+      </c>
+    </row>
+    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>91</v>
+      </c>
+      <c r="C28" t="s">
+        <v>92</v>
+      </c>
+      <c r="D28" t="s">
+        <v>10</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
wind onshore com_fr changed back
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B83DE2A7-7D8F-480D-9532-6ADAF78838DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2190A064-F286-4944-86CD-4DABF1D4EBD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1480,7 +1480,7 @@
         <v>95</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>0.12923909287156352</v>
       </c>
       <c r="Q4" t="s">
         <v>41</v>
@@ -1566,7 +1566,7 @@
         <v>98</v>
       </c>
       <c r="P5">
-        <v>0</v>
+        <v>2.3904696128463698E-2</v>
       </c>
       <c r="Q5" t="s">
         <v>41</v>
@@ -1646,7 +1646,7 @@
         <v>100</v>
       </c>
       <c r="P6">
-        <v>0</v>
+        <v>0.11223960491803744</v>
       </c>
       <c r="Q6" t="s">
         <v>41</v>
@@ -1723,7 +1723,7 @@
         <v>101</v>
       </c>
       <c r="P7">
-        <v>0</v>
+        <v>0.11331093849743473</v>
       </c>
       <c r="Q7" t="s">
         <v>41</v>
@@ -1791,7 +1791,7 @@
         <v>102</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>2.178054005059079E-2</v>
       </c>
       <c r="Q8" t="s">
         <v>41</v>
@@ -1859,7 +1859,7 @@
         <v>103</v>
       </c>
       <c r="P9">
-        <v>0</v>
+        <v>7.9597285699010006E-2</v>
       </c>
       <c r="Q9" t="s">
         <v>41</v>
@@ -1927,7 +1927,7 @@
         <v>104</v>
       </c>
       <c r="P10">
-        <v>0</v>
+        <v>8.1809459054675793E-2</v>
       </c>
       <c r="Q10" t="s">
         <v>41</v>
@@ -1995,7 +1995,7 @@
         <v>105</v>
       </c>
       <c r="P11">
-        <v>0</v>
+        <v>1.5762397414136396E-2</v>
       </c>
       <c r="Q11" t="s">
         <v>41</v>
@@ -2063,7 +2063,7 @@
         <v>106</v>
       </c>
       <c r="P12">
-        <v>0</v>
+        <v>0.13910975598870917</v>
       </c>
       <c r="Q12" t="s">
         <v>41</v>
@@ -2131,7 +2131,7 @@
         <v>107</v>
       </c>
       <c r="P13">
-        <v>0</v>
+        <v>0.1328412824161386</v>
       </c>
       <c r="Q13" t="s">
         <v>41</v>
@@ -2199,7 +2199,7 @@
         <v>108</v>
       </c>
       <c r="P14">
-        <v>0</v>
+        <v>2.5358428918473137E-2</v>
       </c>
       <c r="Q14" t="s">
         <v>41</v>
@@ -2267,7 +2267,7 @@
         <v>92</v>
       </c>
       <c r="P15">
-        <v>0</v>
+        <v>0.12553296894209429</v>
       </c>
       <c r="Q15" t="s">
         <v>41</v>
@@ -2314,7 +2314,7 @@
         <v>95</v>
       </c>
       <c r="P16">
-        <v>0</v>
+        <v>0.1325213456520582</v>
       </c>
       <c r="Q16" t="s">
         <v>41</v>
@@ -2361,7 +2361,7 @@
         <v>98</v>
       </c>
       <c r="P17">
-        <v>0</v>
+        <v>2.4645667696570315E-2</v>
       </c>
       <c r="Q17" t="s">
         <v>41</v>
@@ -2408,7 +2408,7 @@
         <v>100</v>
       </c>
       <c r="P18">
-        <v>0</v>
+        <v>0.10072660432774716</v>
       </c>
       <c r="Q18" t="s">
         <v>41</v>
@@ -2455,7 +2455,7 @@
         <v>101</v>
       </c>
       <c r="P19">
-        <v>0</v>
+        <v>0.11313834221180283</v>
       </c>
       <c r="Q19" t="s">
         <v>41</v>
@@ -2502,7 +2502,7 @@
         <v>102</v>
       </c>
       <c r="P20">
-        <v>0</v>
+        <v>2.0367354299406455E-2</v>
       </c>
       <c r="Q20" t="s">
         <v>41</v>
@@ -2549,7 +2549,7 @@
         <v>103</v>
       </c>
       <c r="P21">
-        <v>0</v>
+        <v>7.4851005301479756E-2</v>
       </c>
       <c r="Q21" t="s">
         <v>41</v>
@@ -2596,7 +2596,7 @@
         <v>104</v>
       </c>
       <c r="P22">
-        <v>0</v>
+        <v>8.2921888656091305E-2</v>
       </c>
       <c r="Q22" t="s">
         <v>41</v>
@@ -2643,7 +2643,7 @@
         <v>105</v>
       </c>
       <c r="P23">
-        <v>0</v>
+        <v>1.4816908194568044E-2</v>
       </c>
       <c r="Q23" t="s">
         <v>41</v>
@@ -2690,7 +2690,7 @@
         <v>106</v>
       </c>
       <c r="P24">
-        <v>0</v>
+        <v>0.14476340865714046</v>
       </c>
       <c r="Q24" t="s">
         <v>41</v>
@@ -2737,7 +2737,7 @@
         <v>107</v>
       </c>
       <c r="P25">
-        <v>0</v>
+        <v>0.13980790689267938</v>
       </c>
       <c r="Q25" t="s">
         <v>41</v>
@@ -2784,7 +2784,7 @@
         <v>108</v>
       </c>
       <c r="P26">
-        <v>0</v>
+        <v>2.5906599168361417E-2</v>
       </c>
       <c r="Q26" t="s">
         <v>41</v>
@@ -2831,7 +2831,7 @@
         <v>92</v>
       </c>
       <c r="P27">
-        <v>0</v>
+        <v>0.12351433556883835</v>
       </c>
       <c r="Q27" t="s">
         <v>41</v>
@@ -2869,7 +2869,7 @@
         <v>95</v>
       </c>
       <c r="P28">
-        <v>0</v>
+        <v>0.1276064124261225</v>
       </c>
       <c r="Q28" t="s">
         <v>41</v>
@@ -2907,7 +2907,7 @@
         <v>98</v>
       </c>
       <c r="P29">
-        <v>0</v>
+        <v>2.4071670414895937E-2</v>
       </c>
       <c r="Q29" t="s">
         <v>41</v>
@@ -2945,7 +2945,7 @@
         <v>100</v>
       </c>
       <c r="P30">
-        <v>0</v>
+        <v>0.10743651573839856</v>
       </c>
       <c r="Q30" t="s">
         <v>41</v>
@@ -2983,7 +2983,7 @@
         <v>101</v>
       </c>
       <c r="P31">
-        <v>0</v>
+        <v>0.11261469323631694</v>
       </c>
       <c r="Q31" t="s">
         <v>41</v>
@@ -3021,7 +3021,7 @@
         <v>102</v>
       </c>
       <c r="P32">
-        <v>0</v>
+        <v>2.0812569196136516E-2</v>
       </c>
       <c r="Q32" t="s">
         <v>41</v>
@@ -3059,7 +3059,7 @@
         <v>103</v>
       </c>
       <c r="P33">
-        <v>0</v>
+        <v>8.1661604151791981E-2</v>
       </c>
       <c r="Q33" t="s">
         <v>41</v>
@@ -3097,7 +3097,7 @@
         <v>104</v>
       </c>
       <c r="P34">
-        <v>0</v>
+        <v>8.4711064271707354E-2</v>
       </c>
       <c r="Q34" t="s">
         <v>41</v>
@@ -3135,7 +3135,7 @@
         <v>105</v>
       </c>
       <c r="P35">
-        <v>0</v>
+        <v>1.6467166750910506E-2</v>
       </c>
       <c r="Q35" t="s">
         <v>41</v>
@@ -3173,7 +3173,7 @@
         <v>106</v>
       </c>
       <c r="P36">
-        <v>0</v>
+        <v>0.13903683459611321</v>
       </c>
       <c r="Q36" t="s">
         <v>41</v>
@@ -3211,7 +3211,7 @@
         <v>107</v>
       </c>
       <c r="P37">
-        <v>0</v>
+        <v>0.1366006422733719</v>
       </c>
       <c r="Q37" t="s">
         <v>41</v>
@@ -3249,7 +3249,7 @@
         <v>108</v>
       </c>
       <c r="P38">
-        <v>0</v>
+        <v>2.5466491375397582E-2</v>
       </c>
       <c r="Q38" t="s">
         <v>41</v>
@@ -3287,7 +3287,7 @@
         <v>92</v>
       </c>
       <c r="P39">
-        <v>0</v>
+        <v>0.13047343663957478</v>
       </c>
       <c r="Q39" t="s">
         <v>41</v>
@@ -3325,7 +3325,7 @@
         <v>95</v>
       </c>
       <c r="P40">
-        <v>0</v>
+        <v>0.1431973274361146</v>
       </c>
       <c r="Q40" t="s">
         <v>41</v>
@@ -3363,7 +3363,7 @@
         <v>98</v>
       </c>
       <c r="P41">
-        <v>0</v>
+        <v>2.4574192809648652E-2</v>
       </c>
       <c r="Q41" t="s">
         <v>41</v>
@@ -3401,7 +3401,7 @@
         <v>100</v>
       </c>
       <c r="P42">
-        <v>0</v>
+        <v>0.10204606651976254</v>
       </c>
       <c r="Q42" t="s">
         <v>41</v>
@@ -3439,7 +3439,7 @@
         <v>101</v>
       </c>
       <c r="P43">
-        <v>0</v>
+        <v>0.12042192738740498</v>
       </c>
       <c r="Q43" t="s">
         <v>41</v>
@@ -3477,7 +3477,7 @@
         <v>102</v>
       </c>
       <c r="P44">
-        <v>0</v>
+        <v>2.1339892428197442E-2</v>
       </c>
       <c r="Q44" t="s">
         <v>41</v>
@@ -3515,7 +3515,7 @@
         <v>103</v>
       </c>
       <c r="P45">
-        <v>0</v>
+        <v>6.2841226611418957E-2</v>
       </c>
       <c r="Q45" t="s">
         <v>41</v>
@@ -3553,7 +3553,7 @@
         <v>104</v>
       </c>
       <c r="P46">
-        <v>0</v>
+        <v>7.5773194606755301E-2</v>
       </c>
       <c r="Q46" t="s">
         <v>41</v>
@@ -3591,7 +3591,7 @@
         <v>105</v>
       </c>
       <c r="P47">
-        <v>0</v>
+        <v>1.1933080578166047E-2</v>
       </c>
       <c r="Q47" t="s">
         <v>41</v>
@@ -3629,7 +3629,7 @@
         <v>106</v>
       </c>
       <c r="P48">
-        <v>0</v>
+        <v>0.14210599138999719</v>
       </c>
       <c r="Q48" t="s">
         <v>41</v>
@@ -3667,7 +3667,7 @@
         <v>107</v>
       </c>
       <c r="P49">
-        <v>0</v>
+        <v>0.1390792088165978</v>
       </c>
       <c r="Q49" t="s">
         <v>41</v>
@@ -3705,7 +3705,7 @@
         <v>108</v>
       </c>
       <c r="P50">
-        <v>0</v>
+        <v>2.6214454776361244E-2</v>
       </c>
       <c r="Q50" t="s">
         <v>41</v>
@@ -3743,7 +3743,7 @@
         <v>92</v>
       </c>
       <c r="P51">
-        <v>0</v>
+        <v>0.12809669945662192</v>
       </c>
       <c r="Q51" t="s">
         <v>41</v>
@@ -3781,7 +3781,7 @@
         <v>95</v>
       </c>
       <c r="P52">
-        <v>0</v>
+        <v>0.14294726666526825</v>
       </c>
       <c r="Q52" t="s">
         <v>41</v>
@@ -3819,7 +3819,7 @@
         <v>98</v>
       </c>
       <c r="P53">
-        <v>0</v>
+        <v>2.4189539484698222E-2</v>
       </c>
       <c r="Q53" t="s">
         <v>41</v>
@@ -3857,7 +3857,7 @@
         <v>100</v>
       </c>
       <c r="P54">
-        <v>0</v>
+        <v>0.10285460315212781</v>
       </c>
       <c r="Q54" t="s">
         <v>41</v>
@@ -3895,7 +3895,7 @@
         <v>101</v>
       </c>
       <c r="P55">
-        <v>0</v>
+        <v>0.12296274182225456</v>
       </c>
       <c r="Q55" t="s">
         <v>41</v>
@@ -3933,7 +3933,7 @@
         <v>102</v>
       </c>
       <c r="P56">
-        <v>0</v>
+        <v>2.0846528140558419E-2</v>
       </c>
       <c r="Q56" t="s">
         <v>41</v>
@@ -3971,7 +3971,7 @@
         <v>103</v>
       </c>
       <c r="P57">
-        <v>0</v>
+        <v>6.4472987117987726E-2</v>
       </c>
       <c r="Q57" t="s">
         <v>41</v>
@@ -4009,7 +4009,7 @@
         <v>104</v>
       </c>
       <c r="P58">
-        <v>0</v>
+        <v>7.9953031459588916E-2</v>
       </c>
       <c r="Q58" t="s">
         <v>41</v>
@@ -4047,7 +4047,7 @@
         <v>105</v>
       </c>
       <c r="P59">
-        <v>0</v>
+        <v>1.0831192914898173E-2</v>
       </c>
       <c r="Q59" t="s">
         <v>41</v>
@@ -4085,7 +4085,7 @@
         <v>106</v>
       </c>
       <c r="P60">
-        <v>0</v>
+        <v>0.13902163776782839</v>
       </c>
       <c r="Q60" t="s">
         <v>41</v>
@@ -4123,7 +4123,7 @@
         <v>107</v>
       </c>
       <c r="P61">
-        <v>0</v>
+        <v>0.13757753926262756</v>
       </c>
       <c r="Q61" t="s">
         <v>41</v>
@@ -4161,7 +4161,7 @@
         <v>108</v>
       </c>
       <c r="P62">
-        <v>0</v>
+        <v>2.6246232755542848E-2</v>
       </c>
       <c r="Q62" t="s">
         <v>41</v>
@@ -4199,7 +4199,7 @@
         <v>92</v>
       </c>
       <c r="P63">
-        <v>0</v>
+        <v>0.12919913405979461</v>
       </c>
       <c r="Q63" t="s">
         <v>41</v>
@@ -4237,7 +4237,7 @@
         <v>95</v>
       </c>
       <c r="P64">
-        <v>0</v>
+        <v>0.14280869488679127</v>
       </c>
       <c r="Q64" t="s">
         <v>41</v>
@@ -4275,7 +4275,7 @@
         <v>98</v>
       </c>
       <c r="P65">
-        <v>0</v>
+        <v>2.4746674590950292E-2</v>
       </c>
       <c r="Q65" t="s">
         <v>41</v>
@@ -4313,7 +4313,7 @@
         <v>100</v>
       </c>
       <c r="P66">
-        <v>0</v>
+        <v>0.10145405837111347</v>
       </c>
       <c r="Q66" t="s">
         <v>41</v>
@@ -4351,7 +4351,7 @@
         <v>101</v>
       </c>
       <c r="P67">
-        <v>0</v>
+        <v>0.1224410278960416</v>
       </c>
       <c r="Q67" t="s">
         <v>41</v>
@@ -4389,7 +4389,7 @@
         <v>102</v>
       </c>
       <c r="P68">
-        <v>0</v>
+        <v>2.1439916031275898E-2</v>
       </c>
       <c r="Q68" t="s">
         <v>41</v>
@@ -4427,7 +4427,7 @@
         <v>103</v>
       </c>
       <c r="P69">
-        <v>0</v>
+        <v>6.4543167279016975E-2</v>
       </c>
       <c r="Q69" t="s">
         <v>41</v>
@@ -4465,7 +4465,7 @@
         <v>104</v>
       </c>
       <c r="P70">
-        <v>0</v>
+        <v>7.6872225586629289E-2</v>
       </c>
       <c r="Q70" t="s">
         <v>41</v>
@@ -4503,7 +4503,7 @@
         <v>105</v>
       </c>
       <c r="P71">
-        <v>0</v>
+        <v>1.1833148583530682E-2</v>
       </c>
       <c r="Q71" t="s">
         <v>41</v>
@@ -4541,7 +4541,7 @@
         <v>106</v>
       </c>
       <c r="P72">
-        <v>0</v>
+        <v>0.14072958796265375</v>
       </c>
       <c r="Q72" t="s">
         <v>41</v>
@@ -4579,7 +4579,7 @@
         <v>107</v>
       </c>
       <c r="P73">
-        <v>0</v>
+        <v>0.13765800710196696</v>
       </c>
       <c r="Q73" t="s">
         <v>41</v>
@@ -4617,7 +4617,7 @@
         <v>108</v>
       </c>
       <c r="P74">
-        <v>0</v>
+        <v>2.6274357650236987E-2</v>
       </c>
       <c r="Q74" t="s">
         <v>41</v>
@@ -4655,7 +4655,7 @@
         <v>92</v>
       </c>
       <c r="P75">
-        <v>0</v>
+        <v>0.12638981598557553</v>
       </c>
       <c r="Q75" t="s">
         <v>41</v>
@@ -4693,7 +4693,7 @@
         <v>95</v>
       </c>
       <c r="P76">
-        <v>0</v>
+        <v>0.13795376593518585</v>
       </c>
       <c r="Q76" t="s">
         <v>41</v>
@@ -4731,7 +4731,7 @@
         <v>98</v>
       </c>
       <c r="P77">
-        <v>0</v>
+        <v>2.4843309428039376E-2</v>
       </c>
       <c r="Q77" t="s">
         <v>41</v>
@@ -4769,7 +4769,7 @@
         <v>100</v>
       </c>
       <c r="P78">
-        <v>0</v>
+        <v>0.1016527773886627</v>
       </c>
       <c r="Q78" t="s">
         <v>41</v>
@@ -4807,7 +4807,7 @@
         <v>101</v>
       </c>
       <c r="P79">
-        <v>0</v>
+        <v>0.12060953065136704</v>
       </c>
       <c r="Q79" t="s">
         <v>41</v>
@@ -4845,7 +4845,7 @@
         <v>102</v>
       </c>
       <c r="P80">
-        <v>0</v>
+        <v>2.1498054495739747E-2</v>
       </c>
       <c r="Q80" t="s">
         <v>41</v>
@@ -4883,7 +4883,7 @@
         <v>103</v>
       </c>
       <c r="P81">
-        <v>0</v>
+        <v>6.554953323933016E-2</v>
       </c>
       <c r="Q81" t="s">
         <v>41</v>
@@ -4921,7 +4921,7 @@
         <v>104</v>
       </c>
       <c r="P82">
-        <v>0</v>
+        <v>7.5936162267840598E-2</v>
       </c>
       <c r="Q82" t="s">
         <v>41</v>
@@ -4959,7 +4959,7 @@
         <v>105</v>
       </c>
       <c r="P83">
-        <v>0</v>
+        <v>1.2418773706407926E-2</v>
       </c>
       <c r="Q83" t="s">
         <v>41</v>
@@ -4997,7 +4997,7 @@
         <v>106</v>
       </c>
       <c r="P84">
-        <v>0</v>
+        <v>0.14750541621321081</v>
       </c>
       <c r="Q84" t="s">
         <v>41</v>
@@ -5035,7 +5035,7 @@
         <v>107</v>
       </c>
       <c r="P85">
-        <v>0</v>
+        <v>0.13936386512639157</v>
       </c>
       <c r="Q85" t="s">
         <v>41</v>
@@ -5073,7 +5073,7 @@
         <v>108</v>
       </c>
       <c r="P86">
-        <v>0</v>
+        <v>2.6278995562247855E-2</v>
       </c>
       <c r="Q86" t="s">
         <v>41</v>
@@ -5111,7 +5111,7 @@
         <v>92</v>
       </c>
       <c r="P87">
-        <v>0</v>
+        <v>0.12580073214139489</v>
       </c>
       <c r="Q87" t="s">
         <v>41</v>
@@ -5149,7 +5149,7 @@
         <v>95</v>
       </c>
       <c r="P88">
-        <v>0</v>
+        <v>0.13943599824207575</v>
       </c>
       <c r="Q88" t="s">
         <v>41</v>
@@ -5187,7 +5187,7 @@
         <v>98</v>
       </c>
       <c r="P89">
-        <v>0</v>
+        <v>2.5136160161585271E-2</v>
       </c>
       <c r="Q89" t="s">
         <v>41</v>
@@ -5225,7 +5225,7 @@
         <v>100</v>
       </c>
       <c r="P90">
-        <v>0</v>
+        <v>0.10991843774896405</v>
       </c>
       <c r="Q90" t="s">
         <v>41</v>
@@ -5263,7 +5263,7 @@
         <v>101</v>
       </c>
       <c r="P91">
-        <v>0</v>
+        <v>0.11945616844315941</v>
       </c>
       <c r="Q91" t="s">
         <v>41</v>
@@ -5301,7 +5301,7 @@
         <v>102</v>
       </c>
       <c r="P92">
-        <v>0</v>
+        <v>2.2436381028912631E-2</v>
       </c>
       <c r="Q92" t="s">
         <v>41</v>
@@ -5339,7 +5339,7 @@
         <v>103</v>
       </c>
       <c r="P93">
-        <v>0</v>
+        <v>6.593608910998304E-2</v>
       </c>
       <c r="Q93" t="s">
         <v>41</v>
@@ -5377,7 +5377,7 @@
         <v>104</v>
       </c>
       <c r="P94">
-        <v>0</v>
+        <v>7.8642770753477795E-2</v>
       </c>
       <c r="Q94" t="s">
         <v>41</v>
@@ -5415,7 +5415,7 @@
         <v>105</v>
       </c>
       <c r="P95">
-        <v>0</v>
+        <v>1.3836938284508195E-2</v>
       </c>
       <c r="Q95" t="s">
         <v>41</v>
@@ -5453,7 +5453,7 @@
         <v>106</v>
       </c>
       <c r="P96">
-        <v>0</v>
+        <v>0.1386152975371186</v>
       </c>
       <c r="Q96" t="s">
         <v>41</v>
@@ -5491,7 +5491,7 @@
         <v>107</v>
       </c>
       <c r="P97">
-        <v>0</v>
+        <v>0.13512354523104875</v>
       </c>
       <c r="Q97" t="s">
         <v>41</v>
@@ -5529,7 +5529,7 @@
         <v>108</v>
       </c>
       <c r="P98">
-        <v>0</v>
+        <v>2.5661481317773408E-2</v>
       </c>
       <c r="Q98" t="s">
         <v>41</v>
@@ -5567,7 +5567,7 @@
         <v>92</v>
       </c>
       <c r="P99">
-        <v>0</v>
+        <v>0.1267671949798799</v>
       </c>
       <c r="Q99" t="s">
         <v>41</v>
@@ -5605,7 +5605,7 @@
         <v>95</v>
       </c>
       <c r="P100">
-        <v>0</v>
+        <v>0.13876772986981015</v>
       </c>
       <c r="Q100" t="s">
         <v>41</v>
@@ -5643,7 +5643,7 @@
         <v>98</v>
       </c>
       <c r="P101">
-        <v>0</v>
+        <v>2.506295410048941E-2</v>
       </c>
       <c r="Q101" t="s">
         <v>41</v>
@@ -5681,7 +5681,7 @@
         <v>100</v>
       </c>
       <c r="P102">
-        <v>0</v>
+        <v>0.10332983278032665</v>
       </c>
       <c r="Q102" t="s">
         <v>41</v>
@@ -5719,7 +5719,7 @@
         <v>101</v>
       </c>
       <c r="P103">
-        <v>0</v>
+        <v>0.11777530862955292</v>
       </c>
       <c r="Q103" t="s">
         <v>41</v>
@@ -5757,7 +5757,7 @@
         <v>102</v>
       </c>
       <c r="P104">
-        <v>0</v>
+        <v>2.1128161076743861E-2</v>
       </c>
       <c r="Q104" t="s">
         <v>41</v>
@@ -5795,7 +5795,7 @@
         <v>103</v>
       </c>
       <c r="P105">
-        <v>0</v>
+        <v>6.9630153205998191E-2</v>
       </c>
       <c r="Q105" t="s">
         <v>41</v>
@@ -5833,7 +5833,7 @@
         <v>104</v>
       </c>
       <c r="P106">
-        <v>0</v>
+        <v>7.567705618236456E-2</v>
       </c>
       <c r="Q106" t="s">
         <v>41</v>
@@ -5871,7 +5871,7 @@
         <v>105</v>
       </c>
       <c r="P107">
-        <v>0</v>
+        <v>1.405419420329863E-2</v>
       </c>
       <c r="Q107" t="s">
         <v>41</v>
@@ -5909,7 +5909,7 @@
         <v>106</v>
       </c>
       <c r="P108">
-        <v>0</v>
+        <v>0.14235751042892741</v>
       </c>
       <c r="Q108" t="s">
         <v>41</v>
@@ -5947,7 +5947,7 @@
         <v>107</v>
       </c>
       <c r="P109">
-        <v>0</v>
+        <v>0.13917553905188212</v>
       </c>
       <c r="Q109" t="s">
         <v>41</v>
@@ -5985,7 +5985,7 @@
         <v>108</v>
       </c>
       <c r="P110">
-        <v>0</v>
+        <v>2.6274365490724042E-2</v>
       </c>
       <c r="Q110" t="s">
         <v>41</v>
@@ -6023,7 +6023,7 @@
         <v>92</v>
       </c>
       <c r="P111">
-        <v>0</v>
+        <v>0.12733260672506325</v>
       </c>
       <c r="Q111" t="s">
         <v>41</v>
@@ -6061,7 +6061,7 @@
         <v>95</v>
       </c>
       <c r="P112">
-        <v>0</v>
+        <v>0.14173308433155787</v>
       </c>
       <c r="Q112" t="s">
         <v>41</v>
@@ -6099,7 +6099,7 @@
         <v>98</v>
       </c>
       <c r="P113">
-        <v>0</v>
+        <v>2.5244253728599505E-2</v>
       </c>
       <c r="Q113" t="s">
         <v>41</v>
@@ -6137,7 +6137,7 @@
         <v>100</v>
       </c>
       <c r="P114">
-        <v>0</v>
+        <v>0.10375622367614544</v>
       </c>
       <c r="Q114" t="s">
         <v>41</v>
@@ -6175,7 +6175,7 @@
         <v>101</v>
       </c>
       <c r="P115">
-        <v>0</v>
+        <v>0.12028123022816023</v>
       </c>
       <c r="Q115" t="s">
         <v>41</v>
@@ -6213,7 +6213,7 @@
         <v>102</v>
       </c>
       <c r="P116">
-        <v>0</v>
+        <v>2.1737932659842332E-2</v>
       </c>
       <c r="Q116" t="s">
         <v>41</v>
@@ -6251,7 +6251,7 @@
         <v>103</v>
       </c>
       <c r="P117">
-        <v>0</v>
+        <v>6.3532964121559052E-2</v>
       </c>
       <c r="Q117" t="s">
         <v>41</v>
@@ -6289,7 +6289,7 @@
         <v>104</v>
       </c>
       <c r="P118">
-        <v>0</v>
+        <v>7.6382750604245514E-2</v>
       </c>
       <c r="Q118" t="s">
         <v>41</v>
@@ -6327,7 +6327,7 @@
         <v>105</v>
       </c>
       <c r="P119">
-        <v>0</v>
+        <v>1.2385615422098289E-2</v>
       </c>
       <c r="Q119" t="s">
         <v>41</v>
@@ -6365,7 +6365,7 @@
         <v>106</v>
       </c>
       <c r="P120">
-        <v>0</v>
+        <v>0.14263676093132049</v>
       </c>
       <c r="Q120" t="s">
         <v>41</v>
@@ -6403,7 +6403,7 @@
         <v>107</v>
       </c>
       <c r="P121">
-        <v>0</v>
+        <v>0.1385722979114157</v>
       </c>
       <c r="Q121" t="s">
         <v>41</v>
@@ -6441,7 +6441,7 @@
         <v>108</v>
       </c>
       <c r="P122">
-        <v>0</v>
+        <v>2.6404279659992709E-2</v>
       </c>
       <c r="Q122" t="s">
         <v>41</v>

</xml_diff>

<commit_message>
Adding windonshore timsliced ncap_af
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2190A064-F286-4944-86CD-4DABF1D4EBD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A68250C1-B49F-4ED2-8A34-246DC9999CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demand" sheetId="1" r:id="rId1"/>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1300" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1361" uniqueCount="119">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -397,25 +397,49 @@
   </si>
   <si>
     <t>WaP</t>
+  </si>
+  <si>
+    <t>~TimeSlices</t>
+  </si>
+  <si>
+    <t>~TFM_DINS-AT</t>
+  </si>
+  <si>
+    <t>Limtype</t>
+  </si>
+  <si>
+    <t>UP</t>
+  </si>
+  <si>
+    <t>ncap_af</t>
+  </si>
+  <si>
+    <t>Wind onshore</t>
+  </si>
+  <si>
+    <t>PSET_PN</t>
+  </si>
+  <si>
+    <t>~TFM_DINS</t>
+  </si>
+  <si>
+    <t>Attribute</t>
+  </si>
+  <si>
+    <t>AllRegions</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -483,21 +507,21 @@
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
+      <sheetData sheetId="11" refreshError="1"/>
+      <sheetData sheetId="12" refreshError="1"/>
+      <sheetData sheetId="13" refreshError="1"/>
+      <sheetData sheetId="14" refreshError="1"/>
+      <sheetData sheetId="15" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -785,20 +809,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B3:T31"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.81640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:20" x14ac:dyDescent="0.35">
       <c r="N3" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="4" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>0</v>
       </c>
@@ -824,7 +848,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="5" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>1</v>
       </c>
@@ -874,7 +898,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>74</v>
       </c>
@@ -903,7 +927,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>5</v>
       </c>
@@ -932,7 +956,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>6</v>
       </c>
@@ -961,7 +985,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>7</v>
       </c>
@@ -990,12 +1014,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>8</v>
       </c>
@@ -1024,7 +1048,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>3</v>
       </c>
@@ -1053,12 +1077,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>2</v>
       </c>
@@ -1078,7 +1102,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
         <v>80</v>
       </c>
@@ -1092,7 +1116,7 @@
         <v>338.40000000000003</v>
       </c>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
         <v>80</v>
       </c>
@@ -1106,7 +1130,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B21" t="s">
         <v>80</v>
       </c>
@@ -1120,7 +1144,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
         <v>85</v>
       </c>
@@ -1134,12 +1158,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>1</v>
       </c>
@@ -1168,7 +1192,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
         <v>9</v>
       </c>
@@ -1176,7 +1200,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:10" x14ac:dyDescent="0.35">
       <c r="B29" t="s">
         <v>10</v>
       </c>
@@ -1208,7 +1232,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:10" x14ac:dyDescent="0.35">
       <c r="C31">
         <v>80</v>
       </c>
@@ -1227,49 +1251,49 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05B64E1E-DC66-450D-AA2A-D1B01A72BCA4}">
-  <dimension ref="A1:AL122"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AS122"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="7" max="7" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="C1" t="str">
-        <f>IF(A3="x","DeActivated","~TimeSlices")</f>
-        <v>~TimeSlices</v>
-      </c>
-      <c r="I1" t="str">
-        <f>IF(A3="x","DeActivated","~TFM_DINS-AT")</f>
-        <v>~TFM_DINS-AT</v>
-      </c>
-      <c r="N1" t="str">
-        <f>IF(A3="x","DeActivated","~TFM_DINS-AT")</f>
-        <v>~TFM_DINS-AT</v>
-      </c>
-      <c r="S1" t="str">
-        <f>IF(A3="x","DeActivated","~TFM_DINS-AT")</f>
-        <v>~TFM_DINS-AT</v>
-      </c>
-      <c r="X1" t="str">
-        <f>IF(A3="x","DeActivated","~TFM_DINS-AT")</f>
-        <v>~TFM_DINS-AT</v>
-      </c>
-      <c r="AC1" t="str">
-        <f>IF(A3="x","DeActivated","~TFM_DINS-AT")</f>
-        <v>~TFM_DINS-AT</v>
-      </c>
-      <c r="AG1" t="str">
-        <f>IF(A3="x","DeActivated","~TFM_DINS-AT")</f>
-        <v>~TFM_DINS-AT</v>
-      </c>
-    </row>
-    <row r="2" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:45" x14ac:dyDescent="0.35">
+      <c r="C1" t="s">
+        <v>109</v>
+      </c>
+      <c r="I1" t="s">
+        <v>110</v>
+      </c>
+      <c r="N1" t="s">
+        <v>110</v>
+      </c>
+      <c r="S1" t="s">
+        <v>110</v>
+      </c>
+      <c r="X1" t="s">
+        <v>116</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>110</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>110</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>88</v>
       </c>
@@ -1325,37 +1349,52 @@
         <v>12</v>
       </c>
       <c r="X2" t="s">
+        <v>32</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>111</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>117</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>115</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>118</v>
+      </c>
+      <c r="AE2" t="s">
         <v>34</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="AF2" t="s">
         <v>33</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="AG2" t="s">
         <v>32</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="AH2" t="s">
         <v>1</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AJ2" t="s">
         <v>1</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AK2" t="s">
         <v>32</v>
       </c>
-      <c r="AE2" t="s">
+      <c r="AL2" t="s">
         <v>33</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AN2" t="s">
         <v>1</v>
       </c>
-      <c r="AH2" t="s">
+      <c r="AO2" t="s">
         <v>32</v>
       </c>
-      <c r="AI2" t="s">
+      <c r="AP2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A3" t="str">
         <f>IFERROR(IF([1]Veda!#REF!=A2,"ok","x"),"")</f>
         <v/>
@@ -1394,7 +1433,7 @@
         <v>92</v>
       </c>
       <c r="P3">
-        <v>0</v>
+        <v>0.12504651804277112</v>
       </c>
       <c r="Q3" t="s">
         <v>41</v>
@@ -1411,47 +1450,62 @@
       <c r="V3" t="s">
         <v>41</v>
       </c>
-      <c r="X3">
+      <c r="X3" t="s">
+        <v>92</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>112</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>113</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>114</v>
+      </c>
+      <c r="AB3">
+        <v>9.8663766736899333E-2</v>
+      </c>
+      <c r="AE3">
         <v>0.11426940639269406</v>
       </c>
-      <c r="Y3">
+      <c r="AF3">
         <v>0.16087081189037786</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="AG3" t="s">
         <v>92</v>
       </c>
-      <c r="AA3" t="s">
+      <c r="AH3" t="s">
         <v>8</v>
       </c>
-      <c r="AC3" t="s">
+      <c r="AJ3" t="s">
         <v>6</v>
       </c>
-      <c r="AD3" t="s">
+      <c r="AK3" t="s">
         <v>92</v>
       </c>
-      <c r="AE3">
+      <c r="AL3">
         <v>0.11820818077291764</v>
       </c>
-      <c r="AG3" t="s">
+      <c r="AN3" t="s">
         <v>44</v>
       </c>
-      <c r="AH3" t="s">
+      <c r="AO3" t="s">
         <v>92</v>
       </c>
-      <c r="AI3">
+      <c r="AP3">
         <v>6.7453183173023845E-2</v>
       </c>
-      <c r="AJ3" t="s">
+      <c r="AQ3" t="s">
         <v>32</v>
       </c>
-      <c r="AK3" t="s">
+      <c r="AR3" t="s">
         <v>36</v>
       </c>
-      <c r="AL3" t="s">
+      <c r="AS3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:45" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
         <v>93</v>
       </c>
@@ -1497,47 +1551,62 @@
       <c r="V4" t="s">
         <v>41</v>
       </c>
-      <c r="X4">
+      <c r="X4" t="s">
+        <v>95</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>112</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>113</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>114</v>
+      </c>
+      <c r="AB4">
+        <v>0.10284697206552026</v>
+      </c>
+      <c r="AE4">
         <v>0.11426940639269406</v>
       </c>
-      <c r="Y4">
+      <c r="AF4">
         <v>5.2547713165767528E-2</v>
       </c>
-      <c r="Z4" t="s">
+      <c r="AG4" t="s">
         <v>95</v>
       </c>
-      <c r="AA4" t="s">
+      <c r="AH4" t="s">
         <v>8</v>
       </c>
-      <c r="AC4" t="s">
+      <c r="AJ4" t="s">
         <v>6</v>
       </c>
-      <c r="AD4" t="s">
+      <c r="AK4" t="s">
         <v>95</v>
       </c>
-      <c r="AE4">
+      <c r="AL4">
         <v>9.765399900437545E-2</v>
       </c>
-      <c r="AG4" t="s">
+      <c r="AN4" t="s">
         <v>44</v>
       </c>
-      <c r="AH4" t="s">
+      <c r="AO4" t="s">
         <v>95</v>
       </c>
-      <c r="AI4">
+      <c r="AP4">
         <v>0.21742041059208561</v>
       </c>
-      <c r="AJ4" t="s">
+      <c r="AQ4" t="s">
         <v>38</v>
       </c>
-      <c r="AK4">
+      <c r="AR4">
         <v>0</v>
       </c>
-      <c r="AL4" t="s">
+      <c r="AS4" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:45" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>96</v>
       </c>
@@ -1583,47 +1652,62 @@
       <c r="V5" t="s">
         <v>41</v>
       </c>
-      <c r="X5">
+      <c r="X5" t="s">
+        <v>98</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>112</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>113</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>114</v>
+      </c>
+      <c r="AB5">
+        <v>0.10723479236049754</v>
+      </c>
+      <c r="AE5">
         <v>2.0776255707762557E-2</v>
       </c>
-      <c r="Y5">
+      <c r="AF5">
         <v>3.5896543437005365E-2</v>
       </c>
-      <c r="Z5" t="s">
+      <c r="AG5" t="s">
         <v>98</v>
       </c>
-      <c r="AA5" t="s">
+      <c r="AH5" t="s">
         <v>8</v>
       </c>
-      <c r="AC5" t="s">
+      <c r="AJ5" t="s">
         <v>6</v>
       </c>
-      <c r="AD5" t="s">
+      <c r="AK5" t="s">
         <v>98</v>
       </c>
-      <c r="AE5">
+      <c r="AL5">
         <v>2.1376827284429509E-2</v>
       </c>
-      <c r="AG5" t="s">
+      <c r="AN5" t="s">
         <v>44</v>
       </c>
-      <c r="AH5" t="s">
+      <c r="AO5" t="s">
         <v>98</v>
       </c>
-      <c r="AI5">
+      <c r="AP5">
         <v>6.4867911695789315E-2</v>
       </c>
-      <c r="AJ5" t="s">
+      <c r="AQ5" t="s">
         <v>38</v>
       </c>
-      <c r="AK5">
+      <c r="AR5">
         <v>0</v>
       </c>
-      <c r="AL5" t="s">
+      <c r="AS5" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:45" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>99</v>
       </c>
@@ -1663,47 +1747,62 @@
       <c r="V6" t="s">
         <v>41</v>
       </c>
-      <c r="X6">
+      <c r="X6" t="s">
+        <v>100</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>112</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>113</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>114</v>
+      </c>
+      <c r="AB6">
+        <v>9.9768911846666211E-2</v>
+      </c>
+      <c r="AE6">
         <v>0.11552511415525114</v>
       </c>
-      <c r="Y6">
+      <c r="AF6">
         <v>0.16263862301005233</v>
       </c>
-      <c r="Z6" t="s">
+      <c r="AG6" t="s">
         <v>100</v>
       </c>
-      <c r="AA6" t="s">
+      <c r="AH6" t="s">
         <v>8</v>
       </c>
-      <c r="AC6" t="s">
+      <c r="AJ6" t="s">
         <v>6</v>
       </c>
-      <c r="AD6" t="s">
+      <c r="AK6" t="s">
         <v>100</v>
       </c>
-      <c r="AE6">
+      <c r="AL6">
         <v>0.13104968035048054</v>
       </c>
-      <c r="AG6" t="s">
+      <c r="AN6" t="s">
         <v>44</v>
       </c>
-      <c r="AH6" t="s">
+      <c r="AO6" t="s">
         <v>100</v>
       </c>
-      <c r="AI6">
+      <c r="AP6">
         <v>0.181059958051627</v>
       </c>
-      <c r="AJ6" t="s">
+      <c r="AQ6" t="s">
         <v>38</v>
       </c>
-      <c r="AK6">
+      <c r="AR6">
         <v>0</v>
       </c>
-      <c r="AL6" t="s">
+      <c r="AS6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I7" t="s">
         <v>40</v>
       </c>
@@ -1740,38 +1839,53 @@
       <c r="V7" t="s">
         <v>41</v>
       </c>
-      <c r="X7">
+      <c r="X7" t="s">
+        <v>101</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>112</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>113</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>114</v>
+      </c>
+      <c r="AB7">
+        <v>0.11643668864269692</v>
+      </c>
+      <c r="AE7">
         <v>0.11552511415525114</v>
       </c>
-      <c r="Y7">
+      <c r="AF7">
         <v>5.3125160563193538E-2</v>
       </c>
-      <c r="Z7" t="s">
+      <c r="AG7" t="s">
         <v>101</v>
       </c>
-      <c r="AA7" t="s">
+      <c r="AH7" t="s">
         <v>8</v>
       </c>
-      <c r="AC7" t="s">
+      <c r="AJ7" t="s">
         <v>6</v>
       </c>
-      <c r="AD7" t="s">
+      <c r="AK7" t="s">
         <v>101</v>
       </c>
-      <c r="AE7">
+      <c r="AL7">
         <v>0.11255019110607196</v>
       </c>
-      <c r="AG7" t="s">
+      <c r="AN7" t="s">
         <v>44</v>
       </c>
-      <c r="AH7" t="s">
+      <c r="AO7" t="s">
         <v>101</v>
       </c>
-      <c r="AI7">
+      <c r="AP7">
         <v>0.29479690034051531</v>
       </c>
     </row>
-    <row r="8" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I8" t="s">
         <v>40</v>
       </c>
@@ -1808,38 +1922,53 @@
       <c r="V8" t="s">
         <v>41</v>
       </c>
-      <c r="X8">
+      <c r="X8" t="s">
+        <v>102</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>112</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>113</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>114</v>
+      </c>
+      <c r="AB8">
+        <v>0.10940838034391356</v>
+      </c>
+      <c r="AE8">
         <v>2.1004566210045664E-2</v>
       </c>
-      <c r="Y8">
+      <c r="AF8">
         <v>3.6291010947302131E-2</v>
       </c>
-      <c r="Z8" t="s">
+      <c r="AG8" t="s">
         <v>102</v>
       </c>
-      <c r="AA8" t="s">
+      <c r="AH8" t="s">
         <v>8</v>
       </c>
-      <c r="AC8" t="s">
+      <c r="AJ8" t="s">
         <v>6</v>
       </c>
-      <c r="AD8" t="s">
+      <c r="AK8" t="s">
         <v>102</v>
       </c>
-      <c r="AE8">
+      <c r="AL8">
         <v>2.3834110177054908E-2</v>
       </c>
-      <c r="AG8" t="s">
+      <c r="AN8" t="s">
         <v>44</v>
       </c>
-      <c r="AH8" t="s">
+      <c r="AO8" t="s">
         <v>102</v>
       </c>
-      <c r="AI8">
+      <c r="AP8">
         <v>0.18791773337227902</v>
       </c>
     </row>
-    <row r="9" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I9" t="s">
         <v>40</v>
       </c>
@@ -1876,38 +2005,53 @@
       <c r="V9" t="s">
         <v>41</v>
       </c>
-      <c r="X9">
+      <c r="X9" t="s">
+        <v>103</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>112</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>113</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>114</v>
+      </c>
+      <c r="AB9">
+        <v>0.10847532794127643</v>
+      </c>
+      <c r="AE9">
         <v>0.11552511415525114</v>
       </c>
-      <c r="Y9">
+      <c r="AF9">
         <v>0.16263862301005233</v>
       </c>
-      <c r="Z9" t="s">
+      <c r="AG9" t="s">
         <v>103</v>
       </c>
-      <c r="AA9" t="s">
+      <c r="AH9" t="s">
         <v>8</v>
       </c>
-      <c r="AC9" t="s">
+      <c r="AJ9" t="s">
         <v>6</v>
       </c>
-      <c r="AD9" t="s">
+      <c r="AK9" t="s">
         <v>103</v>
       </c>
-      <c r="AE9">
+      <c r="AL9">
         <v>0.11748145961359424</v>
       </c>
-      <c r="AG9" t="s">
+      <c r="AN9" t="s">
         <v>44</v>
       </c>
-      <c r="AH9" t="s">
+      <c r="AO9" t="s">
         <v>103</v>
       </c>
-      <c r="AI9">
+      <c r="AP9">
         <v>0.13319460828738694</v>
       </c>
     </row>
-    <row r="10" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I10" t="s">
         <v>40</v>
       </c>
@@ -1944,38 +2088,53 @@
       <c r="V10" t="s">
         <v>41</v>
       </c>
-      <c r="X10">
+      <c r="X10" t="s">
+        <v>104</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>112</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>113</v>
+      </c>
+      <c r="AA10" t="s">
+        <v>114</v>
+      </c>
+      <c r="AB10">
+        <v>9.6906035478828256E-2</v>
+      </c>
+      <c r="AE10">
         <v>0.11552511415525114</v>
       </c>
-      <c r="Y10">
+      <c r="AF10">
         <v>5.3125160563193538E-2</v>
       </c>
-      <c r="Z10" t="s">
+      <c r="AG10" t="s">
         <v>104</v>
       </c>
-      <c r="AA10" t="s">
+      <c r="AH10" t="s">
         <v>8</v>
       </c>
-      <c r="AC10" t="s">
+      <c r="AJ10" t="s">
         <v>6</v>
       </c>
-      <c r="AD10" t="s">
+      <c r="AK10" t="s">
         <v>104</v>
       </c>
-      <c r="AE10">
+      <c r="AL10">
         <v>8.4800799390331486E-2</v>
       </c>
-      <c r="AG10" t="s">
+      <c r="AN10" t="s">
         <v>44</v>
       </c>
-      <c r="AH10" t="s">
+      <c r="AO10" t="s">
         <v>104</v>
       </c>
-      <c r="AI10">
+      <c r="AP10">
         <v>0.27571202448049736</v>
       </c>
     </row>
-    <row r="11" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I11" t="s">
         <v>40</v>
       </c>
@@ -2012,38 +2171,53 @@
       <c r="V11" t="s">
         <v>41</v>
       </c>
-      <c r="X11">
+      <c r="X11" t="s">
+        <v>105</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>112</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>113</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>114</v>
+      </c>
+      <c r="AB11">
+        <v>0.10141534697206553</v>
+      </c>
+      <c r="AE11">
         <v>2.1004566210045664E-2</v>
       </c>
-      <c r="Y11">
+      <c r="AF11">
         <v>3.6291010947302131E-2</v>
       </c>
-      <c r="Z11" t="s">
+      <c r="AG11" t="s">
         <v>105</v>
       </c>
-      <c r="AA11" t="s">
+      <c r="AH11" t="s">
         <v>8</v>
       </c>
-      <c r="AC11" t="s">
+      <c r="AJ11" t="s">
         <v>6</v>
       </c>
-      <c r="AD11" t="s">
+      <c r="AK11" t="s">
         <v>105</v>
       </c>
-      <c r="AE11">
+      <c r="AL11">
         <v>2.0570847331150249E-2</v>
       </c>
-      <c r="AG11" t="s">
+      <c r="AN11" t="s">
         <v>44</v>
       </c>
-      <c r="AH11" t="s">
+      <c r="AO11" t="s">
         <v>105</v>
       </c>
-      <c r="AI11">
+      <c r="AP11">
         <v>9.8544131462115603E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I12" t="s">
         <v>40</v>
       </c>
@@ -2080,38 +2254,53 @@
       <c r="V12" t="s">
         <v>41</v>
       </c>
-      <c r="X12">
+      <c r="X12" t="s">
+        <v>106</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>112</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>113</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>114</v>
+      </c>
+      <c r="AB12">
+        <v>0.12014008020118261</v>
+      </c>
+      <c r="AE12">
         <v>0.11301369863013698</v>
       </c>
-      <c r="Y12">
+      <c r="AF12">
         <v>0.15910300077070333</v>
       </c>
-      <c r="Z12" t="s">
+      <c r="AG12" t="s">
         <v>106</v>
       </c>
-      <c r="AA12" t="s">
+      <c r="AH12" t="s">
         <v>8</v>
       </c>
-      <c r="AC12" t="s">
+      <c r="AJ12" t="s">
         <v>6</v>
       </c>
-      <c r="AD12" t="s">
+      <c r="AK12" t="s">
         <v>106</v>
       </c>
-      <c r="AE12">
+      <c r="AL12">
         <v>0.13067071966028027</v>
       </c>
-      <c r="AG12" t="s">
+      <c r="AN12" t="s">
         <v>44</v>
       </c>
-      <c r="AH12" t="s">
+      <c r="AO12" t="s">
         <v>106</v>
       </c>
-      <c r="AI12">
+      <c r="AP12">
         <v>9.4996431311812124E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I13" t="s">
         <v>40</v>
       </c>
@@ -2148,38 +2337,53 @@
       <c r="V13" t="s">
         <v>41</v>
       </c>
-      <c r="X13">
+      <c r="X13" t="s">
+        <v>107</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>112</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>113</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>114</v>
+      </c>
+      <c r="AB13">
+        <v>0.14508291986678451</v>
+      </c>
+      <c r="AE13">
         <v>0.11301369863013698</v>
       </c>
-      <c r="Y13">
+      <c r="AF13">
         <v>5.197026576834151E-2</v>
       </c>
-      <c r="Z13" t="s">
+      <c r="AG13" t="s">
         <v>107</v>
       </c>
-      <c r="AA13" t="s">
+      <c r="AH13" t="s">
         <v>8</v>
       </c>
-      <c r="AC13" t="s">
+      <c r="AJ13" t="s">
         <v>6</v>
       </c>
-      <c r="AD13" t="s">
+      <c r="AK13" t="s">
         <v>107</v>
       </c>
-      <c r="AE13">
+      <c r="AL13">
         <v>0.11789293365992742</v>
       </c>
-      <c r="AG13" t="s">
+      <c r="AN13" t="s">
         <v>44</v>
       </c>
-      <c r="AH13" t="s">
+      <c r="AO13" t="s">
         <v>107</v>
       </c>
-      <c r="AI13">
+      <c r="AP13">
         <v>0.17683972082772126</v>
       </c>
     </row>
-    <row r="14" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I14" t="s">
         <v>40</v>
       </c>
@@ -2216,38 +2420,53 @@
       <c r="V14" t="s">
         <v>41</v>
       </c>
-      <c r="X14">
+      <c r="X14" t="s">
+        <v>108</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>112</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>113</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>114</v>
+      </c>
+      <c r="AB14">
+        <v>0.17450530143410589</v>
+      </c>
+      <c r="AE14">
         <v>2.0547945205479451E-2</v>
       </c>
-      <c r="Y14">
+      <c r="AF14">
         <v>3.5502075926708607E-2</v>
       </c>
-      <c r="Z14" t="s">
+      <c r="AG14" t="s">
         <v>108</v>
       </c>
-      <c r="AA14" t="s">
+      <c r="AH14" t="s">
         <v>8</v>
       </c>
-      <c r="AC14" t="s">
+      <c r="AJ14" t="s">
         <v>6</v>
       </c>
-      <c r="AD14" t="s">
+      <c r="AK14" t="s">
         <v>108</v>
       </c>
-      <c r="AE14">
+      <c r="AL14">
         <v>2.3910251649386354E-2</v>
       </c>
-      <c r="AG14" t="s">
+      <c r="AN14" t="s">
         <v>44</v>
       </c>
-      <c r="AH14" t="s">
+      <c r="AO14" t="s">
         <v>108</v>
       </c>
-      <c r="AI14">
+      <c r="AP14">
         <v>7.423298333369277E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I15" t="s">
         <v>46</v>
       </c>
@@ -2284,17 +2503,17 @@
       <c r="V15" t="s">
         <v>41</v>
       </c>
-      <c r="AC15" t="s">
+      <c r="AJ15" t="s">
         <v>5</v>
       </c>
-      <c r="AD15" t="s">
+      <c r="AK15" t="s">
         <v>92</v>
       </c>
-      <c r="AE15">
+      <c r="AL15">
         <v>0.11491480071761173</v>
       </c>
     </row>
-    <row r="16" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I16" t="s">
         <v>46</v>
       </c>
@@ -2331,17 +2550,17 @@
       <c r="V16" t="s">
         <v>41</v>
       </c>
-      <c r="AC16" t="s">
+      <c r="AJ16" t="s">
         <v>5</v>
       </c>
-      <c r="AD16" t="s">
+      <c r="AK16" t="s">
         <v>95</v>
       </c>
-      <c r="AE16">
+      <c r="AL16">
         <v>0.11343014511581903</v>
       </c>
     </row>
-    <row r="17" spans="9:31" x14ac:dyDescent="0.25">
+    <row r="17" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I17" t="s">
         <v>46</v>
       </c>
@@ -2378,17 +2597,17 @@
       <c r="V17" t="s">
         <v>41</v>
       </c>
-      <c r="AC17" t="s">
+      <c r="AJ17" t="s">
         <v>5</v>
       </c>
-      <c r="AD17" t="s">
+      <c r="AK17" t="s">
         <v>98</v>
       </c>
-      <c r="AE17">
+      <c r="AL17">
         <v>2.0885252413625318E-2</v>
       </c>
     </row>
-    <row r="18" spans="9:31" x14ac:dyDescent="0.25">
+    <row r="18" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I18" t="s">
         <v>46</v>
       </c>
@@ -2425,17 +2644,17 @@
       <c r="V18" t="s">
         <v>41</v>
       </c>
-      <c r="AC18" t="s">
+      <c r="AJ18" t="s">
         <v>5</v>
       </c>
-      <c r="AD18" t="s">
+      <c r="AK18" t="s">
         <v>100</v>
       </c>
-      <c r="AE18">
+      <c r="AL18">
         <v>0.11618686907147086</v>
       </c>
     </row>
-    <row r="19" spans="9:31" x14ac:dyDescent="0.25">
+    <row r="19" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I19" t="s">
         <v>46</v>
       </c>
@@ -2472,17 +2691,17 @@
       <c r="V19" t="s">
         <v>41</v>
       </c>
-      <c r="AC19" t="s">
+      <c r="AJ19" t="s">
         <v>5</v>
       </c>
-      <c r="AD19" t="s">
+      <c r="AK19" t="s">
         <v>101</v>
       </c>
-      <c r="AE19">
+      <c r="AL19">
         <v>0.11485062661500635</v>
       </c>
     </row>
-    <row r="20" spans="9:31" x14ac:dyDescent="0.25">
+    <row r="20" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I20" t="s">
         <v>46</v>
       </c>
@@ -2519,17 +2738,17 @@
       <c r="V20" t="s">
         <v>41</v>
       </c>
-      <c r="AC20" t="s">
+      <c r="AJ20" t="s">
         <v>5</v>
       </c>
-      <c r="AD20" t="s">
+      <c r="AK20" t="s">
         <v>102</v>
       </c>
-      <c r="AE20">
+      <c r="AL20">
         <v>2.1125383361665393E-2</v>
       </c>
     </row>
-    <row r="21" spans="9:31" x14ac:dyDescent="0.25">
+    <row r="21" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I21" t="s">
         <v>46</v>
       </c>
@@ -2566,17 +2785,17 @@
       <c r="V21" t="s">
         <v>41</v>
       </c>
-      <c r="AC21" t="s">
+      <c r="AJ21" t="s">
         <v>5</v>
       </c>
-      <c r="AD21" t="s">
+      <c r="AK21" t="s">
         <v>103</v>
       </c>
-      <c r="AE21">
+      <c r="AL21">
         <v>0.11653911207601672</v>
       </c>
     </row>
-    <row r="22" spans="9:31" x14ac:dyDescent="0.25">
+    <row r="22" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I22" t="s">
         <v>46</v>
       </c>
@@ -2613,17 +2832,17 @@
       <c r="V22" t="s">
         <v>41</v>
       </c>
-      <c r="AC22" t="s">
+      <c r="AJ22" t="s">
         <v>5</v>
       </c>
-      <c r="AD22" t="s">
+      <c r="AK22" t="s">
         <v>104</v>
       </c>
-      <c r="AE22">
+      <c r="AL22">
         <v>0.11417854497501884</v>
       </c>
     </row>
-    <row r="23" spans="9:31" x14ac:dyDescent="0.25">
+    <row r="23" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I23" t="s">
         <v>46</v>
       </c>
@@ -2660,17 +2879,17 @@
       <c r="V23" t="s">
         <v>41</v>
       </c>
-      <c r="AC23" t="s">
+      <c r="AJ23" t="s">
         <v>5</v>
       </c>
-      <c r="AD23" t="s">
+      <c r="AK23" t="s">
         <v>105</v>
       </c>
-      <c r="AE23">
+      <c r="AL23">
         <v>2.1131908763385672E-2</v>
       </c>
     </row>
-    <row r="24" spans="9:31" x14ac:dyDescent="0.25">
+    <row r="24" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I24" t="s">
         <v>46</v>
       </c>
@@ -2707,17 +2926,17 @@
       <c r="V24" t="s">
         <v>41</v>
       </c>
-      <c r="AC24" t="s">
+      <c r="AJ24" t="s">
         <v>5</v>
       </c>
-      <c r="AD24" t="s">
+      <c r="AK24" t="s">
         <v>106</v>
       </c>
-      <c r="AE24">
+      <c r="AL24">
         <v>0.11351511345077332</v>
       </c>
     </row>
-    <row r="25" spans="9:31" x14ac:dyDescent="0.25">
+    <row r="25" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I25" t="s">
         <v>46</v>
       </c>
@@ -2754,17 +2973,17 @@
       <c r="V25" t="s">
         <v>41</v>
       </c>
-      <c r="AC25" t="s">
+      <c r="AJ25" t="s">
         <v>5</v>
       </c>
-      <c r="AD25" t="s">
+      <c r="AK25" t="s">
         <v>107</v>
       </c>
-      <c r="AE25">
+      <c r="AL25">
         <v>0.11259215715032031</v>
       </c>
     </row>
-    <row r="26" spans="9:31" x14ac:dyDescent="0.25">
+    <row r="26" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I26" t="s">
         <v>46</v>
       </c>
@@ -2801,17 +3020,17 @@
       <c r="V26" t="s">
         <v>41</v>
       </c>
-      <c r="AC26" t="s">
+      <c r="AJ26" t="s">
         <v>5</v>
       </c>
-      <c r="AD26" t="s">
+      <c r="AK26" t="s">
         <v>108</v>
       </c>
-      <c r="AE26">
+      <c r="AL26">
         <v>2.0650086289286402E-2</v>
       </c>
     </row>
-    <row r="27" spans="9:31" x14ac:dyDescent="0.25">
+    <row r="27" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I27" t="s">
         <v>49</v>
       </c>
@@ -2849,7 +3068,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="28" spans="9:31" x14ac:dyDescent="0.25">
+    <row r="28" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I28" t="s">
         <v>49</v>
       </c>
@@ -2887,7 +3106,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="29" spans="9:31" x14ac:dyDescent="0.25">
+    <row r="29" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I29" t="s">
         <v>49</v>
       </c>
@@ -2925,7 +3144,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="30" spans="9:31" x14ac:dyDescent="0.25">
+    <row r="30" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I30" t="s">
         <v>49</v>
       </c>
@@ -2963,7 +3182,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="31" spans="9:31" x14ac:dyDescent="0.25">
+    <row r="31" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I31" t="s">
         <v>49</v>
       </c>
@@ -3001,7 +3220,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="32" spans="9:31" x14ac:dyDescent="0.25">
+    <row r="32" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I32" t="s">
         <v>49</v>
       </c>
@@ -3039,7 +3258,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="33" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="33" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I33" t="s">
         <v>49</v>
       </c>
@@ -3077,7 +3296,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="34" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="34" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I34" t="s">
         <v>49</v>
       </c>
@@ -3115,7 +3334,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="35" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="35" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I35" t="s">
         <v>49</v>
       </c>
@@ -3153,7 +3372,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="36" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="36" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I36" t="s">
         <v>49</v>
       </c>
@@ -3191,7 +3410,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="37" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I37" t="s">
         <v>49</v>
       </c>
@@ -3229,7 +3448,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="38" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="38" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I38" t="s">
         <v>49</v>
       </c>
@@ -3267,7 +3486,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="39" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="39" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I39" t="s">
         <v>52</v>
       </c>
@@ -3305,7 +3524,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="40" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="40" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I40" t="s">
         <v>52</v>
       </c>
@@ -3343,7 +3562,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="41" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I41" t="s">
         <v>52</v>
       </c>
@@ -3381,7 +3600,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="42" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="42" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I42" t="s">
         <v>52</v>
       </c>
@@ -3419,7 +3638,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="43" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I43" t="s">
         <v>52</v>
       </c>
@@ -3457,7 +3676,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="44" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I44" t="s">
         <v>52</v>
       </c>
@@ -3495,7 +3714,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="45" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="45" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I45" t="s">
         <v>52</v>
       </c>
@@ -3533,7 +3752,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="46" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="46" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I46" t="s">
         <v>52</v>
       </c>
@@ -3571,7 +3790,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="47" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="47" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I47" t="s">
         <v>52</v>
       </c>
@@ -3609,7 +3828,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="48" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="48" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I48" t="s">
         <v>52</v>
       </c>
@@ -3647,7 +3866,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="49" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="49" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I49" t="s">
         <v>52</v>
       </c>
@@ -3685,7 +3904,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="50" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="50" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I50" t="s">
         <v>52</v>
       </c>
@@ -3723,7 +3942,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="51" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="51" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I51" t="s">
         <v>55</v>
       </c>
@@ -3761,7 +3980,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="52" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="52" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I52" t="s">
         <v>55</v>
       </c>
@@ -3799,7 +4018,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="53" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="53" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I53" t="s">
         <v>55</v>
       </c>
@@ -3837,7 +4056,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="54" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="54" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I54" t="s">
         <v>55</v>
       </c>
@@ -3875,7 +4094,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="55" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="55" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I55" t="s">
         <v>55</v>
       </c>
@@ -3913,7 +4132,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="56" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="56" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I56" t="s">
         <v>55</v>
       </c>
@@ -3951,7 +4170,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="57" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="57" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I57" t="s">
         <v>55</v>
       </c>
@@ -3989,7 +4208,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="58" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="58" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I58" t="s">
         <v>55</v>
       </c>
@@ -4027,7 +4246,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="59" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="59" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I59" t="s">
         <v>55</v>
       </c>
@@ -4065,7 +4284,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="60" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="60" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I60" t="s">
         <v>55</v>
       </c>
@@ -4103,7 +4322,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="61" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="61" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I61" t="s">
         <v>55</v>
       </c>
@@ -4141,7 +4360,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="62" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="62" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I62" t="s">
         <v>55</v>
       </c>
@@ -4179,7 +4398,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="63" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="63" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I63" t="s">
         <v>58</v>
       </c>
@@ -4217,7 +4436,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="64" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="64" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I64" t="s">
         <v>58</v>
       </c>
@@ -4255,7 +4474,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="65" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="65" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I65" t="s">
         <v>58</v>
       </c>
@@ -4293,7 +4512,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="66" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="66" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I66" t="s">
         <v>58</v>
       </c>
@@ -4331,7 +4550,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="67" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="67" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I67" t="s">
         <v>58</v>
       </c>
@@ -4369,7 +4588,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="68" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="68" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I68" t="s">
         <v>58</v>
       </c>
@@ -4407,7 +4626,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="69" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="69" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I69" t="s">
         <v>58</v>
       </c>
@@ -4445,7 +4664,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="70" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="70" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I70" t="s">
         <v>58</v>
       </c>
@@ -4483,7 +4702,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="71" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="71" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I71" t="s">
         <v>58</v>
       </c>
@@ -4521,7 +4740,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="72" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="72" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I72" t="s">
         <v>58</v>
       </c>
@@ -4559,7 +4778,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="73" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="73" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I73" t="s">
         <v>58</v>
       </c>
@@ -4597,7 +4816,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="74" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="74" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I74" t="s">
         <v>58</v>
       </c>
@@ -4635,7 +4854,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="75" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="75" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I75" t="s">
         <v>61</v>
       </c>
@@ -4673,7 +4892,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="76" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="76" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I76" t="s">
         <v>61</v>
       </c>
@@ -4711,7 +4930,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="77" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="77" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I77" t="s">
         <v>61</v>
       </c>
@@ -4749,7 +4968,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="78" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="78" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I78" t="s">
         <v>61</v>
       </c>
@@ -4787,7 +5006,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="79" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="79" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I79" t="s">
         <v>61</v>
       </c>
@@ -4825,7 +5044,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="80" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="80" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I80" t="s">
         <v>61</v>
       </c>
@@ -4863,7 +5082,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="81" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="81" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I81" t="s">
         <v>61</v>
       </c>
@@ -4901,7 +5120,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="82" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="82" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I82" t="s">
         <v>61</v>
       </c>
@@ -4939,7 +5158,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="83" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="83" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I83" t="s">
         <v>61</v>
       </c>
@@ -4977,7 +5196,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="84" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="84" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I84" t="s">
         <v>61</v>
       </c>
@@ -5015,7 +5234,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="85" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="85" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I85" t="s">
         <v>61</v>
       </c>
@@ -5053,7 +5272,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="86" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="86" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I86" t="s">
         <v>61</v>
       </c>
@@ -5091,7 +5310,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="87" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="87" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I87" t="s">
         <v>64</v>
       </c>
@@ -5129,7 +5348,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="88" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="88" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I88" t="s">
         <v>64</v>
       </c>
@@ -5167,7 +5386,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="89" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="89" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I89" t="s">
         <v>64</v>
       </c>
@@ -5205,7 +5424,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="90" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="90" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I90" t="s">
         <v>64</v>
       </c>
@@ -5243,7 +5462,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="91" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="91" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I91" t="s">
         <v>64</v>
       </c>
@@ -5281,7 +5500,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="92" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="92" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I92" t="s">
         <v>64</v>
       </c>
@@ -5319,7 +5538,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="93" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="93" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I93" t="s">
         <v>64</v>
       </c>
@@ -5357,7 +5576,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="94" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="94" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I94" t="s">
         <v>64</v>
       </c>
@@ -5395,7 +5614,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="95" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="95" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I95" t="s">
         <v>64</v>
       </c>
@@ -5433,7 +5652,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="96" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="96" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I96" t="s">
         <v>64</v>
       </c>
@@ -5471,7 +5690,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="97" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="97" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I97" t="s">
         <v>64</v>
       </c>
@@ -5509,7 +5728,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="98" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="98" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I98" t="s">
         <v>64</v>
       </c>
@@ -5547,7 +5766,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="99" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="99" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I99" t="s">
         <v>67</v>
       </c>
@@ -5585,7 +5804,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="100" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="100" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I100" t="s">
         <v>67</v>
       </c>
@@ -5623,7 +5842,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="101" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="101" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I101" t="s">
         <v>67</v>
       </c>
@@ -5661,7 +5880,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="102" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="102" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I102" t="s">
         <v>67</v>
       </c>
@@ -5699,7 +5918,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="103" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="103" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I103" t="s">
         <v>67</v>
       </c>
@@ -5737,7 +5956,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="104" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="104" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I104" t="s">
         <v>67</v>
       </c>
@@ -5775,7 +5994,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="105" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="105" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I105" t="s">
         <v>67</v>
       </c>
@@ -5813,7 +6032,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="106" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="106" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I106" t="s">
         <v>67</v>
       </c>
@@ -5851,7 +6070,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="107" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="107" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I107" t="s">
         <v>67</v>
       </c>
@@ -5889,7 +6108,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="108" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="108" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I108" t="s">
         <v>67</v>
       </c>
@@ -5927,7 +6146,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="109" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="109" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I109" t="s">
         <v>67</v>
       </c>
@@ -5965,7 +6184,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="110" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="110" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I110" t="s">
         <v>67</v>
       </c>
@@ -6003,7 +6222,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="111" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="111" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I111" t="s">
         <v>70</v>
       </c>
@@ -6041,7 +6260,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="112" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="112" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I112" t="s">
         <v>70</v>
       </c>
@@ -6079,7 +6298,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="113" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="113" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I113" t="s">
         <v>70</v>
       </c>
@@ -6117,7 +6336,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="114" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="114" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I114" t="s">
         <v>70</v>
       </c>
@@ -6155,7 +6374,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="115" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="115" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I115" t="s">
         <v>70</v>
       </c>
@@ -6193,7 +6412,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="116" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="116" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I116" t="s">
         <v>70</v>
       </c>
@@ -6231,7 +6450,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="117" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="117" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I117" t="s">
         <v>70</v>
       </c>
@@ -6269,7 +6488,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="118" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="118" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I118" t="s">
         <v>70</v>
       </c>
@@ -6307,7 +6526,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="119" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="119" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I119" t="s">
         <v>70</v>
       </c>
@@ -6345,7 +6564,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="120" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="120" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I120" t="s">
         <v>70</v>
       </c>
@@ -6383,7 +6602,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="121" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="121" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I121" t="s">
         <v>70</v>
       </c>
@@ -6421,7 +6640,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="122" spans="9:22" x14ac:dyDescent="0.25">
+    <row r="122" spans="9:22" x14ac:dyDescent="0.35">
       <c r="I122" t="s">
         <v>70</v>
       </c>
@@ -6467,17 +6686,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F0573AE-84FA-4F18-8D18-B7F3EC5B3273}">
   <dimension ref="B4:K14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>12</v>
       </c>
@@ -6509,7 +6728,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>14</v>
       </c>
@@ -6523,7 +6742,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>17</v>
       </c>
@@ -6537,12 +6756,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>12</v>
       </c>
@@ -6562,7 +6781,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>17</v>
       </c>
@@ -6582,7 +6801,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:11" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>14</v>
       </c>
@@ -6610,18 +6829,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48BDE16D-C995-4313-9FD3-ABCD01C0EB3D}">
   <dimension ref="B6:T11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="6" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>1</v>
       </c>
@@ -6653,7 +6872,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>20</v>
       </c>
@@ -6682,7 +6901,7 @@
         <v>44.756</v>
       </c>
     </row>
-    <row r="9" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>21</v>
       </c>
@@ -6711,7 +6930,7 @@
         <v>15.344000000000001</v>
       </c>
     </row>
-    <row r="10" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>22</v>
       </c>
@@ -6740,7 +6959,7 @@
         <v>60.419999999999995</v>
       </c>
     </row>
-    <row r="11" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:20" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
adding wind onshore chartericis through ncap_af
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72AECADC-72FD-43AA-939A-06918316C16E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BBCE6ED-7741-4A96-BBBB-4F9FCFD9A17F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -426,10 +426,10 @@
     <t>Year</t>
   </si>
   <si>
-    <t>TFM_DINS</t>
-  </si>
-  <si>
     <t>~TFM_INS-AT</t>
+  </si>
+  <si>
+    <t>TFM_INS</t>
   </si>
 </sst>
 </file>
@@ -1284,7 +1284,7 @@
         <v>109</v>
       </c>
       <c r="X1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="AE1" t="s">
         <v>109</v>
@@ -1296,7 +1296,7 @@
         <v>109</v>
       </c>
       <c r="AR1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" spans="1:47" x14ac:dyDescent="0.35">
@@ -1481,7 +1481,7 @@
         <v>113</v>
       </c>
       <c r="AB3">
-        <v>9.8663766736899333E-2</v>
+        <v>1E-3</v>
       </c>
       <c r="AE3">
         <v>0.11426940639269406</v>
@@ -1585,7 +1585,7 @@
         <v>113</v>
       </c>
       <c r="AB4">
-        <v>0.10284697206552026</v>
+        <v>1E-3</v>
       </c>
       <c r="AE4">
         <v>0.11426940639269406</v>
@@ -1689,7 +1689,7 @@
         <v>113</v>
       </c>
       <c r="AB5">
-        <v>0.10723479236049754</v>
+        <v>1E-3</v>
       </c>
       <c r="AE5">
         <v>2.0776255707762557E-2</v>
@@ -1787,7 +1787,7 @@
         <v>113</v>
       </c>
       <c r="AB6">
-        <v>9.9768911846666211E-2</v>
+        <v>1E-3</v>
       </c>
       <c r="AE6">
         <v>0.11552511415525114</v>
@@ -1882,7 +1882,7 @@
         <v>113</v>
       </c>
       <c r="AB7">
-        <v>0.11643668864269692</v>
+        <v>1E-3</v>
       </c>
       <c r="AE7">
         <v>0.11552511415525114</v>
@@ -1977,7 +1977,7 @@
         <v>113</v>
       </c>
       <c r="AB8">
-        <v>0.10940838034391356</v>
+        <v>1E-3</v>
       </c>
       <c r="AE8">
         <v>2.1004566210045664E-2</v>
@@ -2072,7 +2072,7 @@
         <v>113</v>
       </c>
       <c r="AB9">
-        <v>0.10847532794127643</v>
+        <v>1E-3</v>
       </c>
       <c r="AE9">
         <v>0.11552511415525114</v>
@@ -2167,7 +2167,7 @@
         <v>113</v>
       </c>
       <c r="AB10">
-        <v>9.6906035478828256E-2</v>
+        <v>1E-3</v>
       </c>
       <c r="AE10">
         <v>0.11552511415525114</v>
@@ -2262,7 +2262,7 @@
         <v>113</v>
       </c>
       <c r="AB11">
-        <v>0.10141534697206553</v>
+        <v>1E-3</v>
       </c>
       <c r="AE11">
         <v>2.1004566210045664E-2</v>
@@ -2357,7 +2357,7 @@
         <v>113</v>
       </c>
       <c r="AB12">
-        <v>0.12014008020118261</v>
+        <v>1E-3</v>
       </c>
       <c r="AE12">
         <v>0.11301369863013698</v>
@@ -2452,7 +2452,7 @@
         <v>113</v>
       </c>
       <c r="AB13">
-        <v>0.14508291986678451</v>
+        <v>1E-3</v>
       </c>
       <c r="AE13">
         <v>0.11301369863013698</v>
@@ -2547,7 +2547,7 @@
         <v>113</v>
       </c>
       <c r="AB14">
-        <v>0.17450530143410589</v>
+        <v>1E-3</v>
       </c>
       <c r="AE14">
         <v>2.0547945205479451E-2</v>

</xml_diff>

<commit_message>
adding wind onshore chartericis through ncap_af II
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BBCE6ED-7741-4A96-BBBB-4F9FCFD9A17F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47AC793A-7B53-4227-AA08-1A72392CC977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1381" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1381" uniqueCount="119">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -427,9 +427,6 @@
   </si>
   <si>
     <t>~TFM_INS-AT</t>
-  </si>
-  <si>
-    <t>TFM_INS</t>
   </si>
 </sst>
 </file>
@@ -1284,7 +1281,7 @@
         <v>109</v>
       </c>
       <c r="X1" t="s">
-        <v>119</v>
+        <v>75</v>
       </c>
       <c r="AE1" t="s">
         <v>109</v>

</xml_diff>

<commit_message>
adding wind onshore chartericis through ncap_af III
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47AC793A-7B53-4227-AA08-1A72392CC977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5B5E3A0-78A5-4624-BAC4-A58BD3DC998F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -411,9 +411,6 @@
     <t>ncap_af</t>
   </si>
   <si>
-    <t>Wind onshore</t>
-  </si>
-  <si>
     <t>PSET_PN</t>
   </si>
   <si>
@@ -427,6 +424,9 @@
   </si>
   <si>
     <t>~TFM_INS-AT</t>
+  </si>
+  <si>
+    <t>e*won*</t>
   </si>
 </sst>
 </file>
@@ -1293,7 +1293,7 @@
         <v>109</v>
       </c>
       <c r="AR1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:47" x14ac:dyDescent="0.35">
@@ -1358,13 +1358,13 @@
         <v>110</v>
       </c>
       <c r="Z2" t="s">
+        <v>114</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>113</v>
+      </c>
+      <c r="AB2" t="s">
         <v>115</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>114</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>116</v>
       </c>
       <c r="AE2" t="s">
         <v>34</v>
@@ -1397,7 +1397,7 @@
         <v>35</v>
       </c>
       <c r="AR2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="AS2" t="s">
         <v>32</v>
@@ -1475,7 +1475,7 @@
         <v>112</v>
       </c>
       <c r="AA3" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="AB3">
         <v>1E-3</v>
@@ -1579,7 +1579,7 @@
         <v>112</v>
       </c>
       <c r="AA4" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="AB4">
         <v>1E-3</v>
@@ -1683,7 +1683,7 @@
         <v>112</v>
       </c>
       <c r="AA5" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="AB5">
         <v>1E-3</v>
@@ -1781,7 +1781,7 @@
         <v>112</v>
       </c>
       <c r="AA6" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="AB6">
         <v>1E-3</v>
@@ -1876,7 +1876,7 @@
         <v>112</v>
       </c>
       <c r="AA7" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="AB7">
         <v>1E-3</v>
@@ -1971,7 +1971,7 @@
         <v>112</v>
       </c>
       <c r="AA8" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="AB8">
         <v>1E-3</v>
@@ -2066,7 +2066,7 @@
         <v>112</v>
       </c>
       <c r="AA9" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="AB9">
         <v>1E-3</v>
@@ -2161,7 +2161,7 @@
         <v>112</v>
       </c>
       <c r="AA10" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="AB10">
         <v>1E-3</v>
@@ -2256,7 +2256,7 @@
         <v>112</v>
       </c>
       <c r="AA11" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="AB11">
         <v>1E-3</v>
@@ -2351,7 +2351,7 @@
         <v>112</v>
       </c>
       <c r="AA12" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="AB12">
         <v>1E-3</v>
@@ -2446,7 +2446,7 @@
         <v>112</v>
       </c>
       <c r="AA13" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="AB13">
         <v>1E-3</v>
@@ -2541,7 +2541,7 @@
         <v>112</v>
       </c>
       <c r="AA14" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="AB14">
         <v>1E-3</v>

</xml_diff>

<commit_message>
adding wind onshore chartericis through ncap_af IV
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5B5E3A0-78A5-4624-BAC4-A58BD3DC998F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F09CC301-8C54-4095-AE1E-35AE88C1C474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1381" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1478" uniqueCount="119">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -1352,18 +1352,21 @@
         <v>12</v>
       </c>
       <c r="X2" t="s">
+        <v>116</v>
+      </c>
+      <c r="Y2" t="s">
         <v>32</v>
       </c>
-      <c r="Y2" t="s">
+      <c r="Z2" t="s">
         <v>110</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="AA2" t="s">
         <v>114</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="AB2" t="s">
         <v>113</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AC2" t="s">
         <v>115</v>
       </c>
       <c r="AE2" t="s">
@@ -1465,19 +1468,22 @@
       <c r="V3" t="s">
         <v>40</v>
       </c>
-      <c r="X3" t="s">
+      <c r="X3">
+        <v>2022</v>
+      </c>
+      <c r="Y3" t="s">
         <v>91</v>
       </c>
-      <c r="Y3" t="s">
+      <c r="Z3" t="s">
         <v>111</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="AA3" t="s">
         <v>112</v>
       </c>
-      <c r="AA3" t="s">
+      <c r="AB3" t="s">
         <v>118</v>
       </c>
-      <c r="AB3">
+      <c r="AC3">
         <v>1E-3</v>
       </c>
       <c r="AE3">
@@ -1569,19 +1575,22 @@
       <c r="V4" t="s">
         <v>40</v>
       </c>
-      <c r="X4" t="s">
+      <c r="X4">
+        <v>2022</v>
+      </c>
+      <c r="Y4" t="s">
         <v>94</v>
       </c>
-      <c r="Y4" t="s">
+      <c r="Z4" t="s">
         <v>111</v>
       </c>
-      <c r="Z4" t="s">
+      <c r="AA4" t="s">
         <v>112</v>
       </c>
-      <c r="AA4" t="s">
+      <c r="AB4" t="s">
         <v>118</v>
       </c>
-      <c r="AB4">
+      <c r="AC4">
         <v>1E-3</v>
       </c>
       <c r="AE4">
@@ -1673,19 +1682,22 @@
       <c r="V5" t="s">
         <v>40</v>
       </c>
-      <c r="X5" t="s">
+      <c r="X5">
+        <v>2022</v>
+      </c>
+      <c r="Y5" t="s">
         <v>97</v>
       </c>
-      <c r="Y5" t="s">
+      <c r="Z5" t="s">
         <v>111</v>
       </c>
-      <c r="Z5" t="s">
+      <c r="AA5" t="s">
         <v>112</v>
       </c>
-      <c r="AA5" t="s">
+      <c r="AB5" t="s">
         <v>118</v>
       </c>
-      <c r="AB5">
+      <c r="AC5">
         <v>1E-3</v>
       </c>
       <c r="AE5">
@@ -1771,19 +1783,22 @@
       <c r="V6" t="s">
         <v>40</v>
       </c>
-      <c r="X6" t="s">
+      <c r="X6">
+        <v>2022</v>
+      </c>
+      <c r="Y6" t="s">
         <v>99</v>
       </c>
-      <c r="Y6" t="s">
+      <c r="Z6" t="s">
         <v>111</v>
       </c>
-      <c r="Z6" t="s">
+      <c r="AA6" t="s">
         <v>112</v>
       </c>
-      <c r="AA6" t="s">
+      <c r="AB6" t="s">
         <v>118</v>
       </c>
-      <c r="AB6">
+      <c r="AC6">
         <v>1E-3</v>
       </c>
       <c r="AE6">
@@ -1866,19 +1881,22 @@
       <c r="V7" t="s">
         <v>40</v>
       </c>
-      <c r="X7" t="s">
+      <c r="X7">
+        <v>2022</v>
+      </c>
+      <c r="Y7" t="s">
         <v>100</v>
       </c>
-      <c r="Y7" t="s">
+      <c r="Z7" t="s">
         <v>111</v>
       </c>
-      <c r="Z7" t="s">
+      <c r="AA7" t="s">
         <v>112</v>
       </c>
-      <c r="AA7" t="s">
+      <c r="AB7" t="s">
         <v>118</v>
       </c>
-      <c r="AB7">
+      <c r="AC7">
         <v>1E-3</v>
       </c>
       <c r="AE7">
@@ -1961,19 +1979,22 @@
       <c r="V8" t="s">
         <v>40</v>
       </c>
-      <c r="X8" t="s">
+      <c r="X8">
+        <v>2022</v>
+      </c>
+      <c r="Y8" t="s">
         <v>101</v>
       </c>
-      <c r="Y8" t="s">
+      <c r="Z8" t="s">
         <v>111</v>
       </c>
-      <c r="Z8" t="s">
+      <c r="AA8" t="s">
         <v>112</v>
       </c>
-      <c r="AA8" t="s">
+      <c r="AB8" t="s">
         <v>118</v>
       </c>
-      <c r="AB8">
+      <c r="AC8">
         <v>1E-3</v>
       </c>
       <c r="AE8">
@@ -2056,19 +2077,22 @@
       <c r="V9" t="s">
         <v>40</v>
       </c>
-      <c r="X9" t="s">
+      <c r="X9">
+        <v>2022</v>
+      </c>
+      <c r="Y9" t="s">
         <v>102</v>
       </c>
-      <c r="Y9" t="s">
+      <c r="Z9" t="s">
         <v>111</v>
       </c>
-      <c r="Z9" t="s">
+      <c r="AA9" t="s">
         <v>112</v>
       </c>
-      <c r="AA9" t="s">
+      <c r="AB9" t="s">
         <v>118</v>
       </c>
-      <c r="AB9">
+      <c r="AC9">
         <v>1E-3</v>
       </c>
       <c r="AE9">
@@ -2151,19 +2175,22 @@
       <c r="V10" t="s">
         <v>40</v>
       </c>
-      <c r="X10" t="s">
+      <c r="X10">
+        <v>2022</v>
+      </c>
+      <c r="Y10" t="s">
         <v>103</v>
       </c>
-      <c r="Y10" t="s">
+      <c r="Z10" t="s">
         <v>111</v>
       </c>
-      <c r="Z10" t="s">
+      <c r="AA10" t="s">
         <v>112</v>
       </c>
-      <c r="AA10" t="s">
+      <c r="AB10" t="s">
         <v>118</v>
       </c>
-      <c r="AB10">
+      <c r="AC10">
         <v>1E-3</v>
       </c>
       <c r="AE10">
@@ -2246,19 +2273,22 @@
       <c r="V11" t="s">
         <v>40</v>
       </c>
-      <c r="X11" t="s">
+      <c r="X11">
+        <v>2022</v>
+      </c>
+      <c r="Y11" t="s">
         <v>104</v>
       </c>
-      <c r="Y11" t="s">
+      <c r="Z11" t="s">
         <v>111</v>
       </c>
-      <c r="Z11" t="s">
+      <c r="AA11" t="s">
         <v>112</v>
       </c>
-      <c r="AA11" t="s">
+      <c r="AB11" t="s">
         <v>118</v>
       </c>
-      <c r="AB11">
+      <c r="AC11">
         <v>1E-3</v>
       </c>
       <c r="AE11">
@@ -2341,19 +2371,22 @@
       <c r="V12" t="s">
         <v>40</v>
       </c>
-      <c r="X12" t="s">
+      <c r="X12">
+        <v>2022</v>
+      </c>
+      <c r="Y12" t="s">
         <v>105</v>
       </c>
-      <c r="Y12" t="s">
+      <c r="Z12" t="s">
         <v>111</v>
       </c>
-      <c r="Z12" t="s">
+      <c r="AA12" t="s">
         <v>112</v>
       </c>
-      <c r="AA12" t="s">
+      <c r="AB12" t="s">
         <v>118</v>
       </c>
-      <c r="AB12">
+      <c r="AC12">
         <v>1E-3</v>
       </c>
       <c r="AE12">
@@ -2436,19 +2469,22 @@
       <c r="V13" t="s">
         <v>40</v>
       </c>
-      <c r="X13" t="s">
+      <c r="X13">
+        <v>2022</v>
+      </c>
+      <c r="Y13" t="s">
         <v>106</v>
       </c>
-      <c r="Y13" t="s">
+      <c r="Z13" t="s">
         <v>111</v>
       </c>
-      <c r="Z13" t="s">
+      <c r="AA13" t="s">
         <v>112</v>
       </c>
-      <c r="AA13" t="s">
+      <c r="AB13" t="s">
         <v>118</v>
       </c>
-      <c r="AB13">
+      <c r="AC13">
         <v>1E-3</v>
       </c>
       <c r="AE13">
@@ -2531,19 +2567,22 @@
       <c r="V14" t="s">
         <v>40</v>
       </c>
-      <c r="X14" t="s">
+      <c r="X14">
+        <v>2022</v>
+      </c>
+      <c r="Y14" t="s">
         <v>107</v>
       </c>
-      <c r="Y14" t="s">
+      <c r="Z14" t="s">
         <v>111</v>
       </c>
-      <c r="Z14" t="s">
+      <c r="AA14" t="s">
         <v>112</v>
       </c>
-      <c r="AA14" t="s">
+      <c r="AB14" t="s">
         <v>118</v>
       </c>
-      <c r="AB14">
+      <c r="AC14">
         <v>1E-3</v>
       </c>
       <c r="AE14">
@@ -2626,6 +2665,24 @@
       <c r="V15" t="s">
         <v>40</v>
       </c>
+      <c r="X15">
+        <v>2025</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>91</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB15" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC15">
+        <v>1E-3</v>
+      </c>
       <c r="AJ15" t="s">
         <v>5</v>
       </c>
@@ -2673,6 +2730,24 @@
       <c r="V16" t="s">
         <v>40</v>
       </c>
+      <c r="X16">
+        <v>2025</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>94</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB16" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC16">
+        <v>1E-3</v>
+      </c>
       <c r="AJ16" t="s">
         <v>5</v>
       </c>
@@ -2720,6 +2795,24 @@
       <c r="V17" t="s">
         <v>40</v>
       </c>
+      <c r="X17">
+        <v>2025</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>97</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB17" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC17">
+        <v>1E-3</v>
+      </c>
       <c r="AJ17" t="s">
         <v>5</v>
       </c>
@@ -2767,6 +2860,24 @@
       <c r="V18" t="s">
         <v>40</v>
       </c>
+      <c r="X18">
+        <v>2025</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>99</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB18" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC18">
+        <v>1E-3</v>
+      </c>
       <c r="AJ18" t="s">
         <v>5</v>
       </c>
@@ -2814,6 +2925,24 @@
       <c r="V19" t="s">
         <v>40</v>
       </c>
+      <c r="X19">
+        <v>2025</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>100</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB19" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC19">
+        <v>1E-3</v>
+      </c>
       <c r="AJ19" t="s">
         <v>5</v>
       </c>
@@ -2861,6 +2990,24 @@
       <c r="V20" t="s">
         <v>40</v>
       </c>
+      <c r="X20">
+        <v>2025</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>101</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC20">
+        <v>1E-3</v>
+      </c>
       <c r="AJ20" t="s">
         <v>5</v>
       </c>
@@ -2908,6 +3055,24 @@
       <c r="V21" t="s">
         <v>40</v>
       </c>
+      <c r="X21">
+        <v>2025</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>102</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB21" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC21">
+        <v>1E-3</v>
+      </c>
       <c r="AJ21" t="s">
         <v>5</v>
       </c>
@@ -2955,6 +3120,24 @@
       <c r="V22" t="s">
         <v>40</v>
       </c>
+      <c r="X22">
+        <v>2025</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>103</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB22" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC22">
+        <v>1E-3</v>
+      </c>
       <c r="AJ22" t="s">
         <v>5</v>
       </c>
@@ -3002,6 +3185,24 @@
       <c r="V23" t="s">
         <v>40</v>
       </c>
+      <c r="X23">
+        <v>2025</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>104</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB23" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC23">
+        <v>1E-3</v>
+      </c>
       <c r="AJ23" t="s">
         <v>5</v>
       </c>
@@ -3049,6 +3250,24 @@
       <c r="V24" t="s">
         <v>40</v>
       </c>
+      <c r="X24">
+        <v>2025</v>
+      </c>
+      <c r="Y24" t="s">
+        <v>105</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB24" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC24">
+        <v>1E-3</v>
+      </c>
       <c r="AJ24" t="s">
         <v>5</v>
       </c>
@@ -3096,6 +3315,24 @@
       <c r="V25" t="s">
         <v>40</v>
       </c>
+      <c r="X25">
+        <v>2025</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>106</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB25" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC25">
+        <v>1E-3</v>
+      </c>
       <c r="AJ25" t="s">
         <v>5</v>
       </c>
@@ -3143,6 +3380,24 @@
       <c r="V26" t="s">
         <v>40</v>
       </c>
+      <c r="X26">
+        <v>2025</v>
+      </c>
+      <c r="Y26" t="s">
+        <v>107</v>
+      </c>
+      <c r="Z26" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA26" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB26" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC26">
+        <v>1E-3</v>
+      </c>
       <c r="AJ26" t="s">
         <v>5</v>
       </c>
@@ -3190,6 +3445,24 @@
       <c r="V27" t="s">
         <v>40</v>
       </c>
+      <c r="X27">
+        <v>2030</v>
+      </c>
+      <c r="Y27" t="s">
+        <v>91</v>
+      </c>
+      <c r="Z27" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA27" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB27" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC27">
+        <v>1E-3</v>
+      </c>
     </row>
     <row r="28" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I28" t="s">
@@ -3228,6 +3501,24 @@
       <c r="V28" t="s">
         <v>40</v>
       </c>
+      <c r="X28">
+        <v>2030</v>
+      </c>
+      <c r="Y28" t="s">
+        <v>94</v>
+      </c>
+      <c r="Z28" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA28" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB28" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC28">
+        <v>1E-3</v>
+      </c>
     </row>
     <row r="29" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I29" t="s">
@@ -3266,6 +3557,24 @@
       <c r="V29" t="s">
         <v>40</v>
       </c>
+      <c r="X29">
+        <v>2030</v>
+      </c>
+      <c r="Y29" t="s">
+        <v>97</v>
+      </c>
+      <c r="Z29" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA29" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB29" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC29">
+        <v>1E-3</v>
+      </c>
     </row>
     <row r="30" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I30" t="s">
@@ -3304,6 +3613,24 @@
       <c r="V30" t="s">
         <v>40</v>
       </c>
+      <c r="X30">
+        <v>2030</v>
+      </c>
+      <c r="Y30" t="s">
+        <v>99</v>
+      </c>
+      <c r="Z30" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA30" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB30" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC30">
+        <v>1E-3</v>
+      </c>
     </row>
     <row r="31" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I31" t="s">
@@ -3342,6 +3669,24 @@
       <c r="V31" t="s">
         <v>40</v>
       </c>
+      <c r="X31">
+        <v>2030</v>
+      </c>
+      <c r="Y31" t="s">
+        <v>100</v>
+      </c>
+      <c r="Z31" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA31" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB31" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC31">
+        <v>1E-3</v>
+      </c>
     </row>
     <row r="32" spans="9:38" x14ac:dyDescent="0.35">
       <c r="I32" t="s">
@@ -3380,8 +3725,26 @@
       <c r="V32" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="33" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="X32">
+        <v>2030</v>
+      </c>
+      <c r="Y32" t="s">
+        <v>101</v>
+      </c>
+      <c r="Z32" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA32" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB32" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC32">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="33" spans="9:29" x14ac:dyDescent="0.35">
       <c r="I33" t="s">
         <v>48</v>
       </c>
@@ -3418,8 +3781,26 @@
       <c r="V33" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="34" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="X33">
+        <v>2030</v>
+      </c>
+      <c r="Y33" t="s">
+        <v>102</v>
+      </c>
+      <c r="Z33" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA33" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB33" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC33">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="34" spans="9:29" x14ac:dyDescent="0.35">
       <c r="I34" t="s">
         <v>48</v>
       </c>
@@ -3456,8 +3837,26 @@
       <c r="V34" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="35" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="X34">
+        <v>2030</v>
+      </c>
+      <c r="Y34" t="s">
+        <v>103</v>
+      </c>
+      <c r="Z34" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA34" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB34" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC34">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="35" spans="9:29" x14ac:dyDescent="0.35">
       <c r="I35" t="s">
         <v>48</v>
       </c>
@@ -3494,8 +3893,26 @@
       <c r="V35" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="36" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="X35">
+        <v>2030</v>
+      </c>
+      <c r="Y35" t="s">
+        <v>104</v>
+      </c>
+      <c r="Z35" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA35" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB35" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC35">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="36" spans="9:29" x14ac:dyDescent="0.35">
       <c r="I36" t="s">
         <v>48</v>
       </c>
@@ -3532,8 +3949,26 @@
       <c r="V36" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="37" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="X36">
+        <v>2030</v>
+      </c>
+      <c r="Y36" t="s">
+        <v>105</v>
+      </c>
+      <c r="Z36" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA36" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB36" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC36">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="37" spans="9:29" x14ac:dyDescent="0.35">
       <c r="I37" t="s">
         <v>48</v>
       </c>
@@ -3570,8 +4005,26 @@
       <c r="V37" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="38" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="X37">
+        <v>2030</v>
+      </c>
+      <c r="Y37" t="s">
+        <v>106</v>
+      </c>
+      <c r="Z37" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA37" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB37" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC37">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="38" spans="9:29" x14ac:dyDescent="0.35">
       <c r="I38" t="s">
         <v>48</v>
       </c>
@@ -3608,8 +4061,26 @@
       <c r="V38" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="39" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="X38">
+        <v>2030</v>
+      </c>
+      <c r="Y38" t="s">
+        <v>107</v>
+      </c>
+      <c r="Z38" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA38" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB38" t="s">
+        <v>118</v>
+      </c>
+      <c r="AC38">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="39" spans="9:29" x14ac:dyDescent="0.35">
       <c r="I39" t="s">
         <v>51</v>
       </c>
@@ -3647,7 +4118,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="40" spans="9:22" x14ac:dyDescent="0.35">
+    <row r="40" spans="9:29" x14ac:dyDescent="0.35">
       <c r="I40" t="s">
         <v>51</v>
       </c>
@@ -3685,7 +4156,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="41" spans="9:22" x14ac:dyDescent="0.35">
+    <row r="41" spans="9:29" x14ac:dyDescent="0.35">
       <c r="I41" t="s">
         <v>51</v>
       </c>
@@ -3723,7 +4194,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="9:22" x14ac:dyDescent="0.35">
+    <row r="42" spans="9:29" x14ac:dyDescent="0.35">
       <c r="I42" t="s">
         <v>51</v>
       </c>
@@ -3761,7 +4232,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="9:22" x14ac:dyDescent="0.35">
+    <row r="43" spans="9:29" x14ac:dyDescent="0.35">
       <c r="I43" t="s">
         <v>51</v>
       </c>
@@ -3799,7 +4270,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="44" spans="9:22" x14ac:dyDescent="0.35">
+    <row r="44" spans="9:29" x14ac:dyDescent="0.35">
       <c r="I44" t="s">
         <v>51</v>
       </c>
@@ -3837,7 +4308,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="45" spans="9:22" x14ac:dyDescent="0.35">
+    <row r="45" spans="9:29" x14ac:dyDescent="0.35">
       <c r="I45" t="s">
         <v>51</v>
       </c>
@@ -3875,7 +4346,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="46" spans="9:22" x14ac:dyDescent="0.35">
+    <row r="46" spans="9:29" x14ac:dyDescent="0.35">
       <c r="I46" t="s">
         <v>51</v>
       </c>
@@ -3913,7 +4384,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="47" spans="9:22" x14ac:dyDescent="0.35">
+    <row r="47" spans="9:29" x14ac:dyDescent="0.35">
       <c r="I47" t="s">
         <v>51</v>
       </c>
@@ -3951,7 +4422,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="48" spans="9:22" x14ac:dyDescent="0.35">
+    <row r="48" spans="9:29" x14ac:dyDescent="0.35">
       <c r="I48" t="s">
         <v>51</v>
       </c>

</xml_diff>

<commit_message>
adding wind onshore chartericis through ncap_af V
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D2F80CB-A3B6-4E1A-AD39-F2C5BC673D5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8EA5780-A88A-4DFB-B9B3-873C0EC33556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1478" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="117">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -400,12 +400,6 @@
   </si>
   <si>
     <t>~TFM_DINS-AT</t>
-  </si>
-  <si>
-    <t>Limtype</t>
-  </si>
-  <si>
-    <t>UP</t>
   </si>
   <si>
     <t>ncap_af</t>
@@ -1251,7 +1245,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05B64E1E-DC66-450D-AA2A-D1B01A72BCA4}">
-  <dimension ref="A1:AU122"/>
+  <dimension ref="A1:AT122"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="7" max="7" width="14.1796875" bestFit="1" customWidth="1"/>
@@ -1267,7 +1261,7 @@
     <col min="40" max="40" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:46" x14ac:dyDescent="0.35">
       <c r="C1" t="s">
         <v>108</v>
       </c>
@@ -1293,10 +1287,10 @@
         <v>109</v>
       </c>
       <c r="AR1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="2" spans="1:47" x14ac:dyDescent="0.35">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="2" spans="1:46" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>87</v>
       </c>
@@ -1352,67 +1346,64 @@
         <v>12</v>
       </c>
       <c r="X2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="Y2" t="s">
         <v>32</v>
       </c>
       <c r="Z2" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="AA2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="AB2" t="s">
         <v>113</v>
       </c>
-      <c r="AC2" t="s">
-        <v>115</v>
+      <c r="AD2" t="s">
+        <v>34</v>
       </c>
       <c r="AE2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="AF2" t="s">
+        <v>32</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>32</v>
+      </c>
+      <c r="AK2" t="s">
         <v>33</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AM2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AN2" t="s">
         <v>32</v>
       </c>
-      <c r="AH2" t="s">
-        <v>1</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>1</v>
-      </c>
-      <c r="AK2" t="s">
+      <c r="AO2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AQ2" t="s">
+        <v>114</v>
+      </c>
+      <c r="AR2" t="s">
         <v>32</v>
       </c>
-      <c r="AL2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>1</v>
-      </c>
-      <c r="AO2" t="s">
-        <v>32</v>
-      </c>
-      <c r="AP2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AR2" t="s">
-        <v>116</v>
-      </c>
       <c r="AS2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="AT2" t="s">
-        <v>36</v>
-      </c>
-      <c r="AU2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:46" x14ac:dyDescent="0.35">
       <c r="A3" t="str">
         <f>IFERROR(IF([1]Veda!#REF!=A2,"ok","x"),"")</f>
         <v/>
@@ -1475,61 +1466,58 @@
         <v>91</v>
       </c>
       <c r="Z3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA3" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC3">
+        <v>116</v>
+      </c>
+      <c r="AB3">
         <v>1E-3</v>
       </c>
+      <c r="AD3">
+        <v>0.11426940639269406</v>
+      </c>
       <c r="AE3">
-        <v>0.11426940639269406</v>
-      </c>
-      <c r="AF3">
         <v>0.16087081189037786</v>
       </c>
+      <c r="AF3" t="s">
+        <v>91</v>
+      </c>
       <c r="AG3" t="s">
+        <v>8</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>6</v>
+      </c>
+      <c r="AJ3" t="s">
         <v>91</v>
       </c>
-      <c r="AH3" t="s">
-        <v>8</v>
-      </c>
-      <c r="AJ3" t="s">
-        <v>6</v>
-      </c>
-      <c r="AK3" t="s">
+      <c r="AK3">
+        <v>0.11820818077291764</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AN3" t="s">
         <v>91</v>
       </c>
-      <c r="AL3">
-        <v>0.11820818077291764</v>
-      </c>
-      <c r="AN3" t="s">
-        <v>43</v>
-      </c>
-      <c r="AO3" t="s">
-        <v>91</v>
-      </c>
-      <c r="AP3">
+      <c r="AO3">
         <v>6.7453183173023845E-2</v>
       </c>
-      <c r="AR3">
+      <c r="AQ3">
         <v>2020</v>
       </c>
-      <c r="AS3" t="s">
+      <c r="AR3" t="s">
         <v>88</v>
       </c>
-      <c r="AT3">
+      <c r="AS3">
         <v>0</v>
       </c>
-      <c r="AU3" t="s">
+      <c r="AT3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:46" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
         <v>92</v>
       </c>
@@ -1582,61 +1570,58 @@
         <v>94</v>
       </c>
       <c r="Z4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA4" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC4">
+        <v>116</v>
+      </c>
+      <c r="AB4">
         <v>1E-3</v>
       </c>
+      <c r="AD4">
+        <v>0.11426940639269406</v>
+      </c>
       <c r="AE4">
-        <v>0.11426940639269406</v>
-      </c>
-      <c r="AF4">
         <v>5.2547713165767528E-2</v>
       </c>
+      <c r="AF4" t="s">
+        <v>94</v>
+      </c>
       <c r="AG4" t="s">
+        <v>8</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>6</v>
+      </c>
+      <c r="AJ4" t="s">
         <v>94</v>
       </c>
-      <c r="AH4" t="s">
-        <v>8</v>
-      </c>
-      <c r="AJ4" t="s">
-        <v>6</v>
-      </c>
-      <c r="AK4" t="s">
+      <c r="AK4">
+        <v>9.765399900437545E-2</v>
+      </c>
+      <c r="AM4" t="s">
+        <v>43</v>
+      </c>
+      <c r="AN4" t="s">
         <v>94</v>
       </c>
-      <c r="AL4">
-        <v>9.765399900437545E-2</v>
-      </c>
-      <c r="AN4" t="s">
-        <v>43</v>
-      </c>
-      <c r="AO4" t="s">
-        <v>94</v>
-      </c>
-      <c r="AP4">
+      <c r="AO4">
         <v>0.21742041059208561</v>
       </c>
-      <c r="AR4">
+      <c r="AQ4">
         <v>2020</v>
       </c>
-      <c r="AS4" t="s">
+      <c r="AR4" t="s">
         <v>92</v>
       </c>
-      <c r="AT4">
+      <c r="AS4">
         <v>0</v>
       </c>
-      <c r="AU4" t="s">
+      <c r="AT4" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:46" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>95</v>
       </c>
@@ -1689,61 +1674,58 @@
         <v>97</v>
       </c>
       <c r="Z5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA5" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB5" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC5">
+        <v>116</v>
+      </c>
+      <c r="AB5">
         <v>1E-3</v>
       </c>
+      <c r="AD5">
+        <v>2.0776255707762557E-2</v>
+      </c>
       <c r="AE5">
-        <v>2.0776255707762557E-2</v>
-      </c>
-      <c r="AF5">
         <v>3.5896543437005365E-2</v>
       </c>
+      <c r="AF5" t="s">
+        <v>97</v>
+      </c>
       <c r="AG5" t="s">
+        <v>8</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>6</v>
+      </c>
+      <c r="AJ5" t="s">
         <v>97</v>
       </c>
-      <c r="AH5" t="s">
-        <v>8</v>
-      </c>
-      <c r="AJ5" t="s">
-        <v>6</v>
-      </c>
-      <c r="AK5" t="s">
+      <c r="AK5">
+        <v>2.1376827284429509E-2</v>
+      </c>
+      <c r="AM5" t="s">
+        <v>43</v>
+      </c>
+      <c r="AN5" t="s">
         <v>97</v>
       </c>
-      <c r="AL5">
-        <v>2.1376827284429509E-2</v>
-      </c>
-      <c r="AN5" t="s">
-        <v>43</v>
-      </c>
-      <c r="AO5" t="s">
-        <v>97</v>
-      </c>
-      <c r="AP5">
+      <c r="AO5">
         <v>6.4867911695789315E-2</v>
       </c>
-      <c r="AR5">
+      <c r="AQ5">
         <v>2020</v>
       </c>
-      <c r="AS5" t="s">
+      <c r="AR5" t="s">
         <v>95</v>
       </c>
-      <c r="AT5">
+      <c r="AS5">
         <v>0</v>
       </c>
-      <c r="AU5" t="s">
+      <c r="AT5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:46" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>98</v>
       </c>
@@ -1790,61 +1772,58 @@
         <v>99</v>
       </c>
       <c r="Z6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA6" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB6" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC6">
+        <v>116</v>
+      </c>
+      <c r="AB6">
         <v>1E-3</v>
       </c>
+      <c r="AD6">
+        <v>0.11552511415525114</v>
+      </c>
       <c r="AE6">
-        <v>0.11552511415525114</v>
-      </c>
-      <c r="AF6">
         <v>0.16263862301005233</v>
       </c>
+      <c r="AF6" t="s">
+        <v>99</v>
+      </c>
       <c r="AG6" t="s">
+        <v>8</v>
+      </c>
+      <c r="AI6" t="s">
+        <v>6</v>
+      </c>
+      <c r="AJ6" t="s">
         <v>99</v>
       </c>
-      <c r="AH6" t="s">
-        <v>8</v>
-      </c>
-      <c r="AJ6" t="s">
-        <v>6</v>
-      </c>
-      <c r="AK6" t="s">
+      <c r="AK6">
+        <v>0.13104968035048054</v>
+      </c>
+      <c r="AM6" t="s">
+        <v>43</v>
+      </c>
+      <c r="AN6" t="s">
         <v>99</v>
       </c>
-      <c r="AL6">
-        <v>0.13104968035048054</v>
-      </c>
-      <c r="AN6" t="s">
-        <v>43</v>
-      </c>
-      <c r="AO6" t="s">
-        <v>99</v>
-      </c>
-      <c r="AP6">
+      <c r="AO6">
         <v>0.181059958051627</v>
       </c>
-      <c r="AR6">
+      <c r="AQ6">
         <v>2020</v>
       </c>
-      <c r="AS6" t="s">
+      <c r="AR6" t="s">
         <v>98</v>
       </c>
-      <c r="AT6">
+      <c r="AS6">
         <v>0</v>
       </c>
-      <c r="AU6" t="s">
+      <c r="AT6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:46" x14ac:dyDescent="0.35">
       <c r="I7" t="s">
         <v>39</v>
       </c>
@@ -1888,61 +1867,58 @@
         <v>100</v>
       </c>
       <c r="Z7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA7" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB7" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC7">
+        <v>116</v>
+      </c>
+      <c r="AB7">
         <v>1E-3</v>
       </c>
+      <c r="AD7">
+        <v>0.11552511415525114</v>
+      </c>
       <c r="AE7">
-        <v>0.11552511415525114</v>
-      </c>
-      <c r="AF7">
         <v>5.3125160563193538E-2</v>
       </c>
+      <c r="AF7" t="s">
+        <v>100</v>
+      </c>
       <c r="AG7" t="s">
+        <v>8</v>
+      </c>
+      <c r="AI7" t="s">
+        <v>6</v>
+      </c>
+      <c r="AJ7" t="s">
         <v>100</v>
       </c>
-      <c r="AH7" t="s">
-        <v>8</v>
-      </c>
-      <c r="AJ7" t="s">
-        <v>6</v>
-      </c>
-      <c r="AK7" t="s">
+      <c r="AK7">
+        <v>0.11255019110607196</v>
+      </c>
+      <c r="AM7" t="s">
+        <v>43</v>
+      </c>
+      <c r="AN7" t="s">
         <v>100</v>
       </c>
-      <c r="AL7">
-        <v>0.11255019110607196</v>
-      </c>
-      <c r="AN7" t="s">
-        <v>43</v>
-      </c>
-      <c r="AO7" t="s">
-        <v>100</v>
-      </c>
-      <c r="AP7">
+      <c r="AO7">
         <v>0.29479690034051531</v>
       </c>
-      <c r="AR7">
+      <c r="AQ7">
         <v>2021</v>
       </c>
-      <c r="AS7" t="s">
+      <c r="AR7" t="s">
         <v>88</v>
       </c>
-      <c r="AT7">
+      <c r="AS7">
         <v>0</v>
       </c>
-      <c r="AU7" t="s">
+      <c r="AT7" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:46" x14ac:dyDescent="0.35">
       <c r="I8" t="s">
         <v>39</v>
       </c>
@@ -1986,61 +1962,58 @@
         <v>101</v>
       </c>
       <c r="Z8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA8" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB8" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC8">
+        <v>116</v>
+      </c>
+      <c r="AB8">
         <v>1E-3</v>
       </c>
+      <c r="AD8">
+        <v>2.1004566210045664E-2</v>
+      </c>
       <c r="AE8">
-        <v>2.1004566210045664E-2</v>
-      </c>
-      <c r="AF8">
         <v>3.6291010947302131E-2</v>
       </c>
+      <c r="AF8" t="s">
+        <v>101</v>
+      </c>
       <c r="AG8" t="s">
+        <v>8</v>
+      </c>
+      <c r="AI8" t="s">
+        <v>6</v>
+      </c>
+      <c r="AJ8" t="s">
         <v>101</v>
       </c>
-      <c r="AH8" t="s">
-        <v>8</v>
-      </c>
-      <c r="AJ8" t="s">
-        <v>6</v>
-      </c>
-      <c r="AK8" t="s">
+      <c r="AK8">
+        <v>2.3834110177054908E-2</v>
+      </c>
+      <c r="AM8" t="s">
+        <v>43</v>
+      </c>
+      <c r="AN8" t="s">
         <v>101</v>
       </c>
-      <c r="AL8">
-        <v>2.3834110177054908E-2</v>
-      </c>
-      <c r="AN8" t="s">
-        <v>43</v>
-      </c>
-      <c r="AO8" t="s">
-        <v>101</v>
-      </c>
-      <c r="AP8">
+      <c r="AO8">
         <v>0.18791773337227902</v>
       </c>
-      <c r="AR8">
+      <c r="AQ8">
         <v>2021</v>
       </c>
-      <c r="AS8" t="s">
+      <c r="AR8" t="s">
         <v>92</v>
       </c>
-      <c r="AT8">
+      <c r="AS8">
         <v>0</v>
       </c>
-      <c r="AU8" t="s">
+      <c r="AT8" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:46" x14ac:dyDescent="0.35">
       <c r="I9" t="s">
         <v>39</v>
       </c>
@@ -2084,61 +2057,58 @@
         <v>102</v>
       </c>
       <c r="Z9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA9" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB9" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC9">
+        <v>116</v>
+      </c>
+      <c r="AB9">
         <v>1E-3</v>
       </c>
+      <c r="AD9">
+        <v>0.11552511415525114</v>
+      </c>
       <c r="AE9">
-        <v>0.11552511415525114</v>
-      </c>
-      <c r="AF9">
         <v>0.16263862301005233</v>
       </c>
+      <c r="AF9" t="s">
+        <v>102</v>
+      </c>
       <c r="AG9" t="s">
+        <v>8</v>
+      </c>
+      <c r="AI9" t="s">
+        <v>6</v>
+      </c>
+      <c r="AJ9" t="s">
         <v>102</v>
       </c>
-      <c r="AH9" t="s">
-        <v>8</v>
-      </c>
-      <c r="AJ9" t="s">
-        <v>6</v>
-      </c>
-      <c r="AK9" t="s">
+      <c r="AK9">
+        <v>0.11748145961359424</v>
+      </c>
+      <c r="AM9" t="s">
+        <v>43</v>
+      </c>
+      <c r="AN9" t="s">
         <v>102</v>
       </c>
-      <c r="AL9">
-        <v>0.11748145961359424</v>
-      </c>
-      <c r="AN9" t="s">
-        <v>43</v>
-      </c>
-      <c r="AO9" t="s">
-        <v>102</v>
-      </c>
-      <c r="AP9">
+      <c r="AO9">
         <v>0.13319460828738694</v>
       </c>
-      <c r="AR9">
+      <c r="AQ9">
         <v>2021</v>
       </c>
-      <c r="AS9" t="s">
+      <c r="AR9" t="s">
         <v>95</v>
       </c>
-      <c r="AT9">
+      <c r="AS9">
         <v>0</v>
       </c>
-      <c r="AU9" t="s">
+      <c r="AT9" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:46" x14ac:dyDescent="0.35">
       <c r="I10" t="s">
         <v>39</v>
       </c>
@@ -2182,61 +2152,58 @@
         <v>103</v>
       </c>
       <c r="Z10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA10" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB10" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC10">
+        <v>116</v>
+      </c>
+      <c r="AB10">
         <v>1E-3</v>
       </c>
+      <c r="AD10">
+        <v>0.11552511415525114</v>
+      </c>
       <c r="AE10">
-        <v>0.11552511415525114</v>
-      </c>
-      <c r="AF10">
         <v>5.3125160563193538E-2</v>
       </c>
+      <c r="AF10" t="s">
+        <v>103</v>
+      </c>
       <c r="AG10" t="s">
+        <v>8</v>
+      </c>
+      <c r="AI10" t="s">
+        <v>6</v>
+      </c>
+      <c r="AJ10" t="s">
         <v>103</v>
       </c>
-      <c r="AH10" t="s">
-        <v>8</v>
-      </c>
-      <c r="AJ10" t="s">
-        <v>6</v>
-      </c>
-      <c r="AK10" t="s">
+      <c r="AK10">
+        <v>8.4800799390331486E-2</v>
+      </c>
+      <c r="AM10" t="s">
+        <v>43</v>
+      </c>
+      <c r="AN10" t="s">
         <v>103</v>
       </c>
-      <c r="AL10">
-        <v>8.4800799390331486E-2</v>
-      </c>
-      <c r="AN10" t="s">
-        <v>43</v>
-      </c>
-      <c r="AO10" t="s">
-        <v>103</v>
-      </c>
-      <c r="AP10">
+      <c r="AO10">
         <v>0.27571202448049736</v>
       </c>
-      <c r="AR10">
+      <c r="AQ10">
         <v>2021</v>
       </c>
-      <c r="AS10" t="s">
+      <c r="AR10" t="s">
         <v>98</v>
       </c>
-      <c r="AT10">
+      <c r="AS10">
         <v>0</v>
       </c>
-      <c r="AU10" t="s">
+      <c r="AT10" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:46" x14ac:dyDescent="0.35">
       <c r="I11" t="s">
         <v>39</v>
       </c>
@@ -2280,61 +2247,58 @@
         <v>104</v>
       </c>
       <c r="Z11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA11" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB11" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC11">
+        <v>116</v>
+      </c>
+      <c r="AB11">
         <v>1E-3</v>
       </c>
+      <c r="AD11">
+        <v>2.1004566210045664E-2</v>
+      </c>
       <c r="AE11">
-        <v>2.1004566210045664E-2</v>
-      </c>
-      <c r="AF11">
         <v>3.6291010947302131E-2</v>
       </c>
+      <c r="AF11" t="s">
+        <v>104</v>
+      </c>
       <c r="AG11" t="s">
+        <v>8</v>
+      </c>
+      <c r="AI11" t="s">
+        <v>6</v>
+      </c>
+      <c r="AJ11" t="s">
         <v>104</v>
       </c>
-      <c r="AH11" t="s">
-        <v>8</v>
-      </c>
-      <c r="AJ11" t="s">
-        <v>6</v>
-      </c>
-      <c r="AK11" t="s">
+      <c r="AK11">
+        <v>2.0570847331150249E-2</v>
+      </c>
+      <c r="AM11" t="s">
+        <v>43</v>
+      </c>
+      <c r="AN11" t="s">
         <v>104</v>
       </c>
-      <c r="AL11">
-        <v>2.0570847331150249E-2</v>
-      </c>
-      <c r="AN11" t="s">
-        <v>43</v>
-      </c>
-      <c r="AO11" t="s">
-        <v>104</v>
-      </c>
-      <c r="AP11">
+      <c r="AO11">
         <v>9.8544131462115603E-2</v>
       </c>
-      <c r="AR11">
+      <c r="AQ11">
         <v>2022</v>
       </c>
-      <c r="AS11" t="s">
+      <c r="AR11" t="s">
         <v>88</v>
       </c>
-      <c r="AT11">
+      <c r="AS11">
         <v>0</v>
       </c>
-      <c r="AU11" t="s">
+      <c r="AT11" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:46" x14ac:dyDescent="0.35">
       <c r="I12" t="s">
         <v>39</v>
       </c>
@@ -2378,61 +2342,58 @@
         <v>105</v>
       </c>
       <c r="Z12" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA12" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB12" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC12">
+        <v>116</v>
+      </c>
+      <c r="AB12">
         <v>1E-3</v>
       </c>
+      <c r="AD12">
+        <v>0.11301369863013698</v>
+      </c>
       <c r="AE12">
-        <v>0.11301369863013698</v>
-      </c>
-      <c r="AF12">
         <v>0.15910300077070333</v>
       </c>
+      <c r="AF12" t="s">
+        <v>105</v>
+      </c>
       <c r="AG12" t="s">
+        <v>8</v>
+      </c>
+      <c r="AI12" t="s">
+        <v>6</v>
+      </c>
+      <c r="AJ12" t="s">
         <v>105</v>
       </c>
-      <c r="AH12" t="s">
-        <v>8</v>
-      </c>
-      <c r="AJ12" t="s">
-        <v>6</v>
-      </c>
-      <c r="AK12" t="s">
+      <c r="AK12">
+        <v>0.13067071966028027</v>
+      </c>
+      <c r="AM12" t="s">
+        <v>43</v>
+      </c>
+      <c r="AN12" t="s">
         <v>105</v>
       </c>
-      <c r="AL12">
-        <v>0.13067071966028027</v>
-      </c>
-      <c r="AN12" t="s">
-        <v>43</v>
-      </c>
-      <c r="AO12" t="s">
-        <v>105</v>
-      </c>
-      <c r="AP12">
+      <c r="AO12">
         <v>9.4996431311812124E-2</v>
       </c>
-      <c r="AR12">
+      <c r="AQ12">
         <v>2022</v>
       </c>
-      <c r="AS12" t="s">
+      <c r="AR12" t="s">
         <v>92</v>
       </c>
-      <c r="AT12">
+      <c r="AS12">
         <v>0</v>
       </c>
-      <c r="AU12" t="s">
+      <c r="AT12" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:46" x14ac:dyDescent="0.35">
       <c r="I13" t="s">
         <v>39</v>
       </c>
@@ -2476,61 +2437,58 @@
         <v>106</v>
       </c>
       <c r="Z13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA13" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB13" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC13">
+        <v>116</v>
+      </c>
+      <c r="AB13">
         <v>1E-3</v>
       </c>
+      <c r="AD13">
+        <v>0.11301369863013698</v>
+      </c>
       <c r="AE13">
-        <v>0.11301369863013698</v>
-      </c>
-      <c r="AF13">
         <v>5.197026576834151E-2</v>
       </c>
+      <c r="AF13" t="s">
+        <v>106</v>
+      </c>
       <c r="AG13" t="s">
+        <v>8</v>
+      </c>
+      <c r="AI13" t="s">
+        <v>6</v>
+      </c>
+      <c r="AJ13" t="s">
         <v>106</v>
       </c>
-      <c r="AH13" t="s">
-        <v>8</v>
-      </c>
-      <c r="AJ13" t="s">
-        <v>6</v>
-      </c>
-      <c r="AK13" t="s">
+      <c r="AK13">
+        <v>0.11789293365992742</v>
+      </c>
+      <c r="AM13" t="s">
+        <v>43</v>
+      </c>
+      <c r="AN13" t="s">
         <v>106</v>
       </c>
-      <c r="AL13">
-        <v>0.11789293365992742</v>
-      </c>
-      <c r="AN13" t="s">
-        <v>43</v>
-      </c>
-      <c r="AO13" t="s">
-        <v>106</v>
-      </c>
-      <c r="AP13">
+      <c r="AO13">
         <v>0.17683972082772126</v>
       </c>
-      <c r="AR13">
+      <c r="AQ13">
         <v>2022</v>
       </c>
-      <c r="AS13" t="s">
+      <c r="AR13" t="s">
         <v>95</v>
       </c>
-      <c r="AT13">
+      <c r="AS13">
         <v>0</v>
       </c>
-      <c r="AU13" t="s">
+      <c r="AT13" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:46" x14ac:dyDescent="0.35">
       <c r="I14" t="s">
         <v>39</v>
       </c>
@@ -2574,61 +2532,58 @@
         <v>107</v>
       </c>
       <c r="Z14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA14" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB14" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC14">
+        <v>116</v>
+      </c>
+      <c r="AB14">
         <v>1E-3</v>
       </c>
+      <c r="AD14">
+        <v>2.0547945205479451E-2</v>
+      </c>
       <c r="AE14">
-        <v>2.0547945205479451E-2</v>
-      </c>
-      <c r="AF14">
         <v>3.5502075926708607E-2</v>
       </c>
+      <c r="AF14" t="s">
+        <v>107</v>
+      </c>
       <c r="AG14" t="s">
+        <v>8</v>
+      </c>
+      <c r="AI14" t="s">
+        <v>6</v>
+      </c>
+      <c r="AJ14" t="s">
         <v>107</v>
       </c>
-      <c r="AH14" t="s">
-        <v>8</v>
-      </c>
-      <c r="AJ14" t="s">
-        <v>6</v>
-      </c>
-      <c r="AK14" t="s">
+      <c r="AK14">
+        <v>2.3910251649386354E-2</v>
+      </c>
+      <c r="AM14" t="s">
+        <v>43</v>
+      </c>
+      <c r="AN14" t="s">
         <v>107</v>
       </c>
-      <c r="AL14">
-        <v>2.3910251649386354E-2</v>
-      </c>
-      <c r="AN14" t="s">
-        <v>43</v>
-      </c>
-      <c r="AO14" t="s">
-        <v>107</v>
-      </c>
-      <c r="AP14">
+      <c r="AO14">
         <v>7.423298333369277E-2</v>
       </c>
-      <c r="AR14">
+      <c r="AQ14">
         <v>2022</v>
       </c>
-      <c r="AS14" t="s">
+      <c r="AR14" t="s">
         <v>98</v>
       </c>
-      <c r="AT14">
+      <c r="AS14">
         <v>0</v>
       </c>
-      <c r="AU14" t="s">
+      <c r="AT14" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:46" x14ac:dyDescent="0.35">
       <c r="I15" t="s">
         <v>45</v>
       </c>
@@ -2672,28 +2627,25 @@
         <v>91</v>
       </c>
       <c r="Z15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA15" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB15" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC15">
+        <v>116</v>
+      </c>
+      <c r="AB15">
         <v>1E-3</v>
       </c>
+      <c r="AI15" t="s">
+        <v>5</v>
+      </c>
       <c r="AJ15" t="s">
-        <v>5</v>
-      </c>
-      <c r="AK15" t="s">
         <v>91</v>
       </c>
-      <c r="AL15">
+      <c r="AK15">
         <v>0.11491480071761173</v>
       </c>
     </row>
-    <row r="16" spans="1:47" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:46" x14ac:dyDescent="0.35">
       <c r="I16" t="s">
         <v>45</v>
       </c>
@@ -2737,28 +2689,25 @@
         <v>94</v>
       </c>
       <c r="Z16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA16" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB16" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC16">
+        <v>116</v>
+      </c>
+      <c r="AB16">
         <v>1E-3</v>
       </c>
+      <c r="AI16" t="s">
+        <v>5</v>
+      </c>
       <c r="AJ16" t="s">
-        <v>5</v>
-      </c>
-      <c r="AK16" t="s">
         <v>94</v>
       </c>
-      <c r="AL16">
+      <c r="AK16">
         <v>0.11343014511581903</v>
       </c>
     </row>
-    <row r="17" spans="9:38" x14ac:dyDescent="0.35">
+    <row r="17" spans="9:37" x14ac:dyDescent="0.35">
       <c r="I17" t="s">
         <v>45</v>
       </c>
@@ -2802,28 +2751,25 @@
         <v>97</v>
       </c>
       <c r="Z17" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA17" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB17" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC17">
+        <v>116</v>
+      </c>
+      <c r="AB17">
         <v>1E-3</v>
       </c>
+      <c r="AI17" t="s">
+        <v>5</v>
+      </c>
       <c r="AJ17" t="s">
-        <v>5</v>
-      </c>
-      <c r="AK17" t="s">
         <v>97</v>
       </c>
-      <c r="AL17">
+      <c r="AK17">
         <v>2.0885252413625318E-2</v>
       </c>
     </row>
-    <row r="18" spans="9:38" x14ac:dyDescent="0.35">
+    <row r="18" spans="9:37" x14ac:dyDescent="0.35">
       <c r="I18" t="s">
         <v>45</v>
       </c>
@@ -2867,28 +2813,25 @@
         <v>99</v>
       </c>
       <c r="Z18" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA18" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB18" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC18">
+        <v>116</v>
+      </c>
+      <c r="AB18">
         <v>1E-3</v>
       </c>
+      <c r="AI18" t="s">
+        <v>5</v>
+      </c>
       <c r="AJ18" t="s">
-        <v>5</v>
-      </c>
-      <c r="AK18" t="s">
         <v>99</v>
       </c>
-      <c r="AL18">
+      <c r="AK18">
         <v>0.11618686907147086</v>
       </c>
     </row>
-    <row r="19" spans="9:38" x14ac:dyDescent="0.35">
+    <row r="19" spans="9:37" x14ac:dyDescent="0.35">
       <c r="I19" t="s">
         <v>45</v>
       </c>
@@ -2932,28 +2875,25 @@
         <v>100</v>
       </c>
       <c r="Z19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA19" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB19" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC19">
+        <v>116</v>
+      </c>
+      <c r="AB19">
         <v>1E-3</v>
       </c>
+      <c r="AI19" t="s">
+        <v>5</v>
+      </c>
       <c r="AJ19" t="s">
-        <v>5</v>
-      </c>
-      <c r="AK19" t="s">
         <v>100</v>
       </c>
-      <c r="AL19">
+      <c r="AK19">
         <v>0.11485062661500635</v>
       </c>
     </row>
-    <row r="20" spans="9:38" x14ac:dyDescent="0.35">
+    <row r="20" spans="9:37" x14ac:dyDescent="0.35">
       <c r="I20" t="s">
         <v>45</v>
       </c>
@@ -2997,28 +2937,25 @@
         <v>101</v>
       </c>
       <c r="Z20" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA20" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB20" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC20">
+        <v>116</v>
+      </c>
+      <c r="AB20">
         <v>1E-3</v>
       </c>
+      <c r="AI20" t="s">
+        <v>5</v>
+      </c>
       <c r="AJ20" t="s">
-        <v>5</v>
-      </c>
-      <c r="AK20" t="s">
         <v>101</v>
       </c>
-      <c r="AL20">
+      <c r="AK20">
         <v>2.1125383361665393E-2</v>
       </c>
     </row>
-    <row r="21" spans="9:38" x14ac:dyDescent="0.35">
+    <row r="21" spans="9:37" x14ac:dyDescent="0.35">
       <c r="I21" t="s">
         <v>45</v>
       </c>
@@ -3062,28 +2999,25 @@
         <v>102</v>
       </c>
       <c r="Z21" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA21" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB21" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC21">
+        <v>116</v>
+      </c>
+      <c r="AB21">
         <v>1E-3</v>
       </c>
+      <c r="AI21" t="s">
+        <v>5</v>
+      </c>
       <c r="AJ21" t="s">
-        <v>5</v>
-      </c>
-      <c r="AK21" t="s">
         <v>102</v>
       </c>
-      <c r="AL21">
+      <c r="AK21">
         <v>0.11653911207601672</v>
       </c>
     </row>
-    <row r="22" spans="9:38" x14ac:dyDescent="0.35">
+    <row r="22" spans="9:37" x14ac:dyDescent="0.35">
       <c r="I22" t="s">
         <v>45</v>
       </c>
@@ -3127,28 +3061,25 @@
         <v>103</v>
       </c>
       <c r="Z22" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA22" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB22" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC22">
+        <v>116</v>
+      </c>
+      <c r="AB22">
         <v>1E-3</v>
       </c>
+      <c r="AI22" t="s">
+        <v>5</v>
+      </c>
       <c r="AJ22" t="s">
-        <v>5</v>
-      </c>
-      <c r="AK22" t="s">
         <v>103</v>
       </c>
-      <c r="AL22">
+      <c r="AK22">
         <v>0.11417854497501884</v>
       </c>
     </row>
-    <row r="23" spans="9:38" x14ac:dyDescent="0.35">
+    <row r="23" spans="9:37" x14ac:dyDescent="0.35">
       <c r="I23" t="s">
         <v>45</v>
       </c>
@@ -3192,28 +3123,25 @@
         <v>104</v>
       </c>
       <c r="Z23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA23" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB23" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC23">
+        <v>116</v>
+      </c>
+      <c r="AB23">
         <v>1E-3</v>
       </c>
+      <c r="AI23" t="s">
+        <v>5</v>
+      </c>
       <c r="AJ23" t="s">
-        <v>5</v>
-      </c>
-      <c r="AK23" t="s">
         <v>104</v>
       </c>
-      <c r="AL23">
+      <c r="AK23">
         <v>2.1131908763385672E-2</v>
       </c>
     </row>
-    <row r="24" spans="9:38" x14ac:dyDescent="0.35">
+    <row r="24" spans="9:37" x14ac:dyDescent="0.35">
       <c r="I24" t="s">
         <v>45</v>
       </c>
@@ -3257,28 +3185,25 @@
         <v>105</v>
       </c>
       <c r="Z24" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA24" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB24" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC24">
+        <v>116</v>
+      </c>
+      <c r="AB24">
         <v>1E-3</v>
       </c>
+      <c r="AI24" t="s">
+        <v>5</v>
+      </c>
       <c r="AJ24" t="s">
-        <v>5</v>
-      </c>
-      <c r="AK24" t="s">
         <v>105</v>
       </c>
-      <c r="AL24">
+      <c r="AK24">
         <v>0.11351511345077332</v>
       </c>
     </row>
-    <row r="25" spans="9:38" x14ac:dyDescent="0.35">
+    <row r="25" spans="9:37" x14ac:dyDescent="0.35">
       <c r="I25" t="s">
         <v>45</v>
       </c>
@@ -3322,28 +3247,25 @@
         <v>106</v>
       </c>
       <c r="Z25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA25" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB25" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC25">
+        <v>116</v>
+      </c>
+      <c r="AB25">
         <v>1E-3</v>
       </c>
+      <c r="AI25" t="s">
+        <v>5</v>
+      </c>
       <c r="AJ25" t="s">
-        <v>5</v>
-      </c>
-      <c r="AK25" t="s">
         <v>106</v>
       </c>
-      <c r="AL25">
+      <c r="AK25">
         <v>0.11259215715032031</v>
       </c>
     </row>
-    <row r="26" spans="9:38" x14ac:dyDescent="0.35">
+    <row r="26" spans="9:37" x14ac:dyDescent="0.35">
       <c r="I26" t="s">
         <v>45</v>
       </c>
@@ -3387,28 +3309,25 @@
         <v>107</v>
       </c>
       <c r="Z26" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA26" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB26" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC26">
+        <v>116</v>
+      </c>
+      <c r="AB26">
         <v>1E-3</v>
       </c>
+      <c r="AI26" t="s">
+        <v>5</v>
+      </c>
       <c r="AJ26" t="s">
-        <v>5</v>
-      </c>
-      <c r="AK26" t="s">
         <v>107</v>
       </c>
-      <c r="AL26">
+      <c r="AK26">
         <v>2.0650086289286402E-2</v>
       </c>
     </row>
-    <row r="27" spans="9:38" x14ac:dyDescent="0.35">
+    <row r="27" spans="9:37" x14ac:dyDescent="0.35">
       <c r="I27" t="s">
         <v>48</v>
       </c>
@@ -3452,19 +3371,16 @@
         <v>91</v>
       </c>
       <c r="Z27" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA27" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB27" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC27">
+        <v>116</v>
+      </c>
+      <c r="AB27">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="28" spans="9:38" x14ac:dyDescent="0.35">
+    <row r="28" spans="9:37" x14ac:dyDescent="0.35">
       <c r="I28" t="s">
         <v>48</v>
       </c>
@@ -3508,19 +3424,16 @@
         <v>94</v>
       </c>
       <c r="Z28" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA28" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB28" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC28">
+        <v>116</v>
+      </c>
+      <c r="AB28">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="29" spans="9:38" x14ac:dyDescent="0.35">
+    <row r="29" spans="9:37" x14ac:dyDescent="0.35">
       <c r="I29" t="s">
         <v>48</v>
       </c>
@@ -3564,19 +3477,16 @@
         <v>97</v>
       </c>
       <c r="Z29" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA29" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB29" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC29">
+        <v>116</v>
+      </c>
+      <c r="AB29">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="30" spans="9:38" x14ac:dyDescent="0.35">
+    <row r="30" spans="9:37" x14ac:dyDescent="0.35">
       <c r="I30" t="s">
         <v>48</v>
       </c>
@@ -3620,19 +3530,16 @@
         <v>99</v>
       </c>
       <c r="Z30" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA30" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB30" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC30">
+        <v>116</v>
+      </c>
+      <c r="AB30">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="31" spans="9:38" x14ac:dyDescent="0.35">
+    <row r="31" spans="9:37" x14ac:dyDescent="0.35">
       <c r="I31" t="s">
         <v>48</v>
       </c>
@@ -3676,19 +3583,16 @@
         <v>100</v>
       </c>
       <c r="Z31" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA31" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB31" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC31">
+        <v>116</v>
+      </c>
+      <c r="AB31">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="32" spans="9:38" x14ac:dyDescent="0.35">
+    <row r="32" spans="9:37" x14ac:dyDescent="0.35">
       <c r="I32" t="s">
         <v>48</v>
       </c>
@@ -3732,19 +3636,16 @@
         <v>101</v>
       </c>
       <c r="Z32" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA32" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB32" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC32">
+        <v>116</v>
+      </c>
+      <c r="AB32">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="33" spans="9:29" x14ac:dyDescent="0.35">
+    <row r="33" spans="9:28" x14ac:dyDescent="0.35">
       <c r="I33" t="s">
         <v>48</v>
       </c>
@@ -3788,19 +3689,16 @@
         <v>102</v>
       </c>
       <c r="Z33" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA33" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB33" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC33">
+        <v>116</v>
+      </c>
+      <c r="AB33">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="34" spans="9:29" x14ac:dyDescent="0.35">
+    <row r="34" spans="9:28" x14ac:dyDescent="0.35">
       <c r="I34" t="s">
         <v>48</v>
       </c>
@@ -3844,19 +3742,16 @@
         <v>103</v>
       </c>
       <c r="Z34" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA34" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB34" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC34">
+        <v>116</v>
+      </c>
+      <c r="AB34">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="35" spans="9:29" x14ac:dyDescent="0.35">
+    <row r="35" spans="9:28" x14ac:dyDescent="0.35">
       <c r="I35" t="s">
         <v>48</v>
       </c>
@@ -3900,19 +3795,16 @@
         <v>104</v>
       </c>
       <c r="Z35" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA35" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB35" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC35">
+        <v>116</v>
+      </c>
+      <c r="AB35">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="36" spans="9:29" x14ac:dyDescent="0.35">
+    <row r="36" spans="9:28" x14ac:dyDescent="0.35">
       <c r="I36" t="s">
         <v>48</v>
       </c>
@@ -3956,19 +3848,16 @@
         <v>105</v>
       </c>
       <c r="Z36" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA36" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB36" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC36">
+        <v>116</v>
+      </c>
+      <c r="AB36">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="37" spans="9:29" x14ac:dyDescent="0.35">
+    <row r="37" spans="9:28" x14ac:dyDescent="0.35">
       <c r="I37" t="s">
         <v>48</v>
       </c>
@@ -4012,19 +3901,16 @@
         <v>106</v>
       </c>
       <c r="Z37" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA37" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB37" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC37">
+        <v>116</v>
+      </c>
+      <c r="AB37">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="38" spans="9:29" x14ac:dyDescent="0.35">
+    <row r="38" spans="9:28" x14ac:dyDescent="0.35">
       <c r="I38" t="s">
         <v>48</v>
       </c>
@@ -4068,19 +3954,16 @@
         <v>107</v>
       </c>
       <c r="Z38" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AA38" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB38" t="s">
-        <v>118</v>
-      </c>
-      <c r="AC38">
+        <v>116</v>
+      </c>
+      <c r="AB38">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="39" spans="9:29" x14ac:dyDescent="0.35">
+    <row r="39" spans="9:28" x14ac:dyDescent="0.35">
       <c r="I39" t="s">
         <v>51</v>
       </c>
@@ -4118,7 +4001,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="40" spans="9:29" x14ac:dyDescent="0.35">
+    <row r="40" spans="9:28" x14ac:dyDescent="0.35">
       <c r="I40" t="s">
         <v>51</v>
       </c>
@@ -4156,7 +4039,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="41" spans="9:29" x14ac:dyDescent="0.35">
+    <row r="41" spans="9:28" x14ac:dyDescent="0.35">
       <c r="I41" t="s">
         <v>51</v>
       </c>
@@ -4194,7 +4077,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="9:29" x14ac:dyDescent="0.35">
+    <row r="42" spans="9:28" x14ac:dyDescent="0.35">
       <c r="I42" t="s">
         <v>51</v>
       </c>
@@ -4232,7 +4115,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="9:29" x14ac:dyDescent="0.35">
+    <row r="43" spans="9:28" x14ac:dyDescent="0.35">
       <c r="I43" t="s">
         <v>51</v>
       </c>
@@ -4270,7 +4153,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="44" spans="9:29" x14ac:dyDescent="0.35">
+    <row r="44" spans="9:28" x14ac:dyDescent="0.35">
       <c r="I44" t="s">
         <v>51</v>
       </c>
@@ -4308,7 +4191,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="45" spans="9:29" x14ac:dyDescent="0.35">
+    <row r="45" spans="9:28" x14ac:dyDescent="0.35">
       <c r="I45" t="s">
         <v>51</v>
       </c>
@@ -4346,7 +4229,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="46" spans="9:29" x14ac:dyDescent="0.35">
+    <row r="46" spans="9:28" x14ac:dyDescent="0.35">
       <c r="I46" t="s">
         <v>51</v>
       </c>
@@ -4384,7 +4267,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="47" spans="9:29" x14ac:dyDescent="0.35">
+    <row r="47" spans="9:28" x14ac:dyDescent="0.35">
       <c r="I47" t="s">
         <v>51</v>
       </c>
@@ -4422,7 +4305,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="48" spans="9:29" x14ac:dyDescent="0.35">
+    <row r="48" spans="9:28" x14ac:dyDescent="0.35">
       <c r="I48" t="s">
         <v>51</v>
       </c>

</xml_diff>

<commit_message>
adding wind onshore chartericis through ncap_af VI
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8EA5780-A88A-4DFB-B9B3-873C0EC33556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB4C9888-AF5D-4E5A-BF4F-39B0BC144BD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -420,7 +420,7 @@
     <t>~TFM_INS-AT</t>
   </si>
   <si>
-    <t>e*won*</t>
+    <t>e*won*,en*windon*,ep*windon*</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
adding wind onshore chartericis through ncap_af VII
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB4C9888-AF5D-4E5A-BF4F-39B0BC144BD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90F687B1-2888-48B3-AA19-AF8769ADBC97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="118">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -421,6 +421,9 @@
   </si>
   <si>
     <t>e*won*,en*windon*,ep*windon*</t>
+  </si>
+  <si>
+    <t>TFM_DINS-AT</t>
   </si>
 </sst>
 </file>
@@ -1272,7 +1275,7 @@
         <v>109</v>
       </c>
       <c r="S1" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="X1" t="s">
         <v>75</v>

</xml_diff>

<commit_message>
adding wind onshore chartericis through ncap_af VIII
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90F687B1-2888-48B3-AA19-AF8769ADBC97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12B90278-AAB7-4797-8639-DAEF1F8155AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1272,10 +1272,10 @@
         <v>109</v>
       </c>
       <c r="N1" t="s">
+        <v>117</v>
+      </c>
+      <c r="S1" t="s">
         <v>109</v>
-      </c>
-      <c r="S1" t="s">
-        <v>117</v>
       </c>
       <c r="X1" t="s">
         <v>75</v>

</xml_diff>

<commit_message>
adding wind onshore chartericis through ncap_af IX
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12B90278-AAB7-4797-8639-DAEF1F8155AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6188A375-2C2D-446C-963B-0D58353ADC7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1608" uniqueCount="117">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -405,9 +405,6 @@
     <t>ncap_af</t>
   </si>
   <si>
-    <t>PSET_PN</t>
-  </si>
-  <si>
     <t>Attribute</t>
   </si>
   <si>
@@ -420,20 +417,26 @@
     <t>~TFM_INS-AT</t>
   </si>
   <si>
-    <t>e*won*,en*windon*,ep*windon*</t>
-  </si>
-  <si>
     <t>TFM_DINS-AT</t>
+  </si>
+  <si>
+    <t>CSET_CO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1248,15 +1251,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05B64E1E-DC66-450D-AA2A-D1B01A72BCA4}">
-  <dimension ref="A1:AT122"/>
+  <dimension ref="A1:AS122"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="7" max="7" width="14.1796875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.1796875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="13.36328125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.36328125" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="13.36328125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="16.54296875" customWidth="1"/>
+    <col min="27" max="27" width="29.54296875" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="11.81640625" bestFit="1" customWidth="1"/>
     <col min="34" max="34" width="14.1796875" bestFit="1" customWidth="1"/>
     <col min="36" max="36" width="14.1796875" bestFit="1" customWidth="1"/>
@@ -1264,7 +1269,7 @@
     <col min="40" max="40" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:46" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:45" x14ac:dyDescent="0.35">
       <c r="C1" t="s">
         <v>108</v>
       </c>
@@ -1272,7 +1277,7 @@
         <v>109</v>
       </c>
       <c r="N1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="S1" t="s">
         <v>109</v>
@@ -1290,10 +1295,10 @@
         <v>109</v>
       </c>
       <c r="AR1" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="2" spans="1:46" x14ac:dyDescent="0.35">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>87</v>
       </c>
@@ -1349,64 +1354,61 @@
         <v>12</v>
       </c>
       <c r="X2" t="s">
-        <v>114</v>
+        <v>32</v>
       </c>
       <c r="Y2" t="s">
+        <v>111</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>116</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>112</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>34</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE2" t="s">
         <v>32</v>
       </c>
-      <c r="Z2" t="s">
-        <v>112</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>111</v>
-      </c>
-      <c r="AB2" t="s">
+      <c r="AF2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>32</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>33</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>1</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>32</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>35</v>
+      </c>
+      <c r="AP2" t="s">
         <v>113</v>
       </c>
-      <c r="AD2" t="s">
-        <v>34</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AF2" t="s">
+      <c r="AQ2" t="s">
         <v>32</v>
       </c>
-      <c r="AG2" t="s">
-        <v>1</v>
-      </c>
-      <c r="AI2" t="s">
-        <v>1</v>
-      </c>
-      <c r="AJ2" t="s">
-        <v>32</v>
-      </c>
-      <c r="AK2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AM2" t="s">
-        <v>1</v>
-      </c>
-      <c r="AN2" t="s">
-        <v>32</v>
-      </c>
-      <c r="AO2" t="s">
-        <v>35</v>
-      </c>
-      <c r="AQ2" t="s">
-        <v>114</v>
-      </c>
       <c r="AR2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="AS2" t="s">
-        <v>36</v>
-      </c>
-      <c r="AT2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:46" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:45" x14ac:dyDescent="0.35">
       <c r="A3" t="str">
         <f>IFERROR(IF([1]Veda!#REF!=A2,"ok","x"),"")</f>
         <v/>
@@ -1462,65 +1464,62 @@
       <c r="V3" t="s">
         <v>40</v>
       </c>
-      <c r="X3">
-        <v>2022</v>
+      <c r="X3" t="s">
+        <v>91</v>
       </c>
       <c r="Y3" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA3">
+        <v>1E-3</v>
+      </c>
+      <c r="AC3">
+        <v>0.11426940639269406</v>
+      </c>
+      <c r="AD3">
+        <v>0.16087081189037786</v>
+      </c>
+      <c r="AE3" t="s">
         <v>91</v>
       </c>
-      <c r="Z3" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB3">
-        <v>1E-3</v>
-      </c>
-      <c r="AD3">
-        <v>0.11426940639269406</v>
-      </c>
-      <c r="AE3">
-        <v>0.16087081189037786</v>
-      </c>
       <c r="AF3" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI3" t="s">
         <v>91</v>
       </c>
-      <c r="AG3" t="s">
-        <v>8</v>
-      </c>
-      <c r="AI3" t="s">
-        <v>6</v>
-      </c>
-      <c r="AJ3" t="s">
+      <c r="AJ3">
+        <v>0.11820818077291764</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>43</v>
+      </c>
+      <c r="AM3" t="s">
         <v>91</v>
       </c>
-      <c r="AK3">
-        <v>0.11820818077291764</v>
-      </c>
-      <c r="AM3" t="s">
-        <v>43</v>
-      </c>
-      <c r="AN3" t="s">
-        <v>91</v>
-      </c>
-      <c r="AO3">
+      <c r="AN3">
         <v>6.7453183173023845E-2</v>
       </c>
-      <c r="AQ3">
+      <c r="AP3">
         <v>2020</v>
       </c>
-      <c r="AR3" t="s">
+      <c r="AQ3" t="s">
         <v>88</v>
       </c>
-      <c r="AS3">
+      <c r="AR3">
         <v>0</v>
       </c>
-      <c r="AT3" t="s">
+      <c r="AS3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:46" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:45" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
         <v>92</v>
       </c>
@@ -1566,65 +1565,62 @@
       <c r="V4" t="s">
         <v>40</v>
       </c>
-      <c r="X4">
-        <v>2022</v>
+      <c r="X4" t="s">
+        <v>94</v>
       </c>
       <c r="Y4" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA4">
+        <v>1E-3</v>
+      </c>
+      <c r="AC4">
+        <v>0.11426940639269406</v>
+      </c>
+      <c r="AD4">
+        <v>5.2547713165767528E-2</v>
+      </c>
+      <c r="AE4" t="s">
         <v>94</v>
       </c>
-      <c r="Z4" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB4">
-        <v>1E-3</v>
-      </c>
-      <c r="AD4">
-        <v>0.11426940639269406</v>
-      </c>
-      <c r="AE4">
-        <v>5.2547713165767528E-2</v>
-      </c>
       <c r="AF4" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI4" t="s">
         <v>94</v>
       </c>
-      <c r="AG4" t="s">
-        <v>8</v>
-      </c>
-      <c r="AI4" t="s">
-        <v>6</v>
-      </c>
-      <c r="AJ4" t="s">
+      <c r="AJ4">
+        <v>9.765399900437545E-2</v>
+      </c>
+      <c r="AL4" t="s">
+        <v>43</v>
+      </c>
+      <c r="AM4" t="s">
         <v>94</v>
       </c>
-      <c r="AK4">
-        <v>9.765399900437545E-2</v>
-      </c>
-      <c r="AM4" t="s">
-        <v>43</v>
-      </c>
-      <c r="AN4" t="s">
-        <v>94</v>
-      </c>
-      <c r="AO4">
+      <c r="AN4">
         <v>0.21742041059208561</v>
       </c>
-      <c r="AQ4">
+      <c r="AP4">
         <v>2020</v>
       </c>
-      <c r="AR4" t="s">
+      <c r="AQ4" t="s">
         <v>92</v>
       </c>
-      <c r="AS4">
+      <c r="AR4">
         <v>0</v>
       </c>
-      <c r="AT4" t="s">
+      <c r="AS4" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:46" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:45" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>95</v>
       </c>
@@ -1670,65 +1666,62 @@
       <c r="V5" t="s">
         <v>40</v>
       </c>
-      <c r="X5">
-        <v>2022</v>
+      <c r="X5" t="s">
+        <v>97</v>
       </c>
       <c r="Y5" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA5">
+        <v>1E-3</v>
+      </c>
+      <c r="AC5">
+        <v>2.0776255707762557E-2</v>
+      </c>
+      <c r="AD5">
+        <v>3.5896543437005365E-2</v>
+      </c>
+      <c r="AE5" t="s">
         <v>97</v>
       </c>
-      <c r="Z5" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA5" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB5">
-        <v>1E-3</v>
-      </c>
-      <c r="AD5">
-        <v>2.0776255707762557E-2</v>
-      </c>
-      <c r="AE5">
-        <v>3.5896543437005365E-2</v>
-      </c>
       <c r="AF5" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI5" t="s">
         <v>97</v>
       </c>
-      <c r="AG5" t="s">
-        <v>8</v>
-      </c>
-      <c r="AI5" t="s">
-        <v>6</v>
-      </c>
-      <c r="AJ5" t="s">
+      <c r="AJ5">
+        <v>2.1376827284429509E-2</v>
+      </c>
+      <c r="AL5" t="s">
+        <v>43</v>
+      </c>
+      <c r="AM5" t="s">
         <v>97</v>
       </c>
-      <c r="AK5">
-        <v>2.1376827284429509E-2</v>
-      </c>
-      <c r="AM5" t="s">
-        <v>43</v>
-      </c>
-      <c r="AN5" t="s">
-        <v>97</v>
-      </c>
-      <c r="AO5">
+      <c r="AN5">
         <v>6.4867911695789315E-2</v>
       </c>
-      <c r="AQ5">
+      <c r="AP5">
         <v>2020</v>
       </c>
-      <c r="AR5" t="s">
+      <c r="AQ5" t="s">
         <v>95</v>
       </c>
-      <c r="AS5">
+      <c r="AR5">
         <v>0</v>
       </c>
-      <c r="AT5" t="s">
+      <c r="AS5" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:46" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:45" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>98</v>
       </c>
@@ -1768,65 +1761,62 @@
       <c r="V6" t="s">
         <v>40</v>
       </c>
-      <c r="X6">
-        <v>2022</v>
+      <c r="X6" t="s">
+        <v>99</v>
       </c>
       <c r="Y6" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA6">
+        <v>1E-3</v>
+      </c>
+      <c r="AC6">
+        <v>0.11552511415525114</v>
+      </c>
+      <c r="AD6">
+        <v>0.16263862301005233</v>
+      </c>
+      <c r="AE6" t="s">
         <v>99</v>
       </c>
-      <c r="Z6" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA6" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB6">
-        <v>1E-3</v>
-      </c>
-      <c r="AD6">
-        <v>0.11552511415525114</v>
-      </c>
-      <c r="AE6">
-        <v>0.16263862301005233</v>
-      </c>
       <c r="AF6" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH6" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI6" t="s">
         <v>99</v>
       </c>
-      <c r="AG6" t="s">
-        <v>8</v>
-      </c>
-      <c r="AI6" t="s">
-        <v>6</v>
-      </c>
-      <c r="AJ6" t="s">
+      <c r="AJ6">
+        <v>0.13104968035048054</v>
+      </c>
+      <c r="AL6" t="s">
+        <v>43</v>
+      </c>
+      <c r="AM6" t="s">
         <v>99</v>
       </c>
-      <c r="AK6">
-        <v>0.13104968035048054</v>
-      </c>
-      <c r="AM6" t="s">
-        <v>43</v>
-      </c>
-      <c r="AN6" t="s">
-        <v>99</v>
-      </c>
-      <c r="AO6">
+      <c r="AN6">
         <v>0.181059958051627</v>
       </c>
-      <c r="AQ6">
+      <c r="AP6">
         <v>2020</v>
       </c>
-      <c r="AR6" t="s">
+      <c r="AQ6" t="s">
         <v>98</v>
       </c>
-      <c r="AS6">
+      <c r="AR6">
         <v>0</v>
       </c>
-      <c r="AT6" t="s">
+      <c r="AS6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:46" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I7" t="s">
         <v>39</v>
       </c>
@@ -1863,65 +1853,62 @@
       <c r="V7" t="s">
         <v>40</v>
       </c>
-      <c r="X7">
-        <v>2022</v>
+      <c r="X7" t="s">
+        <v>100</v>
       </c>
       <c r="Y7" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA7">
+        <v>1E-3</v>
+      </c>
+      <c r="AC7">
+        <v>0.11552511415525114</v>
+      </c>
+      <c r="AD7">
+        <v>5.3125160563193538E-2</v>
+      </c>
+      <c r="AE7" t="s">
         <v>100</v>
       </c>
-      <c r="Z7" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA7" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB7">
-        <v>1E-3</v>
-      </c>
-      <c r="AD7">
-        <v>0.11552511415525114</v>
-      </c>
-      <c r="AE7">
-        <v>5.3125160563193538E-2</v>
-      </c>
       <c r="AF7" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH7" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI7" t="s">
         <v>100</v>
       </c>
-      <c r="AG7" t="s">
-        <v>8</v>
-      </c>
-      <c r="AI7" t="s">
-        <v>6</v>
-      </c>
-      <c r="AJ7" t="s">
+      <c r="AJ7">
+        <v>0.11255019110607196</v>
+      </c>
+      <c r="AL7" t="s">
+        <v>43</v>
+      </c>
+      <c r="AM7" t="s">
         <v>100</v>
       </c>
-      <c r="AK7">
-        <v>0.11255019110607196</v>
-      </c>
-      <c r="AM7" t="s">
-        <v>43</v>
-      </c>
-      <c r="AN7" t="s">
-        <v>100</v>
-      </c>
-      <c r="AO7">
+      <c r="AN7">
         <v>0.29479690034051531</v>
       </c>
-      <c r="AQ7">
+      <c r="AP7">
         <v>2021</v>
       </c>
-      <c r="AR7" t="s">
+      <c r="AQ7" t="s">
         <v>88</v>
       </c>
-      <c r="AS7">
+      <c r="AR7">
         <v>0</v>
       </c>
-      <c r="AT7" t="s">
+      <c r="AS7" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:46" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I8" t="s">
         <v>39</v>
       </c>
@@ -1958,65 +1945,62 @@
       <c r="V8" t="s">
         <v>40</v>
       </c>
-      <c r="X8">
-        <v>2022</v>
+      <c r="X8" t="s">
+        <v>101</v>
       </c>
       <c r="Y8" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA8">
+        <v>1E-3</v>
+      </c>
+      <c r="AC8">
+        <v>2.1004566210045664E-2</v>
+      </c>
+      <c r="AD8">
+        <v>3.6291010947302131E-2</v>
+      </c>
+      <c r="AE8" t="s">
         <v>101</v>
       </c>
-      <c r="Z8" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA8" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB8">
-        <v>1E-3</v>
-      </c>
-      <c r="AD8">
-        <v>2.1004566210045664E-2</v>
-      </c>
-      <c r="AE8">
-        <v>3.6291010947302131E-2</v>
-      </c>
       <c r="AF8" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH8" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI8" t="s">
         <v>101</v>
       </c>
-      <c r="AG8" t="s">
-        <v>8</v>
-      </c>
-      <c r="AI8" t="s">
-        <v>6</v>
-      </c>
-      <c r="AJ8" t="s">
+      <c r="AJ8">
+        <v>2.3834110177054908E-2</v>
+      </c>
+      <c r="AL8" t="s">
+        <v>43</v>
+      </c>
+      <c r="AM8" t="s">
         <v>101</v>
       </c>
-      <c r="AK8">
-        <v>2.3834110177054908E-2</v>
-      </c>
-      <c r="AM8" t="s">
-        <v>43</v>
-      </c>
-      <c r="AN8" t="s">
-        <v>101</v>
-      </c>
-      <c r="AO8">
+      <c r="AN8">
         <v>0.18791773337227902</v>
       </c>
-      <c r="AQ8">
+      <c r="AP8">
         <v>2021</v>
       </c>
-      <c r="AR8" t="s">
+      <c r="AQ8" t="s">
         <v>92</v>
       </c>
-      <c r="AS8">
+      <c r="AR8">
         <v>0</v>
       </c>
-      <c r="AT8" t="s">
+      <c r="AS8" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:46" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I9" t="s">
         <v>39</v>
       </c>
@@ -2053,65 +2037,62 @@
       <c r="V9" t="s">
         <v>40</v>
       </c>
-      <c r="X9">
-        <v>2022</v>
+      <c r="X9" t="s">
+        <v>102</v>
       </c>
       <c r="Y9" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA9">
+        <v>1E-3</v>
+      </c>
+      <c r="AC9">
+        <v>0.11552511415525114</v>
+      </c>
+      <c r="AD9">
+        <v>0.16263862301005233</v>
+      </c>
+      <c r="AE9" t="s">
         <v>102</v>
       </c>
-      <c r="Z9" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA9" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB9">
-        <v>1E-3</v>
-      </c>
-      <c r="AD9">
-        <v>0.11552511415525114</v>
-      </c>
-      <c r="AE9">
-        <v>0.16263862301005233</v>
-      </c>
       <c r="AF9" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH9" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI9" t="s">
         <v>102</v>
       </c>
-      <c r="AG9" t="s">
-        <v>8</v>
-      </c>
-      <c r="AI9" t="s">
-        <v>6</v>
-      </c>
-      <c r="AJ9" t="s">
+      <c r="AJ9">
+        <v>0.11748145961359424</v>
+      </c>
+      <c r="AL9" t="s">
+        <v>43</v>
+      </c>
+      <c r="AM9" t="s">
         <v>102</v>
       </c>
-      <c r="AK9">
-        <v>0.11748145961359424</v>
-      </c>
-      <c r="AM9" t="s">
-        <v>43</v>
-      </c>
-      <c r="AN9" t="s">
-        <v>102</v>
-      </c>
-      <c r="AO9">
+      <c r="AN9">
         <v>0.13319460828738694</v>
       </c>
-      <c r="AQ9">
+      <c r="AP9">
         <v>2021</v>
       </c>
-      <c r="AR9" t="s">
+      <c r="AQ9" t="s">
         <v>95</v>
       </c>
-      <c r="AS9">
+      <c r="AR9">
         <v>0</v>
       </c>
-      <c r="AT9" t="s">
+      <c r="AS9" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:46" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I10" t="s">
         <v>39</v>
       </c>
@@ -2148,65 +2129,62 @@
       <c r="V10" t="s">
         <v>40</v>
       </c>
-      <c r="X10">
-        <v>2022</v>
+      <c r="X10" t="s">
+        <v>103</v>
       </c>
       <c r="Y10" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA10">
+        <v>1E-3</v>
+      </c>
+      <c r="AC10">
+        <v>0.11552511415525114</v>
+      </c>
+      <c r="AD10">
+        <v>5.3125160563193538E-2</v>
+      </c>
+      <c r="AE10" t="s">
         <v>103</v>
       </c>
-      <c r="Z10" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA10" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB10">
-        <v>1E-3</v>
-      </c>
-      <c r="AD10">
-        <v>0.11552511415525114</v>
-      </c>
-      <c r="AE10">
-        <v>5.3125160563193538E-2</v>
-      </c>
       <c r="AF10" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH10" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI10" t="s">
         <v>103</v>
       </c>
-      <c r="AG10" t="s">
-        <v>8</v>
-      </c>
-      <c r="AI10" t="s">
-        <v>6</v>
-      </c>
-      <c r="AJ10" t="s">
+      <c r="AJ10">
+        <v>8.4800799390331486E-2</v>
+      </c>
+      <c r="AL10" t="s">
+        <v>43</v>
+      </c>
+      <c r="AM10" t="s">
         <v>103</v>
       </c>
-      <c r="AK10">
-        <v>8.4800799390331486E-2</v>
-      </c>
-      <c r="AM10" t="s">
-        <v>43</v>
-      </c>
-      <c r="AN10" t="s">
-        <v>103</v>
-      </c>
-      <c r="AO10">
+      <c r="AN10">
         <v>0.27571202448049736</v>
       </c>
-      <c r="AQ10">
+      <c r="AP10">
         <v>2021</v>
       </c>
-      <c r="AR10" t="s">
+      <c r="AQ10" t="s">
         <v>98</v>
       </c>
-      <c r="AS10">
+      <c r="AR10">
         <v>0</v>
       </c>
-      <c r="AT10" t="s">
+      <c r="AS10" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:46" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I11" t="s">
         <v>39</v>
       </c>
@@ -2243,65 +2221,62 @@
       <c r="V11" t="s">
         <v>40</v>
       </c>
-      <c r="X11">
+      <c r="X11" t="s">
+        <v>104</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA11">
+        <v>1E-3</v>
+      </c>
+      <c r="AC11">
+        <v>2.1004566210045664E-2</v>
+      </c>
+      <c r="AD11">
+        <v>3.6291010947302131E-2</v>
+      </c>
+      <c r="AE11" t="s">
+        <v>104</v>
+      </c>
+      <c r="AF11" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH11" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI11" t="s">
+        <v>104</v>
+      </c>
+      <c r="AJ11">
+        <v>2.0570847331150249E-2</v>
+      </c>
+      <c r="AL11" t="s">
+        <v>43</v>
+      </c>
+      <c r="AM11" t="s">
+        <v>104</v>
+      </c>
+      <c r="AN11">
+        <v>9.8544131462115603E-2</v>
+      </c>
+      <c r="AP11">
         <v>2022</v>
       </c>
-      <c r="Y11" t="s">
-        <v>104</v>
-      </c>
-      <c r="Z11" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA11" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB11">
-        <v>1E-3</v>
-      </c>
-      <c r="AD11">
-        <v>2.1004566210045664E-2</v>
-      </c>
-      <c r="AE11">
-        <v>3.6291010947302131E-2</v>
-      </c>
-      <c r="AF11" t="s">
-        <v>104</v>
-      </c>
-      <c r="AG11" t="s">
-        <v>8</v>
-      </c>
-      <c r="AI11" t="s">
-        <v>6</v>
-      </c>
-      <c r="AJ11" t="s">
-        <v>104</v>
-      </c>
-      <c r="AK11">
-        <v>2.0570847331150249E-2</v>
-      </c>
-      <c r="AM11" t="s">
-        <v>43</v>
-      </c>
-      <c r="AN11" t="s">
-        <v>104</v>
-      </c>
-      <c r="AO11">
-        <v>9.8544131462115603E-2</v>
-      </c>
-      <c r="AQ11">
-        <v>2022</v>
-      </c>
-      <c r="AR11" t="s">
+      <c r="AQ11" t="s">
         <v>88</v>
       </c>
-      <c r="AS11">
+      <c r="AR11">
         <v>0</v>
       </c>
-      <c r="AT11" t="s">
+      <c r="AS11" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:46" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I12" t="s">
         <v>39</v>
       </c>
@@ -2338,65 +2313,62 @@
       <c r="V12" t="s">
         <v>40</v>
       </c>
-      <c r="X12">
+      <c r="X12" t="s">
+        <v>105</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA12">
+        <v>1E-3</v>
+      </c>
+      <c r="AC12">
+        <v>0.11301369863013698</v>
+      </c>
+      <c r="AD12">
+        <v>0.15910300077070333</v>
+      </c>
+      <c r="AE12" t="s">
+        <v>105</v>
+      </c>
+      <c r="AF12" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH12" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI12" t="s">
+        <v>105</v>
+      </c>
+      <c r="AJ12">
+        <v>0.13067071966028027</v>
+      </c>
+      <c r="AL12" t="s">
+        <v>43</v>
+      </c>
+      <c r="AM12" t="s">
+        <v>105</v>
+      </c>
+      <c r="AN12">
+        <v>9.4996431311812124E-2</v>
+      </c>
+      <c r="AP12">
         <v>2022</v>
       </c>
-      <c r="Y12" t="s">
-        <v>105</v>
-      </c>
-      <c r="Z12" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA12" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB12">
-        <v>1E-3</v>
-      </c>
-      <c r="AD12">
-        <v>0.11301369863013698</v>
-      </c>
-      <c r="AE12">
-        <v>0.15910300077070333</v>
-      </c>
-      <c r="AF12" t="s">
-        <v>105</v>
-      </c>
-      <c r="AG12" t="s">
-        <v>8</v>
-      </c>
-      <c r="AI12" t="s">
-        <v>6</v>
-      </c>
-      <c r="AJ12" t="s">
-        <v>105</v>
-      </c>
-      <c r="AK12">
-        <v>0.13067071966028027</v>
-      </c>
-      <c r="AM12" t="s">
-        <v>43</v>
-      </c>
-      <c r="AN12" t="s">
-        <v>105</v>
-      </c>
-      <c r="AO12">
-        <v>9.4996431311812124E-2</v>
-      </c>
-      <c r="AQ12">
-        <v>2022</v>
-      </c>
-      <c r="AR12" t="s">
+      <c r="AQ12" t="s">
         <v>92</v>
       </c>
-      <c r="AS12">
+      <c r="AR12">
         <v>0</v>
       </c>
-      <c r="AT12" t="s">
+      <c r="AS12" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="13" spans="1:46" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I13" t="s">
         <v>39</v>
       </c>
@@ -2433,65 +2405,62 @@
       <c r="V13" t="s">
         <v>40</v>
       </c>
-      <c r="X13">
+      <c r="X13" t="s">
+        <v>106</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA13">
+        <v>1E-3</v>
+      </c>
+      <c r="AC13">
+        <v>0.11301369863013698</v>
+      </c>
+      <c r="AD13">
+        <v>5.197026576834151E-2</v>
+      </c>
+      <c r="AE13" t="s">
+        <v>106</v>
+      </c>
+      <c r="AF13" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH13" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI13" t="s">
+        <v>106</v>
+      </c>
+      <c r="AJ13">
+        <v>0.11789293365992742</v>
+      </c>
+      <c r="AL13" t="s">
+        <v>43</v>
+      </c>
+      <c r="AM13" t="s">
+        <v>106</v>
+      </c>
+      <c r="AN13">
+        <v>0.17683972082772126</v>
+      </c>
+      <c r="AP13">
         <v>2022</v>
       </c>
-      <c r="Y13" t="s">
-        <v>106</v>
-      </c>
-      <c r="Z13" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA13" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB13">
-        <v>1E-3</v>
-      </c>
-      <c r="AD13">
-        <v>0.11301369863013698</v>
-      </c>
-      <c r="AE13">
-        <v>5.197026576834151E-2</v>
-      </c>
-      <c r="AF13" t="s">
-        <v>106</v>
-      </c>
-      <c r="AG13" t="s">
-        <v>8</v>
-      </c>
-      <c r="AI13" t="s">
-        <v>6</v>
-      </c>
-      <c r="AJ13" t="s">
-        <v>106</v>
-      </c>
-      <c r="AK13">
-        <v>0.11789293365992742</v>
-      </c>
-      <c r="AM13" t="s">
-        <v>43</v>
-      </c>
-      <c r="AN13" t="s">
-        <v>106</v>
-      </c>
-      <c r="AO13">
-        <v>0.17683972082772126</v>
-      </c>
-      <c r="AQ13">
-        <v>2022</v>
-      </c>
-      <c r="AR13" t="s">
+      <c r="AQ13" t="s">
         <v>95</v>
       </c>
-      <c r="AS13">
+      <c r="AR13">
         <v>0</v>
       </c>
-      <c r="AT13" t="s">
+      <c r="AS13" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:46" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I14" t="s">
         <v>39</v>
       </c>
@@ -2528,65 +2497,62 @@
       <c r="V14" t="s">
         <v>40</v>
       </c>
-      <c r="X14">
+      <c r="X14" t="s">
+        <v>107</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA14">
+        <v>1E-3</v>
+      </c>
+      <c r="AC14">
+        <v>2.0547945205479451E-2</v>
+      </c>
+      <c r="AD14">
+        <v>3.5502075926708607E-2</v>
+      </c>
+      <c r="AE14" t="s">
+        <v>107</v>
+      </c>
+      <c r="AF14" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH14" t="s">
+        <v>6</v>
+      </c>
+      <c r="AI14" t="s">
+        <v>107</v>
+      </c>
+      <c r="AJ14">
+        <v>2.3910251649386354E-2</v>
+      </c>
+      <c r="AL14" t="s">
+        <v>43</v>
+      </c>
+      <c r="AM14" t="s">
+        <v>107</v>
+      </c>
+      <c r="AN14">
+        <v>7.423298333369277E-2</v>
+      </c>
+      <c r="AP14">
         <v>2022</v>
       </c>
-      <c r="Y14" t="s">
-        <v>107</v>
-      </c>
-      <c r="Z14" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA14" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB14">
-        <v>1E-3</v>
-      </c>
-      <c r="AD14">
-        <v>2.0547945205479451E-2</v>
-      </c>
-      <c r="AE14">
-        <v>3.5502075926708607E-2</v>
-      </c>
-      <c r="AF14" t="s">
-        <v>107</v>
-      </c>
-      <c r="AG14" t="s">
-        <v>8</v>
-      </c>
-      <c r="AI14" t="s">
-        <v>6</v>
-      </c>
-      <c r="AJ14" t="s">
-        <v>107</v>
-      </c>
-      <c r="AK14">
-        <v>2.3910251649386354E-2</v>
-      </c>
-      <c r="AM14" t="s">
-        <v>43</v>
-      </c>
-      <c r="AN14" t="s">
-        <v>107</v>
-      </c>
-      <c r="AO14">
-        <v>7.423298333369277E-2</v>
-      </c>
-      <c r="AQ14">
-        <v>2022</v>
-      </c>
-      <c r="AR14" t="s">
+      <c r="AQ14" t="s">
         <v>98</v>
       </c>
-      <c r="AS14">
+      <c r="AR14">
         <v>0</v>
       </c>
-      <c r="AT14" t="s">
+      <c r="AS14" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:46" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I15" t="s">
         <v>45</v>
       </c>
@@ -2623,32 +2589,29 @@
       <c r="V15" t="s">
         <v>40</v>
       </c>
-      <c r="X15">
-        <v>2025</v>
+      <c r="X15" t="s">
+        <v>91</v>
       </c>
       <c r="Y15" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z15" t="s">
+        <v>47</v>
+      </c>
+      <c r="AA15">
+        <v>1E-3</v>
+      </c>
+      <c r="AH15" t="s">
+        <v>5</v>
+      </c>
+      <c r="AI15" t="s">
         <v>91</v>
       </c>
-      <c r="Z15" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA15" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB15">
-        <v>1E-3</v>
-      </c>
-      <c r="AI15" t="s">
-        <v>5</v>
-      </c>
-      <c r="AJ15" t="s">
-        <v>91</v>
-      </c>
-      <c r="AK15">
+      <c r="AJ15">
         <v>0.11491480071761173</v>
       </c>
     </row>
-    <row r="16" spans="1:46" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:45" x14ac:dyDescent="0.35">
       <c r="I16" t="s">
         <v>45</v>
       </c>
@@ -2685,32 +2648,29 @@
       <c r="V16" t="s">
         <v>40</v>
       </c>
-      <c r="X16">
-        <v>2025</v>
+      <c r="X16" t="s">
+        <v>94</v>
       </c>
       <c r="Y16" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z16" t="s">
+        <v>47</v>
+      </c>
+      <c r="AA16">
+        <v>1E-3</v>
+      </c>
+      <c r="AH16" t="s">
+        <v>5</v>
+      </c>
+      <c r="AI16" t="s">
         <v>94</v>
       </c>
-      <c r="Z16" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA16" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB16">
-        <v>1E-3</v>
-      </c>
-      <c r="AI16" t="s">
-        <v>5</v>
-      </c>
-      <c r="AJ16" t="s">
-        <v>94</v>
-      </c>
-      <c r="AK16">
+      <c r="AJ16">
         <v>0.11343014511581903</v>
       </c>
     </row>
-    <row r="17" spans="9:37" x14ac:dyDescent="0.35">
+    <row r="17" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I17" t="s">
         <v>45</v>
       </c>
@@ -2747,32 +2707,29 @@
       <c r="V17" t="s">
         <v>40</v>
       </c>
-      <c r="X17">
-        <v>2025</v>
+      <c r="X17" t="s">
+        <v>97</v>
       </c>
       <c r="Y17" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z17" t="s">
+        <v>47</v>
+      </c>
+      <c r="AA17">
+        <v>1E-3</v>
+      </c>
+      <c r="AH17" t="s">
+        <v>5</v>
+      </c>
+      <c r="AI17" t="s">
         <v>97</v>
       </c>
-      <c r="Z17" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA17" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB17">
-        <v>1E-3</v>
-      </c>
-      <c r="AI17" t="s">
-        <v>5</v>
-      </c>
-      <c r="AJ17" t="s">
-        <v>97</v>
-      </c>
-      <c r="AK17">
+      <c r="AJ17">
         <v>2.0885252413625318E-2</v>
       </c>
     </row>
-    <row r="18" spans="9:37" x14ac:dyDescent="0.35">
+    <row r="18" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I18" t="s">
         <v>45</v>
       </c>
@@ -2809,32 +2766,29 @@
       <c r="V18" t="s">
         <v>40</v>
       </c>
-      <c r="X18">
-        <v>2025</v>
+      <c r="X18" t="s">
+        <v>99</v>
       </c>
       <c r="Y18" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>47</v>
+      </c>
+      <c r="AA18">
+        <v>1E-3</v>
+      </c>
+      <c r="AH18" t="s">
+        <v>5</v>
+      </c>
+      <c r="AI18" t="s">
         <v>99</v>
       </c>
-      <c r="Z18" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA18" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB18">
-        <v>1E-3</v>
-      </c>
-      <c r="AI18" t="s">
-        <v>5</v>
-      </c>
-      <c r="AJ18" t="s">
-        <v>99</v>
-      </c>
-      <c r="AK18">
+      <c r="AJ18">
         <v>0.11618686907147086</v>
       </c>
     </row>
-    <row r="19" spans="9:37" x14ac:dyDescent="0.35">
+    <row r="19" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I19" t="s">
         <v>45</v>
       </c>
@@ -2871,32 +2825,29 @@
       <c r="V19" t="s">
         <v>40</v>
       </c>
-      <c r="X19">
-        <v>2025</v>
+      <c r="X19" t="s">
+        <v>100</v>
       </c>
       <c r="Y19" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>47</v>
+      </c>
+      <c r="AA19">
+        <v>1E-3</v>
+      </c>
+      <c r="AH19" t="s">
+        <v>5</v>
+      </c>
+      <c r="AI19" t="s">
         <v>100</v>
       </c>
-      <c r="Z19" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA19" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB19">
-        <v>1E-3</v>
-      </c>
-      <c r="AI19" t="s">
-        <v>5</v>
-      </c>
-      <c r="AJ19" t="s">
-        <v>100</v>
-      </c>
-      <c r="AK19">
+      <c r="AJ19">
         <v>0.11485062661500635</v>
       </c>
     </row>
-    <row r="20" spans="9:37" x14ac:dyDescent="0.35">
+    <row r="20" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I20" t="s">
         <v>45</v>
       </c>
@@ -2933,32 +2884,29 @@
       <c r="V20" t="s">
         <v>40</v>
       </c>
-      <c r="X20">
-        <v>2025</v>
+      <c r="X20" t="s">
+        <v>101</v>
       </c>
       <c r="Y20" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>47</v>
+      </c>
+      <c r="AA20">
+        <v>1E-3</v>
+      </c>
+      <c r="AH20" t="s">
+        <v>5</v>
+      </c>
+      <c r="AI20" t="s">
         <v>101</v>
       </c>
-      <c r="Z20" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA20" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB20">
-        <v>1E-3</v>
-      </c>
-      <c r="AI20" t="s">
-        <v>5</v>
-      </c>
-      <c r="AJ20" t="s">
-        <v>101</v>
-      </c>
-      <c r="AK20">
+      <c r="AJ20">
         <v>2.1125383361665393E-2</v>
       </c>
     </row>
-    <row r="21" spans="9:37" x14ac:dyDescent="0.35">
+    <row r="21" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I21" t="s">
         <v>45</v>
       </c>
@@ -2995,32 +2943,29 @@
       <c r="V21" t="s">
         <v>40</v>
       </c>
-      <c r="X21">
-        <v>2025</v>
+      <c r="X21" t="s">
+        <v>102</v>
       </c>
       <c r="Y21" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z21" t="s">
+        <v>47</v>
+      </c>
+      <c r="AA21">
+        <v>1E-3</v>
+      </c>
+      <c r="AH21" t="s">
+        <v>5</v>
+      </c>
+      <c r="AI21" t="s">
         <v>102</v>
       </c>
-      <c r="Z21" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA21" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB21">
-        <v>1E-3</v>
-      </c>
-      <c r="AI21" t="s">
-        <v>5</v>
-      </c>
-      <c r="AJ21" t="s">
-        <v>102</v>
-      </c>
-      <c r="AK21">
+      <c r="AJ21">
         <v>0.11653911207601672</v>
       </c>
     </row>
-    <row r="22" spans="9:37" x14ac:dyDescent="0.35">
+    <row r="22" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I22" t="s">
         <v>45</v>
       </c>
@@ -3057,32 +3002,29 @@
       <c r="V22" t="s">
         <v>40</v>
       </c>
-      <c r="X22">
-        <v>2025</v>
+      <c r="X22" t="s">
+        <v>103</v>
       </c>
       <c r="Y22" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z22" t="s">
+        <v>47</v>
+      </c>
+      <c r="AA22">
+        <v>1E-3</v>
+      </c>
+      <c r="AH22" t="s">
+        <v>5</v>
+      </c>
+      <c r="AI22" t="s">
         <v>103</v>
       </c>
-      <c r="Z22" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA22" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB22">
-        <v>1E-3</v>
-      </c>
-      <c r="AI22" t="s">
-        <v>5</v>
-      </c>
-      <c r="AJ22" t="s">
-        <v>103</v>
-      </c>
-      <c r="AK22">
+      <c r="AJ22">
         <v>0.11417854497501884</v>
       </c>
     </row>
-    <row r="23" spans="9:37" x14ac:dyDescent="0.35">
+    <row r="23" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I23" t="s">
         <v>45</v>
       </c>
@@ -3119,32 +3061,29 @@
       <c r="V23" t="s">
         <v>40</v>
       </c>
-      <c r="X23">
-        <v>2025</v>
+      <c r="X23" t="s">
+        <v>104</v>
       </c>
       <c r="Y23" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z23" t="s">
+        <v>47</v>
+      </c>
+      <c r="AA23">
+        <v>1E-3</v>
+      </c>
+      <c r="AH23" t="s">
+        <v>5</v>
+      </c>
+      <c r="AI23" t="s">
         <v>104</v>
       </c>
-      <c r="Z23" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA23" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB23">
-        <v>1E-3</v>
-      </c>
-      <c r="AI23" t="s">
-        <v>5</v>
-      </c>
-      <c r="AJ23" t="s">
-        <v>104</v>
-      </c>
-      <c r="AK23">
+      <c r="AJ23">
         <v>2.1131908763385672E-2</v>
       </c>
     </row>
-    <row r="24" spans="9:37" x14ac:dyDescent="0.35">
+    <row r="24" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I24" t="s">
         <v>45</v>
       </c>
@@ -3181,32 +3120,29 @@
       <c r="V24" t="s">
         <v>40</v>
       </c>
-      <c r="X24">
-        <v>2025</v>
+      <c r="X24" t="s">
+        <v>105</v>
       </c>
       <c r="Y24" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z24" t="s">
+        <v>47</v>
+      </c>
+      <c r="AA24">
+        <v>1E-3</v>
+      </c>
+      <c r="AH24" t="s">
+        <v>5</v>
+      </c>
+      <c r="AI24" t="s">
         <v>105</v>
       </c>
-      <c r="Z24" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA24" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB24">
-        <v>1E-3</v>
-      </c>
-      <c r="AI24" t="s">
-        <v>5</v>
-      </c>
-      <c r="AJ24" t="s">
-        <v>105</v>
-      </c>
-      <c r="AK24">
+      <c r="AJ24">
         <v>0.11351511345077332</v>
       </c>
     </row>
-    <row r="25" spans="9:37" x14ac:dyDescent="0.35">
+    <row r="25" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I25" t="s">
         <v>45</v>
       </c>
@@ -3243,32 +3179,29 @@
       <c r="V25" t="s">
         <v>40</v>
       </c>
-      <c r="X25">
-        <v>2025</v>
+      <c r="X25" t="s">
+        <v>106</v>
       </c>
       <c r="Y25" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z25" t="s">
+        <v>47</v>
+      </c>
+      <c r="AA25">
+        <v>1E-3</v>
+      </c>
+      <c r="AH25" t="s">
+        <v>5</v>
+      </c>
+      <c r="AI25" t="s">
         <v>106</v>
       </c>
-      <c r="Z25" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA25" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB25">
-        <v>1E-3</v>
-      </c>
-      <c r="AI25" t="s">
-        <v>5</v>
-      </c>
-      <c r="AJ25" t="s">
-        <v>106</v>
-      </c>
-      <c r="AK25">
+      <c r="AJ25">
         <v>0.11259215715032031</v>
       </c>
     </row>
-    <row r="26" spans="9:37" x14ac:dyDescent="0.35">
+    <row r="26" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I26" t="s">
         <v>45</v>
       </c>
@@ -3305,32 +3238,29 @@
       <c r="V26" t="s">
         <v>40</v>
       </c>
-      <c r="X26">
-        <v>2025</v>
+      <c r="X26" t="s">
+        <v>107</v>
       </c>
       <c r="Y26" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z26" t="s">
+        <v>47</v>
+      </c>
+      <c r="AA26">
+        <v>1E-3</v>
+      </c>
+      <c r="AH26" t="s">
+        <v>5</v>
+      </c>
+      <c r="AI26" t="s">
         <v>107</v>
       </c>
-      <c r="Z26" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA26" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB26">
-        <v>1E-3</v>
-      </c>
-      <c r="AI26" t="s">
-        <v>5</v>
-      </c>
-      <c r="AJ26" t="s">
-        <v>107</v>
-      </c>
-      <c r="AK26">
+      <c r="AJ26">
         <v>2.0650086289286402E-2</v>
       </c>
     </row>
-    <row r="27" spans="9:37" x14ac:dyDescent="0.35">
+    <row r="27" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I27" t="s">
         <v>48</v>
       </c>
@@ -3367,23 +3297,20 @@
       <c r="V27" t="s">
         <v>40</v>
       </c>
-      <c r="X27">
-        <v>2030</v>
+      <c r="X27" t="s">
+        <v>91</v>
       </c>
       <c r="Y27" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="Z27" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA27" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB27">
+        <v>50</v>
+      </c>
+      <c r="AA27">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="28" spans="9:37" x14ac:dyDescent="0.35">
+    <row r="28" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I28" t="s">
         <v>48</v>
       </c>
@@ -3420,23 +3347,20 @@
       <c r="V28" t="s">
         <v>40</v>
       </c>
-      <c r="X28">
-        <v>2030</v>
+      <c r="X28" t="s">
+        <v>94</v>
       </c>
       <c r="Y28" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="Z28" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA28" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB28">
+        <v>50</v>
+      </c>
+      <c r="AA28">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="29" spans="9:37" x14ac:dyDescent="0.35">
+    <row r="29" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I29" t="s">
         <v>48</v>
       </c>
@@ -3473,23 +3397,20 @@
       <c r="V29" t="s">
         <v>40</v>
       </c>
-      <c r="X29">
-        <v>2030</v>
+      <c r="X29" t="s">
+        <v>97</v>
       </c>
       <c r="Y29" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="Z29" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA29" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB29">
+        <v>50</v>
+      </c>
+      <c r="AA29">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="30" spans="9:37" x14ac:dyDescent="0.35">
+    <row r="30" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I30" t="s">
         <v>48</v>
       </c>
@@ -3526,23 +3447,20 @@
       <c r="V30" t="s">
         <v>40</v>
       </c>
-      <c r="X30">
-        <v>2030</v>
+      <c r="X30" t="s">
+        <v>99</v>
       </c>
       <c r="Y30" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="Z30" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA30" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB30">
+        <v>50</v>
+      </c>
+      <c r="AA30">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="31" spans="9:37" x14ac:dyDescent="0.35">
+    <row r="31" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I31" t="s">
         <v>48</v>
       </c>
@@ -3579,23 +3497,20 @@
       <c r="V31" t="s">
         <v>40</v>
       </c>
-      <c r="X31">
-        <v>2030</v>
+      <c r="X31" t="s">
+        <v>100</v>
       </c>
       <c r="Y31" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="Z31" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA31" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB31">
+        <v>50</v>
+      </c>
+      <c r="AA31">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="32" spans="9:37" x14ac:dyDescent="0.35">
+    <row r="32" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I32" t="s">
         <v>48</v>
       </c>
@@ -3632,23 +3547,20 @@
       <c r="V32" t="s">
         <v>40</v>
       </c>
-      <c r="X32">
-        <v>2030</v>
+      <c r="X32" t="s">
+        <v>101</v>
       </c>
       <c r="Y32" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="Z32" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA32" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB32">
+        <v>50</v>
+      </c>
+      <c r="AA32">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="33" spans="9:28" x14ac:dyDescent="0.35">
+    <row r="33" spans="9:27" x14ac:dyDescent="0.35">
       <c r="I33" t="s">
         <v>48</v>
       </c>
@@ -3685,23 +3597,20 @@
       <c r="V33" t="s">
         <v>40</v>
       </c>
-      <c r="X33">
-        <v>2030</v>
+      <c r="X33" t="s">
+        <v>102</v>
       </c>
       <c r="Y33" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="Z33" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA33" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB33">
+        <v>50</v>
+      </c>
+      <c r="AA33">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="34" spans="9:28" x14ac:dyDescent="0.35">
+    <row r="34" spans="9:27" x14ac:dyDescent="0.35">
       <c r="I34" t="s">
         <v>48</v>
       </c>
@@ -3738,23 +3647,20 @@
       <c r="V34" t="s">
         <v>40</v>
       </c>
-      <c r="X34">
-        <v>2030</v>
+      <c r="X34" t="s">
+        <v>103</v>
       </c>
       <c r="Y34" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="Z34" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA34" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB34">
+        <v>50</v>
+      </c>
+      <c r="AA34">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="35" spans="9:28" x14ac:dyDescent="0.35">
+    <row r="35" spans="9:27" x14ac:dyDescent="0.35">
       <c r="I35" t="s">
         <v>48</v>
       </c>
@@ -3791,23 +3697,20 @@
       <c r="V35" t="s">
         <v>40</v>
       </c>
-      <c r="X35">
-        <v>2030</v>
+      <c r="X35" t="s">
+        <v>104</v>
       </c>
       <c r="Y35" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="Z35" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA35" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB35">
+        <v>50</v>
+      </c>
+      <c r="AA35">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="36" spans="9:28" x14ac:dyDescent="0.35">
+    <row r="36" spans="9:27" x14ac:dyDescent="0.35">
       <c r="I36" t="s">
         <v>48</v>
       </c>
@@ -3844,23 +3747,20 @@
       <c r="V36" t="s">
         <v>40</v>
       </c>
-      <c r="X36">
-        <v>2030</v>
+      <c r="X36" t="s">
+        <v>105</v>
       </c>
       <c r="Y36" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="Z36" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA36" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB36">
+        <v>50</v>
+      </c>
+      <c r="AA36">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="37" spans="9:28" x14ac:dyDescent="0.35">
+    <row r="37" spans="9:27" x14ac:dyDescent="0.35">
       <c r="I37" t="s">
         <v>48</v>
       </c>
@@ -3897,23 +3797,20 @@
       <c r="V37" t="s">
         <v>40</v>
       </c>
-      <c r="X37">
-        <v>2030</v>
+      <c r="X37" t="s">
+        <v>106</v>
       </c>
       <c r="Y37" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="Z37" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA37" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB37">
+        <v>50</v>
+      </c>
+      <c r="AA37">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="38" spans="9:28" x14ac:dyDescent="0.35">
+    <row r="38" spans="9:27" x14ac:dyDescent="0.35">
       <c r="I38" t="s">
         <v>48</v>
       </c>
@@ -3950,23 +3847,20 @@
       <c r="V38" t="s">
         <v>40</v>
       </c>
-      <c r="X38">
-        <v>2030</v>
+      <c r="X38" t="s">
+        <v>107</v>
       </c>
       <c r="Y38" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="Z38" t="s">
-        <v>110</v>
-      </c>
-      <c r="AA38" t="s">
-        <v>116</v>
-      </c>
-      <c r="AB38">
+        <v>50</v>
+      </c>
+      <c r="AA38">
         <v>1E-3</v>
       </c>
     </row>
-    <row r="39" spans="9:28" x14ac:dyDescent="0.35">
+    <row r="39" spans="9:27" x14ac:dyDescent="0.35">
       <c r="I39" t="s">
         <v>51</v>
       </c>
@@ -4003,8 +3897,14 @@
       <c r="V39" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="40" spans="9:28" x14ac:dyDescent="0.35">
+      <c r="Y39" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z39" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="40" spans="9:27" x14ac:dyDescent="0.35">
       <c r="I40" t="s">
         <v>51</v>
       </c>
@@ -4041,8 +3941,14 @@
       <c r="V40" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="41" spans="9:28" x14ac:dyDescent="0.35">
+      <c r="Y40" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z40" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="41" spans="9:27" x14ac:dyDescent="0.35">
       <c r="I41" t="s">
         <v>51</v>
       </c>
@@ -4079,8 +3985,14 @@
       <c r="V41" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="42" spans="9:28" x14ac:dyDescent="0.35">
+      <c r="Y41" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z41" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="42" spans="9:27" x14ac:dyDescent="0.35">
       <c r="I42" t="s">
         <v>51</v>
       </c>
@@ -4117,8 +4029,14 @@
       <c r="V42" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="43" spans="9:28" x14ac:dyDescent="0.35">
+      <c r="Y42" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z42" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="43" spans="9:27" x14ac:dyDescent="0.35">
       <c r="I43" t="s">
         <v>51</v>
       </c>
@@ -4155,8 +4073,14 @@
       <c r="V43" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="44" spans="9:28" x14ac:dyDescent="0.35">
+      <c r="Y43" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z43" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="44" spans="9:27" x14ac:dyDescent="0.35">
       <c r="I44" t="s">
         <v>51</v>
       </c>
@@ -4193,8 +4117,14 @@
       <c r="V44" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="45" spans="9:28" x14ac:dyDescent="0.35">
+      <c r="Y44" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z44" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="45" spans="9:27" x14ac:dyDescent="0.35">
       <c r="I45" t="s">
         <v>51</v>
       </c>
@@ -4231,8 +4161,14 @@
       <c r="V45" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="46" spans="9:28" x14ac:dyDescent="0.35">
+      <c r="Y45" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z45" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="46" spans="9:27" x14ac:dyDescent="0.35">
       <c r="I46" t="s">
         <v>51</v>
       </c>
@@ -4269,8 +4205,14 @@
       <c r="V46" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="47" spans="9:28" x14ac:dyDescent="0.35">
+      <c r="Y46" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z46" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="47" spans="9:27" x14ac:dyDescent="0.35">
       <c r="I47" t="s">
         <v>51</v>
       </c>
@@ -4307,8 +4249,14 @@
       <c r="V47" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="48" spans="9:28" x14ac:dyDescent="0.35">
+      <c r="Y47" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z47" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="48" spans="9:27" x14ac:dyDescent="0.35">
       <c r="I48" t="s">
         <v>51</v>
       </c>
@@ -4345,8 +4293,14 @@
       <c r="V48" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="49" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y48" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z48" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="49" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I49" t="s">
         <v>51</v>
       </c>
@@ -4383,8 +4337,14 @@
       <c r="V49" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="50" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y49" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z49" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="50" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I50" t="s">
         <v>51</v>
       </c>
@@ -4421,8 +4381,14 @@
       <c r="V50" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="51" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y50" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z50" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="51" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I51" t="s">
         <v>54</v>
       </c>
@@ -4459,8 +4425,14 @@
       <c r="V51" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="52" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y51" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z51" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="52" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I52" t="s">
         <v>54</v>
       </c>
@@ -4497,8 +4469,14 @@
       <c r="V52" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="53" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y52" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z52" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="53" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I53" t="s">
         <v>54</v>
       </c>
@@ -4535,8 +4513,14 @@
       <c r="V53" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="54" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y53" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z53" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="54" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I54" t="s">
         <v>54</v>
       </c>
@@ -4573,8 +4557,14 @@
       <c r="V54" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="55" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y54" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z54" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="55" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I55" t="s">
         <v>54</v>
       </c>
@@ -4611,8 +4601,14 @@
       <c r="V55" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="56" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y55" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z55" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="56" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I56" t="s">
         <v>54</v>
       </c>
@@ -4649,8 +4645,14 @@
       <c r="V56" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="57" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y56" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z56" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="57" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I57" t="s">
         <v>54</v>
       </c>
@@ -4687,8 +4689,14 @@
       <c r="V57" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="58" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y57" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z57" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I58" t="s">
         <v>54</v>
       </c>
@@ -4725,8 +4733,14 @@
       <c r="V58" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="59" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y58" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z58" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="59" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I59" t="s">
         <v>54</v>
       </c>
@@ -4763,8 +4777,14 @@
       <c r="V59" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="60" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y59" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z59" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="60" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I60" t="s">
         <v>54</v>
       </c>
@@ -4801,8 +4821,14 @@
       <c r="V60" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="61" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y60" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z60" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="61" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I61" t="s">
         <v>54</v>
       </c>
@@ -4839,8 +4865,14 @@
       <c r="V61" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="62" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y61" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z61" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="62" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I62" t="s">
         <v>54</v>
       </c>
@@ -4877,8 +4909,14 @@
       <c r="V62" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="63" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y62" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z62" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="63" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I63" t="s">
         <v>57</v>
       </c>
@@ -4915,8 +4953,14 @@
       <c r="V63" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="64" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y63" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z63" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="64" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I64" t="s">
         <v>57</v>
       </c>
@@ -4953,8 +4997,14 @@
       <c r="V64" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="65" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y64" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z64" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="65" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I65" t="s">
         <v>57</v>
       </c>
@@ -4991,8 +5041,14 @@
       <c r="V65" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="66" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y65" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z65" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="66" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I66" t="s">
         <v>57</v>
       </c>
@@ -5029,8 +5085,14 @@
       <c r="V66" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="67" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y66" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z66" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="67" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I67" t="s">
         <v>57</v>
       </c>
@@ -5067,8 +5129,14 @@
       <c r="V67" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="68" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y67" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z67" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="68" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I68" t="s">
         <v>57</v>
       </c>
@@ -5105,8 +5173,14 @@
       <c r="V68" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="69" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y68" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z68" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="69" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I69" t="s">
         <v>57</v>
       </c>
@@ -5143,8 +5217,14 @@
       <c r="V69" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="70" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y69" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z69" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="70" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I70" t="s">
         <v>57</v>
       </c>
@@ -5181,8 +5261,14 @@
       <c r="V70" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="71" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y70" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z70" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="71" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I71" t="s">
         <v>57</v>
       </c>
@@ -5219,8 +5305,14 @@
       <c r="V71" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="72" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y71" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z71" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="72" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I72" t="s">
         <v>57</v>
       </c>
@@ -5257,8 +5349,14 @@
       <c r="V72" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="73" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y72" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z72" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="73" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I73" t="s">
         <v>57</v>
       </c>
@@ -5295,8 +5393,14 @@
       <c r="V73" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="74" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y73" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z73" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="74" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I74" t="s">
         <v>57</v>
       </c>
@@ -5333,8 +5437,14 @@
       <c r="V74" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="75" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y74" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z74" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="75" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I75" t="s">
         <v>60</v>
       </c>
@@ -5371,8 +5481,14 @@
       <c r="V75" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="76" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y75" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z75" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="76" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I76" t="s">
         <v>60</v>
       </c>
@@ -5409,8 +5525,14 @@
       <c r="V76" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="77" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y76" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z76" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="77" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I77" t="s">
         <v>60</v>
       </c>
@@ -5447,8 +5569,14 @@
       <c r="V77" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="78" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y77" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z77" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="78" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I78" t="s">
         <v>60</v>
       </c>
@@ -5485,8 +5613,14 @@
       <c r="V78" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="79" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y78" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z78" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="79" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I79" t="s">
         <v>60</v>
       </c>
@@ -5523,8 +5657,14 @@
       <c r="V79" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="80" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y79" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z79" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="80" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I80" t="s">
         <v>60</v>
       </c>
@@ -5561,8 +5701,14 @@
       <c r="V80" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="81" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y80" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z80" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="81" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I81" t="s">
         <v>60</v>
       </c>
@@ -5599,8 +5745,14 @@
       <c r="V81" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="82" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y81" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z81" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="82" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I82" t="s">
         <v>60</v>
       </c>
@@ -5637,8 +5789,14 @@
       <c r="V82" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="83" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y82" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z82" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="83" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I83" t="s">
         <v>60</v>
       </c>
@@ -5675,8 +5833,14 @@
       <c r="V83" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="84" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y83" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z83" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="84" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I84" t="s">
         <v>60</v>
       </c>
@@ -5713,8 +5877,14 @@
       <c r="V84" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="85" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y84" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z84" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="85" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I85" t="s">
         <v>60</v>
       </c>
@@ -5751,8 +5921,14 @@
       <c r="V85" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="86" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y85" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z85" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="86" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I86" t="s">
         <v>60</v>
       </c>
@@ -5789,8 +5965,14 @@
       <c r="V86" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="87" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y86" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z86" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="87" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I87" t="s">
         <v>63</v>
       </c>
@@ -5827,8 +6009,14 @@
       <c r="V87" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="88" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y87" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z87" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="88" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I88" t="s">
         <v>63</v>
       </c>
@@ -5865,8 +6053,14 @@
       <c r="V88" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="89" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y88" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z88" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="89" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I89" t="s">
         <v>63</v>
       </c>
@@ -5903,8 +6097,14 @@
       <c r="V89" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="90" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y89" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z89" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="90" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I90" t="s">
         <v>63</v>
       </c>
@@ -5941,8 +6141,14 @@
       <c r="V90" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="91" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y90" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z90" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="91" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I91" t="s">
         <v>63</v>
       </c>
@@ -5979,8 +6185,14 @@
       <c r="V91" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="92" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y91" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z91" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="92" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I92" t="s">
         <v>63</v>
       </c>
@@ -6017,8 +6229,14 @@
       <c r="V92" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="93" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y92" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z92" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="93" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I93" t="s">
         <v>63</v>
       </c>
@@ -6055,8 +6273,14 @@
       <c r="V93" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="94" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y93" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z93" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="94" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I94" t="s">
         <v>63</v>
       </c>
@@ -6093,8 +6317,14 @@
       <c r="V94" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="95" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y94" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z94" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="95" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I95" t="s">
         <v>63</v>
       </c>
@@ -6131,8 +6361,14 @@
       <c r="V95" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="96" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y95" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z95" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="96" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I96" t="s">
         <v>63</v>
       </c>
@@ -6169,8 +6405,14 @@
       <c r="V96" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="97" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y96" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z96" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="97" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I97" t="s">
         <v>63</v>
       </c>
@@ -6207,8 +6449,14 @@
       <c r="V97" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="98" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y97" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z97" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="98" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I98" t="s">
         <v>63</v>
       </c>
@@ -6245,8 +6493,14 @@
       <c r="V98" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="99" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y98" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z98" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="99" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I99" t="s">
         <v>66</v>
       </c>
@@ -6283,8 +6537,14 @@
       <c r="V99" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="100" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y99" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z99" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="100" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I100" t="s">
         <v>66</v>
       </c>
@@ -6321,8 +6581,14 @@
       <c r="V100" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="101" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y100" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z100" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="101" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I101" t="s">
         <v>66</v>
       </c>
@@ -6359,8 +6625,14 @@
       <c r="V101" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="102" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y101" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z101" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="102" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I102" t="s">
         <v>66</v>
       </c>
@@ -6397,8 +6669,14 @@
       <c r="V102" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="103" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y102" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z102" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="103" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I103" t="s">
         <v>66</v>
       </c>
@@ -6435,8 +6713,14 @@
       <c r="V103" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="104" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y103" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z103" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="104" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I104" t="s">
         <v>66</v>
       </c>
@@ -6473,8 +6757,14 @@
       <c r="V104" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="105" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y104" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z104" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="105" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I105" t="s">
         <v>66</v>
       </c>
@@ -6511,8 +6801,14 @@
       <c r="V105" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="106" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y105" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z105" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="106" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I106" t="s">
         <v>66</v>
       </c>
@@ -6549,8 +6845,14 @@
       <c r="V106" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="107" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y106" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z106" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="107" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I107" t="s">
         <v>66</v>
       </c>
@@ -6587,8 +6889,14 @@
       <c r="V107" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="108" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y107" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z107" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="108" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I108" t="s">
         <v>66</v>
       </c>
@@ -6625,8 +6933,14 @@
       <c r="V108" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="109" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y108" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z108" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="109" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I109" t="s">
         <v>66</v>
       </c>
@@ -6663,8 +6977,14 @@
       <c r="V109" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="110" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y109" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z109" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="110" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I110" t="s">
         <v>66</v>
       </c>
@@ -6701,8 +7021,14 @@
       <c r="V110" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="111" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y110" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z110" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="111" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I111" t="s">
         <v>69</v>
       </c>
@@ -6739,8 +7065,14 @@
       <c r="V111" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="112" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y111" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z111" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="112" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I112" t="s">
         <v>69</v>
       </c>
@@ -6777,8 +7109,14 @@
       <c r="V112" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="113" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y112" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z112" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="113" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I113" t="s">
         <v>69</v>
       </c>
@@ -6815,8 +7153,14 @@
       <c r="V113" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="114" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y113" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z113" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="114" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I114" t="s">
         <v>69</v>
       </c>
@@ -6853,8 +7197,14 @@
       <c r="V114" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="115" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y114" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z114" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="115" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I115" t="s">
         <v>69</v>
       </c>
@@ -6891,8 +7241,14 @@
       <c r="V115" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="116" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y115" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z115" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="116" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I116" t="s">
         <v>69</v>
       </c>
@@ -6929,8 +7285,14 @@
       <c r="V116" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="117" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y116" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z116" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="117" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I117" t="s">
         <v>69</v>
       </c>
@@ -6967,8 +7329,14 @@
       <c r="V117" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="118" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y117" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z117" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="118" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I118" t="s">
         <v>69</v>
       </c>
@@ -7005,8 +7373,14 @@
       <c r="V118" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="119" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y118" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z118" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="119" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I119" t="s">
         <v>69</v>
       </c>
@@ -7043,8 +7417,14 @@
       <c r="V119" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="120" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y119" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z119" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="120" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I120" t="s">
         <v>69</v>
       </c>
@@ -7081,8 +7461,14 @@
       <c r="V120" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="121" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y120" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z120" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="121" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I121" t="s">
         <v>69</v>
       </c>
@@ -7119,8 +7505,14 @@
       <c r="V121" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="122" spans="9:22" x14ac:dyDescent="0.35">
+      <c r="Y121" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z121" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="122" spans="9:26" x14ac:dyDescent="0.35">
       <c r="I122" t="s">
         <v>69</v>
       </c>
@@ -7157,8 +7549,15 @@
       <c r="V122" t="s">
         <v>40</v>
       </c>
+      <c r="Y122" t="s">
+        <v>110</v>
+      </c>
+      <c r="Z122" t="s">
+        <v>71</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Adding some random thing that was in SCEN_VS with no explanation but seems needed
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_test.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_test.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{093DFA9F-AFE7-4B44-A4B7-B762C34571A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A19D452-B5A4-4B79-87D9-BBB975CE304A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demand" sheetId="1" r:id="rId1"/>
     <sheet name="timeslices" sheetId="4" r:id="rId2"/>
     <sheet name="build rates" sheetId="5" r:id="rId3"/>
-    <sheet name="trade" sheetId="2" r:id="rId4"/>
-    <sheet name="fuel_costs" sheetId="3" r:id="rId5"/>
+    <sheet name="necessary_for_some_reason" sheetId="6" r:id="rId4"/>
+    <sheet name="trade" sheetId="2" r:id="rId5"/>
+    <sheet name="fuel_costs" sheetId="3" r:id="rId6"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId6"/>
+    <externalReference r:id="rId7"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -71,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1635" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1641" uniqueCount="134">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -467,6 +468,12 @@
   </si>
   <si>
     <t>uce_buildrate_windoff</t>
+  </si>
+  <si>
+    <t>START</t>
+  </si>
+  <si>
+    <t>Hydropower - large-scale unit,Solar photovoltaics - Large scale unit,Wind offshore,Wind onshore</t>
   </si>
 </sst>
 </file>
@@ -7787,6 +7794,43 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28A318F2-D986-4B43-9E10-D5047049B529}">
+  <dimension ref="A3:C5"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>132</v>
+      </c>
+      <c r="B5">
+        <v>2100</v>
+      </c>
+      <c r="C5" t="s">
+        <v>133</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F0573AE-84FA-4F18-8D18-B7F3EC5B3273}">
   <dimension ref="B4:K14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -7929,7 +7973,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48BDE16D-C995-4313-9FD3-ABCD01C0EB3D}">
   <dimension ref="B6:T11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>